<commit_message>
update transcription service safely
</commit_message>
<xml_diff>
--- a/audio_transcription_report.xlsx
+++ b/audio_transcription_report.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V36"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -451,10 +451,13 @@
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="52" customWidth="1" min="17" max="17"/>
     <col width="19" customWidth="1" min="18" max="18"/>
-    <col width="52" customWidth="1" min="19" max="19"/>
-    <col width="19" customWidth="1" min="20" max="20"/>
-    <col width="52" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="52" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
+    <col width="52" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -550,22 +553,37 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>passage1_confidence</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>passage2_transcription</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>passage2_language</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>passage2_confidence</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>testaudio_transcription</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>testaudio_language</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>testaudio_confidence</t>
         </is>
       </c>
     </row>
@@ -602,20 +620,24 @@
           <t>mock_eng</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>mock_eng</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio/trialeng.mp3</t>
+          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio_jan26/40_0T.mp3</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio/aeng.mp3</t>
+          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio_jan26/40_0A.mp3</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio/beng.mp3</t>
+          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio_jan26/40_0B.mp3</t>
         </is>
       </c>
       <c r="M2" s="2" t="n"/>
@@ -628,7 +650,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>This is shorthand passage audio for mock exam, technology has transformed the way humans connect  with one another. From handwritten letters to instant messaging, communication methods have  evolved rapidly. Today, a person can speak to someone on the other side of the world within  seconds. While this has made relationships more accessible and convenient, it has also changed  their depth and nature in complex ways. One of the biggest advantages of technology is its ability  to reduce distance. Families separated by cities or countries can stay connected through video  calls and social media. Friendships that might have faded due to lack of contact can now be  maintained with minimal effort. Online platforms also allow people to find communities based on  shared interests, beliefs, or experiences, which can be especially valuable for those who feel  isolated in their immediate surroundings.</t>
+          <t>English shorthand, 60 words per minute. Passage A. Ready, start. Dear Sir, Paira, referring to your letter dated, first instant, I have the honor to state that the information called for could not be supplied immediately from this office as the necessary particulars have it to be collected from various offices under our control. We are anyhow in a position to let you know that steps will be taken shortly to collect the particulars and send them on to you pending the receipt of details from our subordinate offices. I would like to suggest that the statistics in detail may be prepared in your office so that the tabulation may be made according to your requirements. Further, we are just now very busy in connection with the proposed legislation in the local assembly regarding labor immigration. I have very great pleasure to inform you that we are organizing a new department to look after the interests of those people who land in India in utter despair after spending a good deal of their time in foreign lands. The sight of such miserable men has shocked many of us in India and therefore we have been able to get a decent start in funds for our activities. I would expect your cooperation in all our efforts and I hope we can depend upon your guidance. If you will make an appointment next week, I shall be glad to see you and I may be able to give you, and I may be able to give you more particulars, Pira, you are sincerely.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -638,22 +660,37 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>This is shorthand passage B audio for mock exam, failure is often seen as something to be avoided  at all costs. Society tends to celebrate success while ignoring the struggles behind it.  As a result, many people fear failure and view it as a sign of weakness or incompetence.  However, failure plays a crucial role in personal growth and long-term success.  One of the most important lessons failure teaches is resilience.  When people face setbacks, they are forced to adapt, reflect, and try again.  This process builds mental strength and confidence.  Individuals who have experienced failure often develop a deeper understanding of their abilities  and limitations. They learn how to handle pressure and uncertainty more effectively.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 60 words per minute. Passage B. Ready, start. Dear Sirs, Phera, we confirm the following telegram sent to you just now. Delivery will be made tomorrow. Tara, we are really sorry for the delay. We have done our utmost to expedite delivery, but the pressure of orders for good blankets from our own state has made it difficult for us to deliver as promptly as we wish. And this is so even when our meals are working day and night. As a result of the sudden change of weather, we know you require the goods at once. We have in order to how you that we are annexed not to cause you inconvenience put aside other orders which in fact should have been executed before yours. Our customers are pressing on all sides for immediate delivery and the demand is heavy. We are not the only manufacturers of blankets whose resources are overtaxed at present. We are confident that this explanation will convince you of our endeavor to meet your wishes and because until this recent rush we have never failed to execute your orders within the stipulated time. We rely upon your leniency in the present case. We need hardly mention that your orders will always receive our most careful and prompt attention. We request you to remit the amounts due to date by a draft on the Reserve Bank of India. Navi Mumbai at your earliest convenience, there are yours truly Sreya's party.</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>This is shorthand trial audio for mock exam, work has always been a central part of human life,  but its meaning has changed significantly over time.  In earlier societies, work was closely tied to survival.  People farmed, hunted, or crafted goods mainly to meet basic needs.  The value of work was measured by how well it sustained families and communities.  Over time, with the rise of industries and cities, work became more structured,  timed, and specialized.  Today, in the modern world, work has taken on an even broader meaning that goes beyond earning a living.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 60 words per minute, trial passage. Ready? Start. Dear Sirs, Pera, we have given careful consideration to the request contained in your letter of 2 April for the sole agency in your letter of 2nd April for the sole agency in your district of our new machine. We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first-class connections in this type of machinery.</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -690,20 +727,24 @@
           <t>mock_mar</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>mock_mar</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio/trialMarathi.mp3</t>
+          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio_jan26/41_0T.mp3</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio/Amar.mp3</t>
+          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio_jan26/41_0A.mp3</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio/Bmar.mp3</t>
+          <t>https://shorthand2026.s3.ap-south-1.amazonaws.com/audio_jan26/41_0B.mp3</t>
         </is>
       </c>
       <c r="M3" s="2" t="n"/>
@@ -716,7 +757,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>हे मौक परिक्षे साथी शौठर उतारा पासेज अक्चे ओडियो आहे।  तंत्रद्न्यानाने मानवी जीवनात क्रांतिकारक बदल घडबून अनले आहे।  विशेश्टह सम्वादाचा पधतिन मधे मूठा बदल जाला आहे।  पूर्वी पत्र तार किम्मा प्रत्यक्ष भेटी वर अवलंबून असलेले नाते आज मुबाईल, इंटरनेट आणी सोशल मीडिया मुले एका क्षणात जोडले जाते।  या बदला मुए नाते संबंध अधिक सोपे जाले असले तरी त्यांचे स्वरूप गुंता गुंती चेही जाले आहे।  तंत्रध्यानाचा सर्वात मोठा फायदा महंजे अंतर कमी जाले आहे।  वेगवेगया शहरात किम्वा देशात रहनारी कुटुंबे विडियो कॉल द्वारे रोज सम्वाद साधुशक्तात।  मित्रमै त्रिनिंशी संपर्क ठेवने सहज शक्के जाले आहे।  तसेत समान आवडी विचार किम्वा अनुभव असलेली मान से ओनलाइन समुदाया द्वारे एकत्र येवशक्तात जे अनेकान साथी आधार ठरते।</t>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट पॅसेज ए रेडी स्टार्ट परिछित आपल्या देशातील शेती व्यवसा याचे एक दुर्दैव म्हणजे अनेक वर्षांच्या कालावधीनंतर शेतकरी व शेतमजूर यांना आवश्यक असणाऱ्या वाजवी जीवनमानाचा विचार झाला नाही तसेच उत्पादन खर्चाचा विचार करून त्यावर आधारित अशा किफायतशीिर किंमतीची हमी अजून मिळत नाही कारखानदार आपल्या मालाची किंमत स्वत निश्चित करतो व त्याला परवडेल अशा किमतीला तो आपला माल विकतो परंतु शेतकऱ्याने पिकविलेल्या मालाची किंमत बाजारपेठेत लिलावाच्या पद्धतीने केली जाते परिछेत शेतकरी वर्गापैकी मूठभर धनिकांचा वर्ग वगळल्यास बहुसंख्य शेतकरी हे दरिद्री व कर्जबाजारी आहेत त्यातील बहुतेक शेतकरी कनिष्ठ प्रकारचे जीवन तर अनेकजण उपासमारीच्या छायेत कसेबसे जगत आहेत त्यांची नगद पैशांची गरज इतकी तीव्र असते की ते योग्य किंमत येईपर्यंत वाट पाहूच शकत नाहीत सुगीमध्ये किंमती जेव्हा ढासळलेल्या असतात तेव्हाच त्यांना आपला माल मिळेल त्या किंमतीने विकणे भाग पडते परिछेत गरीब शेतकऱ्यांची ही लूट व पिळवणूक थांबविण्यासाठी व त्याच बरोबर बाजारपेठेतील किमतीच्या चढउतारापासून त्यांची मुक्तता करून त्यांच्या मालाला सर्व राज्यभर आणि संपूर्ण हंगामभर एकच भाव मिळावा म्हणून शासन प्रयत्नशील आहे या दिशेने एक प्रयत्न म्हणून कापूस खरेदी योजना पुन्हा हाती घेण्यात आली जो शेतकरी आजपर्यंत केवळ कच्चा कापूस विकत आला आहे त्याला गाठीचा कापूस विकण्याची संधी या योजनामुळे प्राप्त होत आहे</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -726,22 +767,37 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>हे मौक परिक्षे साथी शौठर उतारा बी, पासेज बी, चे ओडियो आहे, काम हे मानवी जीवनाचा अविभाज भाग राहिले आहे.  प्राचीन कायात कामाचा मुख्य उद्देश उपजी विके पूर्ता मर्यादित होता.  शेती करने, शिकार करने किम्मा हस्तकला तयार करने ही कामे मानुस आपल्या कुटूमबाचा गरजा भागवने साथी करत असे  क्या कायात कामाचे मोल हे केवल जग्णे साथी आवश्यक आहे की ना ही, यावर ठरवले जाथ होते.  परंतु कायानुसार समाज, तंत्रद्न्यान आणी जीवन शैली बदलत गेली आणी कामाचे स्वरूप ही बदल्ले</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट महोदय आपले दहा ऑक्टोबर दोन हजार तेवीसचे पत्र मिळाले त्याबद्दल आम्ही आपले आभारी आहोत परिछित आपल्या वरील पत्रात आपण ज्या मालाची मागणी केली आहे त्याचे उत्पादन आम्ही नुकतेच बंद केले आहे कारण त्यासाठी जो कच्चा माल लागतो त्याला परदेशातून हल्ली चांगल्या किमतीला बरीच मागणी येऊ लागली आहे त्यामुळे या देशात तो दिवसेंदिवस महाग होत चालला असून त्याचे आजचे भाव आम्हाला परवडण्यासारखे नाहीत किंबहुना परदेशातील वाढत्या मागणीमुळे चढ्या किमतीत देखील तो माल या देशात दुर्मिळ होत चालला आहे या परिस्थितीत उत्पादनासाठी करावी लागणारी यातायात व खर्च आणि त्यातून शेवटी होणारा नफा यांचा सर्व बाजूननी विचार करून त्या मालाचे उत्पादन बंदच करण्याचा निर्णय आम्हाला नाइलाजाने घ्यावा लागला शिवाय या बाबतीत दुसरी महत्त्वाची गोष्ट अशी आहे की इतके सगळे करून सरून मालाचा उठाव ताबडतोब होईलच याची शाश्वती नाही तसा तो झाला नाही तर त्यासाठी गुंतवलेले भांडवल तर दीर्घकाळ अडकून पडतेच पण त्याखेरीज मालही खराब होऊन फायद्याऐवजी नुकसान सोसण्याची आपत्ती निर्माण होते वरील परिस्थितीत आपली मागणी आम्ही पूर्ण करू शकत नाही याबद्दल आम्हास खेद होतो परिचित आमच्या कंपनीचे दरपत्रक सोबत पाठविले आहे त्यात नमूद केलेल्या मालाची मागणी केल्यास ती पूर्ण करण्यास आम्हाला केव्हाही आनंद वाटेल परिचित आपले विश्वासू</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>हे मौक परिक्षे साथी शोर्ख्र सराव, क्रायल, ओडियो आहे.  अप्यश हां शब्द अईक्ताच अनेकांचा मनात भीती निर्मान होते.  समाजात यशाला गवरव ले जाते, पन अप्यशा कडे दुरलक्ष के ले जाते.  क्या मुले अनेक लोक अप्यशाला कमजोरी समस्तात आणी त्यापासून दूर पएनेचा प्रयत्न करतात.  मात्र प्रत्यक्षात अप्यश हे वयक्तिक विकासा साथी अक्त्यंत आवश्यक अस्ते.  अप्यश मानसाला चिकाटी शिकवते.  जेवहा एकादी गोष्ट अपेक्षे प्रमाने घर्त नाही, तेवहा मानसाला कुन्हा प्रयत्न करावा लागतो.  या प्रक्रियेत मानसिक ताकद वाडते.  अडचनिन्ना सामोरे जान्याची क्षमता विक्सित होते.  अप्यश अनुभवल्या नंतर व्यक्ती स्वताहवर अधिक विश्वास ठेवू लागते.  अप्यश आमुले शिक्णेची संधी मेते.  यश मेयाल्यावर चुका दिसून येत नाही, पन अप्यश त्या स्पष्टपने दाखोते.  काई चुकले, कुठे सुधारणा करावी लागेल है समझते.  अनेक यशस्वी लोकाननी आपल्या आयुशातील अप्यशान मधूनच महत्वाचे धड़े घेतलेले आहेत.</t>
-        </is>
-      </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट ट्रायल पॅसेज रेडी स्टार्ट महाशय पारा आज जगात लोकसंख्या वाढीचा प्रश्न तोंड वासून उभा आहे वेळीच त्याला पायबंद न घातल्यास विपरीत परिणाम झाल्याशिवाय राहणार नाही भारताची एकतीस मार्च एकोणीशे पंच्याऐंशी पर्यंत लोकसंख्या चौऱ्याहत्तर कोटी होती एवढी लोकसंख्या असण्याची मुख्य तीन कारणे आहेत वाढते जन्म प्रमाण घटते मृत्यू प्रमाण व अशिक्षतीपणा</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -778,7 +834,11 @@
           <t>aud1</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>aud2</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>https://hgasggsgkd.s3.ap-south-1.amazonaws.com/marathi+testing+file.m4a</t>
@@ -808,6 +868,9 @@
       <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -872,7 +935,7 @@
       <c r="P5" s="2" t="n"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>English short and 60 words per minute. Passage A. Ready. Start. My dear Vijay Para, I am in receipt  of your letter and noted the contents. If you want to be successful in getting high speed,  you should also cultivate the reading habit. You should also attach as much importance to reading  practice as to the actual note-taking. I would again impress upon you that it is absolutely  necessary that you should read your shorthand notes. Although reading practice is helpful,  transcription is most essential. It is for the errors in the transcript that the shorthand  writer is penalized. Therefore, it is quite useless if you do not pay your attention to transcription  also para. I would say that there is one other method for developing high speed within a very short  period. Select speeches or writings of great men and have them correctly copied in your note book  with the correct outlines and phrases. You should write the same passage over and over again.  you should increase the speed gradually until you are able to write that passage at very high speed.  By following this method, your hand moves freely and your mind will not struggle to think of new outlines  and you will be able to maintain a high speed at all times para. In my practical experience, I have found that  that by merely writing new passages daily in the evening you cannot expect a rapid improvement in the attainment of high speed and it is not a real speed practice.</t>
+          <t>English shorthand, 60 words per minute. Passage A. Ready. Start. My dear Vijay. Para. I am in receipt of your letter and noted the contents. If you want to be successful in getting high speed, you should also cultivate the reading habit. You should also attach as much importance to reading practice as to the actual note-taking. I would again impress upon you that it is absolutely necessary that you should read your shorthand notes. Although reading practice is helpful,  Transcription is most essential. It is for the errors in the transcript that the shorthand writer is penalized. Therefore, it is quite useless if you do not pay your attention to transcription also para. I would say that there is one other method for developing high speed within a very short period. Select speeches or writings of great men and have them correctly copied in your notebook with the correct outlines and phrases. You should write the same passage over and again. You should increase the speed gradually until you are able to write that passage at very high speed by following this method your hand moves freely and your mind will not struggle to think of new outlines and you will be able to maintain a high speed at all times para. In my practical experience, I have found that by merely writing new passages daily in the evening, you cannot expect a rapid improvement in the attainment of high speed and it is not a real speed practice.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -882,22 +945,37 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>English shorthand 60 words per minute. Passage B. Ready. Start. Dear Sir Para, we are in receipt  of your esteemed favour dated 5th of this month and thank you very much for the same.  In this connection, we wish to inform you that the goods of particular quality you want are not readily available.  You are aware that this is the busy season and we have a large number of orders on hand.  However, as you are our permanent customer, we assure you that the goods will be supplied  to you before the end of this month. Please let us know your opinion in this regard as early as possible.  If you are agreeable, kindly fill in the enclosed pro forma and post the same per return of post.  Your reply in this behalf should reach us positively before 20th instant. Otherwise,  it would not be possible for us to accept your orders in the matter. We are also happy  happy to inform you that the remaining goods are being sent to you by passenger train.  The railway parcel receipt and bills in duplicate are dispatched separately by post for your information.  We have taken all precautions to the best of our ability to see that the goods are packed as safely as possible.  We request you kindly to confirm the same. If the goods are damaged in transit,  we assure you that such goods will be replaced at our cost. You may receive the railway parcel receipt and bills on Monday.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 60 words per minute. Passage B. Ready. Start. Dear Sir, Parra, we are in receipt of your esteemed favor dated 5th of this month and thank you very much for the same. In this connection we wish to inform you that the goods of particular quality you want are not readily available. You are aware that this is the busy season and we have a large number of orders on hand. However, as you are our permanent customer, we assure you that the goods will be supplied to you before the end of this month. Please let us know your opinion in this regard as early as possible. If you are agreeable, kindly fill in the enclosed pro forma and post the same per return of post. Your reply in this behalf should reach us positively before 20th instant. Otherwise, it would not be possible for us to accept your orders in the matter. We are also happy to inform you that the remaining goods are being sent to you by passenger train. The railway parcel receipt and bills in duplicate are dispatched separately by post for your information. We have taken all precautions to the best of our ability to see that the goods are packed as safely as possible. We request you kindly to confirm the same. If the goods are damaged in transit, we assure you that such goods will be replaced at our cost. You may receive the railway parcel receipt and bills on Monday.</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>English short hand, 60 words per minute, trial passage. Ready, start.  Dear Sirs Para, we have given careful consideration to the request contained in your letter of 2nd April for the sole agency in your district of our new machine.  We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first class connections  in this type of machinery.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 60 words per minute, trial passage ready. Start. Dear Serves, Para, we have given careful consideration to the request contained in your letter of 2 April for the sole agency in your district of our new machine. We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first class connections in this type of machinery.</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -964,7 +1042,7 @@
       <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 60 WPM.  Passage A. Ready? Start.  Dear Sir, Para, as you are aware, we are one of the largest producers of iron and steel  products, mainly with a view to export from this country.  During the past few years, our exports of these commodities have exceeded Rs. 1 crore  each year while we have been confining ourselves till now to some of the European countries.  We are anxious that we should take full advantage of vast potentialities of the markets in Asia.  We have therefore been planning the expansion of our factory to meet the pressing demands.  In this context, you will kindly appreciate that we would need the fullest cooperation and  help from our department unless and until.  Therefore, we are given the full quota of 2 lakh tons of steel, which we have applied for  on priority basis.  We are afraid our export trade will be greatly affected.  We are anxious as we are sure the government of India too that we should expand our export trade  as much as much as possible and earn the much valuable foreign exchange.  One of the most important considerations in the export trade you will kindly realise is that  that we should keep to the schedule and we cannot do this but for your cooperation in the matter.  It is unfortunate that last year due to variety of factors, we could not get the full quota of our allotment in time,  which had considerably damaged our reputation in the foreign market.  The large units at the intermediaries had for multiple markets…  It is unfortunate that the customers walk will have to be healed and neglected.  That it were difficult to angels andượids.  That is how the customers walk in third时间 reduce the seat of the cost,  especially africольше than the remain its customers in the opinion.  So, this method of the dépendance of the cure that remembers making the commonpuvous and your host essas  Which Meritans is our client at the point station, what people believing have at its Sue's understanding have been</t>
+          <t>English shorthand, 60 WPM, Passage A. Ready, Start. Dear Sir, Para, as you are aware, we are one of the largest producers of iron and steel products, mainly with a view to export from this country. During the past few years, our exports of these commodities have exceeded rupees 1 crore each year, while we have been confining ourselves till now to some of the European countries. We are anxious that we should take full advantage of vast potentialities of the markets in Asia. We have therefore been planning the expansion of our factory to meet the pricing demands. In this context, you will kindly appreciate that we would need the fullest cooperation and help from our department unless and until. Therefore, we are given the full quota of two tons of steel, which we have applied for on priority basis. We are afraid our export trade will be greatly affected. We are anxious as we are sure the government of India to that we should expand our export trade as much as possible and earn the much valuable foreign exchange. One of the most important considerations in the export trade, you will kindly realize is that we should keep to the schedule and we cannot do this but for your cooperation in the matter. It is unfortunate that last year due to variety of factors we could not get the full quota of our allotment in time which had considerably damaged our reputation in the foreign market.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -974,22 +1052,37 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand, 60 WPM. Passage B. Ready? Start.  Dear Sir, Tara, we have received your letter of the seventh instant. Our contract with you was entered into the clear understanding that you will observe  its terms and conditions. We should like to point out that our expectations have not been fulfilled  under the terms of the settlement. The work has to be finished by the middle of May.  And there is no reasonable certainty of this result being achieved.  You had better consider what would be the result of your action if the work you have undertaken is not finished on the date in question.  We should like to have a definite assurance as to your intentions.  You will remember that we went into the matter at great length in our previous communication.  And we should not have had to reopen the subject so soon, but for the way in which our instructions have been disregarded.  We hope you will excuse us for saying so, but it looks as though you will never put your heart  and soul into the work or carry out the terms of the contract.  We cannot resist the conclusion that you could have done more with greater vigilance.  If you could finish work rapidly now, we would not take any technical objection on the ground of delay.  It may seem to you that we are unduly harsh, but on careful consideration, you will find that you are wrong in thinking so.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 60 WPM. Passage B. Ready. Start. Dear Sir, Pera, we have received your letter of the seventh instant. Our contract with you was entered into the clear understanding that you will observe its terms and conditions. We should like to point out that our expectations have not been fulfilled under the terms of the settlement. The work has to be finished by the middle of May and there is no reasonable certainty of this result being achieved, you had better consider what would be the result of your action if the work you have undertaken is not finished on the date in question. We should like to have a definite assurance as to your intentions. You will remember that we went into the matter at great length in our previous communication, and we should not have had to reopen the subject so soon but for the way in which our instructions have been disregarded. We hope you will excuse us for saying so, but it looks as though you will never put your heart and soul into the work or carry out the terms of the contract. We cannot resist the conclusion that you could have done more with greater vigilance. If you could finish work rapidly now, we would not take any technical objection on the ground of delay. It may seem to you that we are unduly harsh but on careful consideration, you will find that you are wrong in thinking so.</t>
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand 60 Words Per Minute  Trial Passage  Ready?  Start  Dear Sirs, Tara,  We have given careful consideration to the request contained in your letter of 2nd April for the sole agency in your district of our new machine.  We have no agency at present in the north of Bombay and as we understand that you are an old established concern  with first class connections in this type of machinery.  Thank you.  Thank you.  Thank you.  Thank you.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 60 words per minute, trial passage. Ready? Start. Dear sirs, para, we have given careful consideration to the request contained in your letter of 2nd April for the sole agency in your district of our new machine. We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first-class connections in this type of machinery.</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1149,7 @@
       <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 60 words per minute. Passage A ready. Start. Dear Sirs Para, I thank you for your prompt reply with enclosures to my letter of the instant regarding my appointment.  I am satisfied with the prospects you hold out and I am worried to show my ability to convince likely customers of the mastery of your productions  over the many replacements now existing.  There are, however, several most important points in the agreement which require adjustment before it can be concluded.  With respect to clothes, I think it would avoid the danger of disputes if it stated exactly what are included.  I am also worried that it should be distinctly understood that I am not expected to be answerable for payments to travelers in connection with commission.  I recommend that you forward each week a check covering the likely amount which I shall disburse holding to your credit any sum remaining in hand.  I respectfully suggest that the sum of thousand rupees be deposited with me for this purpose.  I hope you will have no objection for giving the necessary sanction.  turning to the question of samples.  Turning to the question of samples, I understand these are to be free.  Perhaps you will give instructions for considerable stock of these to be sent passenger trains,  as it is unnecessary for me to say that prospective buyers like to inspect the commodities before giving their orders.  Others respecting calculation of agreement will,  will you kindly state distinctly merely as formality to avoid possibility of future misunderstanding yours faithfully.</t>
+          <t>English shorthand, 60 words per minute. Passage A ready. Start. Dear Sir Spara, I thank you for your prompt reply with enclosures to my letter of the instant regarding my appointment. I am satisfied with the prospects you hold out and I am worried to show my ability to convince likely customers of the mastery of your productions over the many replacements now existing. There are, however, several most important points in the agreement which require adjustment before it can be concluded. With respect to cloths. I think it would avoid the danger of disputes if it stated exactly what are included. I am also worried that it should be distinctly understood that I am not expected to be answerable for payments to travelers in connection with Commission. I recommend that you forward each week a check covering the likely amount which I shall disburse holding to your credit any sum remaining in hand. I respectfully suggest that the sum of thousand rupees be deposited with me for this purpose. I hope you will have no objection for giving the necessary sanction. Turning to the question of samples, I understand these are to be free. Perhaps you will give instructions for considerable stock of these to be sent passenger train as it is unnecessary for me to say that prospective buyers like to inspect the commodities before giving their orders respecting calculation of agreement will you kindly state distinctly merely as formality to avoid possibility of future misunderstanding yours faithfully.</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -1066,22 +1159,37 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 60 words per minute. Passage B. Ready? Start. Dear friend, Para, an opportunity  is provided for everybody in this country to support the efforts of the government to make  this country self-sufficient financial and army. The scheme of gold bonds is so attractive that  if properly explained, it will catch the imagination and swell the gold bond  fund. What is to be explained to the mass of our population is the fact that gold in their  possession, which does not yield any income invested to government for years, will not  only bring some income to the individual but will save the huge interest which government  of India have otherwise to pay to other countries every year in foreign exchange and enable the  government to repurchase gold out of the saving of interest in foreign exchange. In years, this country  will save crores of rupees in foreign exchange by simply parting with gold for this limited period. There  cannot be any greater opportunity for the people of this country than the investment in gold bonds. As you know,  many schemes, howsoever beneficial and praiseworthy they might be, do not catch the imagination unless they are given  proper publicity and explained. I am confident the sincere efforts in every state will swell the gold bond fund much beyond our expectations.  Nationally, it will raise the spirit and boost up the enthusiasm. Internationally, it will raise the prestige and create confidence in ability of this country to be self-sufficient.  .  .</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 60 words per minute. Passage B. Ready? Start. Dear friend, Para, an opportunity is provided for everybody in this country to support the efforts of the government to make this country self-sufficient financial and army. The scheme of gold bonds is so attractive that, properly explained, it will catch the imagination and swell the gold bond fund. What is to be explained to the mass of our population is the fact that gold in their possession, which does not yield any income invested to government for years will not only bring some income to the individual but will save the huge interest which government of India have otherwise to pay to other countries every year in foreign exchange and enable the government to repurchase gold out of the saving of interest in foreign exchange. In years, this country will save croars of rupees in foreign exchange by simply parting with gold for this limited period. There cannot be any greater opportunity for the people of this country than the investment in gold bonds. As you know, many schemes, how so ever beneficial and praiseworthyworthy they might be, do not catch the imagination unless they are given proper publicity and explained, I am confident the sincere efforts in every state will swell the spirit and boost up the enthusiasm internationally. It will raise the prestige and create confidence in ability of this country to be self-sufficient.</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>English short hand, 60 words per minute, trial passage. Ready, start.  Dear Sirs Para, we have given careful consideration to the request contained in your letter of 2nd April for the sole agency in your district of our new machine.  We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first class connections  in this type of machinery.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 60 words per minute, trial passage ready. Start. Dear Serves, Para, we have given careful consideration to the request contained in your letter of 2 April for the sole agency in your district of our new machine. We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first class connections in this type of machinery.</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1256,7 @@
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 60 words per minute, passage A. Ready? Start.  Dear Krishna, many thanks for your report, which I have not yet had time to analyze a casual reading of it.  However, it is sufficient to show that you have done extremely well during the past three months and I heartily congratulate you upon the excellent result obtained.  I will let you have my detailed comments early next week.  At most caution in dealing with him, especially if he asks for credit or for any privileges of a financial character.  I also write to tell you that I have been discussing with Mr. Bajaj the possibilities of an extension of your area.  I am also quite sure that we will achieve it very soon.  I think that it will be practicable to reduce the time that you find it necessary to spend in the near east, which on the whole is not profitable.  As other areas that have not been yet fully worked.  A definite decision will not be reached until next month.  In the meantime, I shall be glad if you will let me have your opinion upon one or two points.  Can you find an expert assistant who will be able to relieve you of some of the indoor work awaiting your reply?  So good.  Bye.  Thank you.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.  Take care.</t>
+          <t>English shorthand, 60 words per minute. Passage 8. Ready? Start. Dear Krishna, Paira, many thanks for your report, which I have not yet had time to analyze a casual reading of it. However, it is sufficient to show that you have done extremely well during the past three months and I heartily congratulate you upon the excellent result obtained. I will let you have my detailed comments early next week. The purpose of this letter is to warn you that Mr. Vijay Patil mentioned on page 4 of your report is most unreliable and to ask you to exercise the utmost caution in dealing with him, especially if he asks for credit or for any privileges of a financial character. I also write to tell you that I have been discussing with Mr. Bajaj the possibilities of an extension of your area. I am also quite sure that we will achieve it very soon. I think that it will be practicable to reduce the time that you find it necessary to spend in the near east which on the whole is not profitable as other areas that have not been yet fully worked. A definite decision will not be reached until next month. In the meantime, I shall be glad if you will let me have your opinion upon one or two points. Can you find a expert assistant who will be able to relieve you of some of the endore work awaiting your so good by thank you take care</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -1158,22 +1266,37 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand, 60 words per minute, passage B. Ready? Start.  Dear Sirs, we acknowledge receipt of your letter of 15 May while thanking you for the consideration you have been extending to us.  We have below given our comments on the points raised by you.  Our office premises are in the famous Bank Street, easily available to all sections of people.  The showroom is in the ground floor and is spacious enough for keeping all types of agricultural machinery  and implements you want us to display.  And as you know, the office is located in the first floor.  We have already taken steps for recruitment of required personnel  we undertake to give adequate security as desired by you for the machinery in display  and inspection by the intending purchasers.  It would, however, be advisable of this stock is booked to your account initially.  We assure you that we will take all responsibility for their servicing and good condition.  We are pleasant for the other terms and conditions specified by you accepting the commission on credit sales.  As you are aware, we are in the line.  Since we are to be responsible for the realization on credit sales,  it would be reasonable if commission of percent on cash sales retained for credit sales as well.  We are expecting good demand for supply of spare parts also.  As the space limited in present premises,  we are bargaining for lease of the land.  Well, euros can pay in the красивű motherboard.  UKUF  ESOIN  ESOIN  езж  ESOIN  ESOIN  ESOIN</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 60 words per minute. Passage B. Ready. Start. Dear Sirs, Pera, we acknowledge receipt of your letter of 15 May, while thanking you for the consideration you have been extending to us. We have below given our comments on the points raised by you. Our office premises are in the famous bank street easily available to all sections of people. The showroom is in the ground floor and is spacious enough for keeping all types of agricultural machinery and implements you want us to display. And as you know, the office is located in the first floor. We have already taken steps for recruitment of required personnel trained in the use of agricultural implements we undertake to give adequate security as desired by you for the machinery in display and inspection by the intending purchasers. It would, however, be advisable of this stop is booked to your account initially. We assure you that we will take all responsibility for their servicing and good condition. We are pleasant for the other terms and conditions specified by you accepting the Commission on credit sales. As you are aware, we are in the line. Since we are to be responsible for the realization on credit sales, it would be reasonable if commission of percent on cash sales retained for credit sales as well. We are expecting good demand for supply of spare parts also. As the space limited in present premises, we are bargaining for lease of the land.</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand, 60 words per minute, trial passage, ready, start.  Dear Sirs, we have given careful consideration to the request contained in your letter of 2nd April for the sole agency in your district of our new machine.  We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first class connections in this type of market.  Thank you.  Thank you.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 60 words per minute, trial passage. Ready, start. Dear Sirs, Pera, we have given careful consideration to the request contained in your letter of 2 April for the sole agency in your district of our new machine. We have no agency at present in the north of Bombay and as we understand that you are an old established concern with first-class connections in this type of machinery.</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1363,7 @@
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>English shorthand. 80 words per minute. Passage A. Ready. Start para. There is abnormal delay in  obtaining revenue records and farmers have to go from pillar to post to obtain their records  and have to spend heavy amounts obtaining no objection certificate according to the Act  normally 1 to 2 months. If this provision is removed from the Act, our bank will be able to sanction  loans within 15 days. The bank has already moved the government for amending the Act and as the  amendment would take some time, I submit to the Honourable Ministers to get an ordinance issued  dispensing with the obtaining of no objection certificate para. At present, state government  has given exemption of stamp duty up to 10,000 only with the increase in the cost of labour and material.  The investment needed to individual borrower for different purposes exceeds 10,000 rupees and  goes up to 30,000 rupees as the borrowers cannot meet the huge cost on account of stamp duty and  registration charges. I request the state government to exempt the stamp duty and registration charges for all  types of loans irrespective of the amount advanced by the land development banks as is vogu in other states  in other states. Yesterday, we celebrated the prestigious mark of sanctioning loans for 1 lakh irrigation wells.  All these wells could be better utilized provided there is supply of power for lifting water.  non-supply of power at a time required by the farmer is a great setback in increasing production.  In spite of making deposits with Karnataka electricity board, the board is pleading inability to supply  power. Unless electric power is supplied, the investment on the well becomes unproductive. May I request  the government to solve this problem with the electricity board by giving priority to this item in their program para.  I now conclude and express my sincere gratitude to the Honourable Chief Minister for Agriculture who have  spent their precious time with us and give their valuable advice.  Thank you.  Thank you.  Thank you.</t>
+          <t>English shorthand, 80 words per minute. Passage A. Ready. Start para. There is abnormal delay in obtaining revenue records and farmers have to go from pillar to post to obtain their records and have to spend heavy amounts, obtaining no objection certificate according to the Act normally one to two months. If this provision is removed from the Act, our Bank will be able to sanction loans within 15 days. The Bank has already moved the government for amending the Act and as the amendment would take some time, I submit to the Honourable Ministers to get an ordinance issued dispensing with the obtaining of no objection certificate para. At present, state government has given exemption of stamp duty up to 10,000 only. With the increase in the cost of labor and material, the investment needed to individual borrower for different purposes exceeds 10,000 rupees and goes up to 30,000 rupees as the borrowers cannot meet the huge cost on account of stamp duty and registration charges. I request the state government to exempt the stamp duty and registration charges for all types of loans, irrespective of the amount advanced by the land development banks as is vogueu in other states' para. Yesterday, we celebrated the prestigious mark of sanctioning loans for one-luck irrigation whales. All these whales could be better utilized, provided there is supply of power for lifting water. Non-supply of power at a time required by the farmer is a great setback in increasing production in spite of making deposits with Karnataka Electricity Board. The board is ple pleading inability to supply power. Unless electric power is supplied, the investment on the well becomes unproductive. May I request the government to solve this problem with the Electric Board by giving priority to this item in their program para. I now conclude and express my sincere gratitude to the Honorable Chief Minister for Agriculture, who have spared their precious time with us and give their valuable advice.</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -1250,22 +1373,37 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>English short and 80 words per minute. Passage B. Ready. Start. Dear Sir. Para. I am happy to inform you that your tender for the supply of stationery and other materials to our main office at Pune and various branch offices  located in Maharashtra, Uttar Pradesh and Madhya Pradesh has been accepted. You are therefore requested to arrange to remit a sum of rupees 5000 as security deposit on or before 10th of this month.  This amount may be paid either in cash or through bank draft drawn in favor of our managing director.  This security deposit will be refunded to you with 5% interest as soon as you complete the contract para.  In this connection, I would like to make it clear once again that all the materials should confirm to the quality you have quoted in your tender.  The actual requirements of our various offices is furnished in the statement appended to this letter.  The goods shall have to be delivered in good condition at the addresses given in the enclosed statement.  You have to bear the transportation and all other incidental expenses in this regard.  The time schedule given should also be adhered to in the event of not adhering to the time schedule.  You will have to renounce 5% of the total bill amount.  Further, if you fail to supply the goods before the end of this month, we will be at liberty to refuse goods at your cost and make alternate arrangements to suit our convenience.  Hence, the payment will be made as per the rates quoted by you and no request for higher rates will be entertained for any reason para.  You are also required to send us a copy of the pro-pharma invoice and delivery note duly signed by our branch managers for having received the materials in good condition.  Your bills will be settled within one week from the date of your furnishing the above documents para.  Thanking you once again, yours faithfully.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 80 words per minute, passage B. Ready. Start. Dear Sir, Para, I am happy to inform you that your tender for the supply of stationary and other materials to our main office at Pune and various branch offices located in Maharashtra, Uttar Pradesh and Madhapradesh has been accepted. You are. Therefore, requested to arrange to remit a sum of rupees, $5,000 as security deposit on or before 10th of this month. This amount may be paid either in cash or through bank draft drawn in favor of our managing director. This security deposit will be repunded to you with 5% interest as soon as you complete the contract para. In this connection, I would like to make it clear once again that all the materials should confirm to the quality you have quoted in your tender. The actual requirements of our various offices is furnished in the statement appended to this letter. The goods shall have to be delivered in good condition at the addresses given in the enclosed statement. You have to bear the transportation and all other incidental expenses in this regard. The time schedule given should also be adhered to, in the event of not adhering to the time schedule, you will have to renounce 5% of the total bill amount. Further, if you fail to supply the goods before the end of this month, we will be at liberty to refuse goods at your cost and make alternate arrangements to suit our convenience. The payment will be made as per the rates quoted by you and no request for higher rates will be entertained for any reason, para. You are also required to send us a copy of the pro forma invoice and delivery note duly signed by our branch managers for having received the materials in good condition. Your bills will be settled within one week from the date of your furnishing the above documents para, thanking you once again, yours, faithfully.</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>English shortened 80 words per minute. Trial passage. Ready. Start. Para. As you have moved  into our new offices over one week end last May and on the Monday morning, we were operating  in our new surroundings. As planned, the whole exercise was a great credit to the chief office  staff and such was their cooperation that there was no hold up in the normal running of our business  para. Now that we have been in occupation for some months, it is a great pleasure to report  our complete satisfaction with the new office.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand 80 words per minute. Trial passage ready. Start. Para. As you have moved into our new offices over one week and last May, and on the Monday morning, we were operating in our new surroundings as planned. The whole exercise was a great credit to the chief office staff and such was there. Cooperation that there was no hold up in the normal running of our business para. Now, that we have been in occupation for some months. It is a great pleasure to report our complete satisfaction with the new office.</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1470,7 @@
       <c r="P10" s="2" t="n"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 80 words per minute. Passage A. Ready? Start.  Dear Sirs Para, we thank you for your letter of the second instant enclosing a cheque for Rs. 30,000 in full settlement of our three outstanding bills.  In this connection, we have great pleasure to inform you that we are having clearance sale of our toilet articles  as it is necessary for us to dispose of some of our stocks as early as possible.  We are sending herewith copy of our latest catalog as well as few pamphlets which we think you will like to have.  Our catalog describes the different items fully.  You will please note that each item has been given separate code number.  In order to enable you to make a selection, we are also sending per passenger train few samples of the different toilet items  that we can offer.  In view of the fact that this is our last clearance sale, we are giving special discount on this occasion.  We hope you will take advantage of this special offer and favor us with your valuable order which will receive our prompt attention.  We have also to inform you that during the next month, we propose to increase the prices of number of items at present included in our catalog.  The increases have become necessary in view of the higher costs that we now have to incur in purchase locally of some of our raw materials  which used to come formerly from the United States, in spite of our best efforts, we could not get the local materials at cheaper rate.  In the circumstances, we have no alternative but to increase our prices.  We extremely regret that we are forced to pass on the higher charges to our customers.  But at the present time, this is the only course which we can follow.  As you are one of our most important dealers, we think we should not take you by surprise by revising our rates without notice.</t>
+          <t>English shorthand, 80 words per minute. Passage A. Ready. Start. Dear Sir's Para, we thank you for your letter of the second instant enclosing a check for rupees 30,000 in full settlement of our three outstanding bills. In this connection, we have great pleasure to inform you that we are having clearance sale of our toilet articles as it is necessary for us to dispose of some of our stocks as early as possible. We are sending here with copy of our latest catalog, as well as few pamphlets which we think you will like to have. Our catalog describes the different items fully. You will please note that each item has been given separate code number. In order to enable you to make a selection, we are also sending per passenger train few samples of the different toilet items that we can offer. In view of the fact that this is our last clearance sale, we are giving special discount on this occasion. We hope you will take advantage of this special offer and favor us with your valuable order which will receive our prompt attention. We have also to inform you that during the next month we propose to increase the prices of number of items at present included in our catalog. The increases have become necessary in view of the higher costs that we now have to incur in purchase locally of some of our raw materials which used to come formerly from the United States. In spite of our best efforts, we could not get the local materials at cheaper rate. In the circumstances, we have no alternative but to increase our prices. We extremely regret that we are forced to pass on the higher charges to our customers. But at the present time, this is the only course which we can follow. As you are one of our most important dealers, we think we should not take you by surprise by revising our rates without notice.</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -1342,22 +1480,37 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 80 words per minute.  Passage B.  Ready? Start.  Dear shareholders, Para, I have pleasure in informing you that your company's automobile, tires and tubes plant  at Pune was successfully commissioned on the month of February.  After the initial trials, commercial production of automobile tires has commenced and the product is being marketed.  The production of tires for trucks and buses, scooters has commenced.  The production of other types of tires for tractors, motorcycles is being gradually taken up coming few months.  As you are aware, this plant has been set up with technical collaboration of General Tire International Company.  And under the collaboration terms, number of foreign technicians are at our plant for training our workers  as well as for assisting us in attaining production targets both in terms of quality and quantity.  A good number of Vikrant tires have been on the road for some time now.  It is indeed heartening to note that they have been well received in market and the response with regard to quality and performance from the consumers is very encouraging.  We have also exported our tires to few countries and have substantial orders on hand awaiting executions.  We shall soon be marketing steel-belted emperor tires both for trucks and cars for the first time in the country.  Emperor tires are the latest innovation in the field of tire technology.  They give up to 100% extra mileage, nearly 10% saving fuel consumption, better road grip and more riding comfort.  Emperor tires will also open new vistas for exports because the world trend is shifting towards the use of such tires.  The company has already established effective distribution organization throughout the country.  You will be glad to know that we have already made supplies to state road transport corporations.  I would request those of you who have not exchanged the receipt letter of allotment for the share certificates from the company to do so at the earliest.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 80 words per minute. Passage B. Ready Start. Dear shareholders, Para, I have pleasure in informing you that your company's automobile tires and tubes planned at Pune was successfully commissioned on the month of February. After the initial trials, commercial production of automobile tires has commenced and the product is being marketed. The production of tires for trucks and buses, scooters has commenced the production of other types of tires for tractors, motorcycles, is being gradually taken up coming few months. As you are aware, this plant has been set up with technical collaboration of General Tyre International Company and under the collaboration terms number of foreign technicians are at our plant for training our workers as well as for assisting us in attaining production targets both in terms of quality and quantity. A good number of Pikrant tyres have been on the road for some time now. It is indeed threatening to note that they have been well received in market and the response with regard to quality and performance from the consumers is very encouraging. We have also exported our tires to few countries and have substantial orders on hand awaiting executions. We shall soon be marketing steel-belted tyres, both for trucks and cars, for the first time in the country. Emperor tires are the latest innovation in the field of tire technology. They give up to 100% extra mileage, nearly 10% saving fuel consumption, better road, grip, and more riding comfort. Emperor tires will also open new vistas for exports because the world trend is shifting towards the use of such tires. The company has already established effective distribution organization throughout the country. You will be glad to know that we have already made supplies to state road transport corporations. I would request those of you who have not exchanged the receipt letter of allotment for the share certificates from the company to do so at the earliest.</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand  80 words per minute  Trial Passage  Ready? Start  As you have moved into our new offices  over one week end last May  and on the Monday morning  We were operating in our new surroundings  as planned  The whole exercise was a great credit  to the chief office staff  and such was their cooperation  that there was no hold up  in the normal running of our business  Now that we have been in occupation  for some months  It is a great pleasure to report our complete satisfaction with the new office  Thank you so much for listening to the application of these!  Outro music  It is a great inquiry  to our  of the public  and also to talk about the way</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 80 words per minute, trial passage. Ready? Start. As you have moved into our new offices over one week end last May. And on the Monday morning, we were operating in our new surroundings as planned. The whole exercise was a great credit to the chief office staff and such was their cooperation that there was no hold up in the normal running of our business. Now that we have been in occupation for some months, it is a great pleasure to report our complete satisfaction with the new office.</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1577,7 @@
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 80 words per minute, passage A. Ready, start.  Dear Sirs Para, we have pleasure in sending you a sample packet of our modern soap powder,  which we have placed on the market. As a result of a long and careful research, this product  has been brought into being. We are confident that it will fulfill a long-felt need from the  catalogue enclosed. You will find that it possesses many special merits which place it ahead of other  competitors. It is highly economical. It dissolves readily in water and cleans all kinds of clothes  quickly. The use of this new powder will save a lot of labour in rubbing and rinsing. 20 grams of  powder mixed in a bucket full of water will work wonders even with a dozen pieces of clothes. A  novel feature added to this is that it acts equally well on any type of clothes. Moreover,  it gives a longer life to the clothes. We have engaged our representatives in the districts all over the  country in order to carry on door-to-door canvassing of our product. They explain to the consumers the  better quality of our soap powder by means of practical demonstration. We have been receiving many  inquiries from different parts of the country. This goes to proof that the public at large have recognized  the merits of the product. We are therefore confident that it is usefulness will easily enable you to find a  a ready market. The terms of our offer of this unique product are very liberal. It has been priced  at a very economical level so as to be within the easy reach of the common man. We offer a 15% discount  discount with 30 days credit on all purchase above 1000 rupees. The goods will be dispatched promptly and  delivered right at your stores, the freight charges being borne by us. We now request you to consider our offer  keeping in view the favorable terms. Thank you. Yours faithfully.</t>
+          <t>English shorthand, 80 words per minute, passage A. Ready. Start. Dear Sir's Para, we have pleasure in sending you a sample packet of our modern soap powder which we have placed on the market as a result of a long and careful research this product has been brought into being. We are confident that it will fulfill a long-failed need from the catalog enclosed. You will find that it possesses many special merits which place it ahead of other competitors. It is highly economical. It dissolves readily in water and cleans all kinds of clothes quickly. The use of this new powder will save a lot of labor in rubbing and rinsing 20 grams of powder mixed in a bucket full of water will work wonders even with a dozen pieces of clothes, a novel feature added to this is that it acts equally well on any type of cloth. Moreover, it gives a longer life to the clothes. We have engaged our representatives all over the clothes. We have engaged our representatives in the districts all over the country in order to carry on door-to-door canvassing of our product. They explain to the consumers the better quality of our soap powder by means of practical demonstration. We have been receiving many inquiries from different parts of the country. This goes to proof that the public at large have recognized the merits of the product. We are. Therefore, confident that it is usefulness will easily enable you to find a ready market. The terms of our offer of this unique product are very liberal. It has been priced at a very economical level so as to be within the easy reach of the common man. We offer a 15% discount with 30 days credit on all purchase above thousand rupees. The goods will be dispatched promptly and delivered right at your stores, the freight charges being borne by us. We now request you to consider our offer keeping in view the favorable terms para, thanking you, yours, faithfully.</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1434,22 +1587,37 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>English shorthand 80 words per minute. Passage B. Ready? Start.  Dear Sir Para, we wish to refer to the discussion held in your chambers on the 10th instant regarding the supply of electronic digital clocks to various branches of your bank.  As already informed by our representative, we can supply your complete requirement and arrange to install clocks at various branches within period of about month from the date of firm orders.  However, we wish to make it clear that the cost of clock would go up in case installation of clocks at different parts of the state has to be done by us.  Since we have to depute our service engineer and his assistant duly meeting their travel expenses.  As such, we suggest to you to take delivery of your requirement at your head office and arrange to distribute to the branches.  We are prepared to provide necessary training in installation and operation of the clock to your staff coming from various branch offices.  The process of installation and operation are quite simple and one of your staff attached to watch and ward duties at the respective places can be trained fully within an hour or two.  Regarding the design and color of the clock suggested by you, we calculated the production cost and we wish to indicate that it involves additional cost.  However, in view of your bulk orders, we are prepared to accept your offer of rupees 2000 per clock.  We need hardly stress here that we are the pioneers in the manufacture of electronic digital clock with large size display.  And so far, we have supplied thousands of clocks to various banks, public sector undertakings, including railway and bus stations.  We have pleasure in accepting your offer and assure you of our best services.  Our terms and conditions include the supply of clocks within a month from the date of firm orders and payment against delivery.  We also offer one-year guarantee for any manufacturing defect.  We also offer one-year guarantee for any manufacturing defect.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 80 words per minute, passage B. Ready? Start. Dear Sir, Para, we wish to refer to the discussion held in your chambers on the 10th instant regarding the supply of electronic digital clocks to various branches of your bank. As already, informed by our representative, we can supply your complete requirement and arrange to install clocks at various branches within period of about month from the date of firm orders. However, we wish to make it clear that the cost of clock would go up in case installation of clocks at different parts of the state has to be done by us since we have to depute our service engineer and his assistant duly meeting their travel expenses. As such, we suggest to you to take delivery of your requirement at your head office and arrange to distribute to the branches. We are prepared to provide necessary training in installation and operation of the clock to your staff coming from various branch offices the process of installation and operation are quite simple and one of your staff attached to watch and ward duties at the respective places can be trained fully within an hour or two. Regarding the design and color of the clock suggested by you, we calculated the production cost and we wish to indicate that it involves additional cost. However, in view of your bulk orders, we are prepared to accept your offer of rupees 2,000 per clock. We need hardly stress here that we are the pioneers in the manufacture of electronic digital clock with large size display. And so far, we have supplied thousands of clocks to various banks, public sector undertakings, including railway and bus stations. We have pleasure in accepting your offer and assure you of our best services. Our terms and conditions include the supply of clocks within a month from the date of firm orders and payment against delivery. We also offer one year guarantee for any manufacturing defect.</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>English shortened 80 words per minute. Trial passage. Ready. Start. Para. As you have moved  into our new offices over one week end last May and on the Monday morning, we were operating  in our new surroundings. As planned, the whole exercise was a great credit to the chief office  staff and such was their cooperation that there was no hold up in the normal running of our business  para. Now that we have been in occupation for some months, it is a great pleasure to report  our complete satisfaction with the new office.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand 80 words per minute. Trial passage ready. Start. Para. As you have moved into our new offices over one week and last May, and on the Monday morning, we were operating in our new surroundings as planned. The whole exercise was a great credit to the chief office staff and such was there. Cooperation that there was no hold up in the normal running of our business para. Now, that we have been in occupation for some months. It is a great pleasure to report our complete satisfaction with the new office.</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1684,7 @@
       <c r="P12" s="2" t="n"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 80 words per minute.  Passage A. Ready. Start.  Dear Sirs,  We thank you for your letter of 1st February asking for the terms and conditions for the supply of printing and developing machines of the specification mentioned therein.  We greatly appreciate your interest for the said machine but regret to inform you that the machine you require is not readily available with us.  In this connection, when we had requested our principals at Mumbai to intimate the stock position and the costs thereof,  our Mumbai office informs that they have only one machine of the said specification but regrets its inability to quote for Pune price due to transport and other difficulties.  They state that the machines at Mumbai will cost Rs. 2000 exclusive of local taxes and advice that the purchaser should arrange for its career.  For your study, we are enclosing a booklet showing all the mechanical details.  We wish to bring to your kind notice that there are two other types of printing and developing machines manufactured by a well-known Nagpur firm and are available from our ready stock.  The machines are of latest design and strongly built with excellent finish.  These machines prove to be more economical in the long run though the initial cost is slightly high.  We hasten to assure you that this slightly higher cost is negligible when compared to the use and performance of the machine.  In this connection, it may be stated that we have quite a large number of orders on hand for these machines  and we will be able to comply with your requests only after two months from the date of receipt of your firm order.  However, we assure you that we will try our utmost to deliver the machine earlier if the transport position improves.  Two booklets regarding the above types of machines are enclosed herewith.  From a study, you will find certain mechanical and practical advantages over the other type of machines.</t>
+          <t>English shorthand, 80 words per minute. Passage A. Ready. Start. Dear Sirs. We thank you for your letter of 1 February asking for the terms and conditions for the supply of printing and developing machines of the specification mentioned therein. We greatly appreciate your interest for the said machine, but regret to inform you that the machine you require is not readily available with us. In this connection, when we had requested our principles at Mumbai to intimate the stock position and the cost. Thereof our Mumbai office informs that they have only one machine of the said specification but regrets its inability to quote for Pune price due to transport and other difficulties. They state that the machines at Mumbai will cost rupees $2,000 exclusive of local taxes and advice that the purchaser should arrange for its career. For your study, we are enclosing a booklet showing all the mechanical details. We wish to bring to your kind notice that there are two other types of printing and developing machines manufactured by a well-known Nagpur firm and are available from our ready stock. The machines are of latest design and strongly built with excellent finish. These machines prove to be more economical in the long run, though the initial cost is slightly high, we hasten to assure you that this slightly higher cost is negligible when compared to the use and performance of the machine. In this connection, it may be stated that we have quite a large number of orders on hand for these machines and we will be able to comply with your request only after two months from the date of receipt of your firm order. However, we assure you that we will try our utmost to deliver the machine earlier if the transport position improves. Two, booklets regarding the above types of machines are enclosed here with. From a study, you will find certain mechanical and practical advantages over the other type of machines.</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
@@ -1526,22 +1694,37 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 80 words per minute.  Passage B.  Ready.  Start.  Dear Sir, Para, we are in receipt of your complaint about the low quality of the goods supplied to you.  We must, however, state that it has caused us considerable surprise because such complaint about the quality of our product has been received from you only in our smooth business.  With regard to our mandate sent to you by railway parcel, we are definitely of a different opinion to that stated in your letter.  It is our practice to examine the products carefully prior to packing and only after confirmation that it is exactly the same as required by the customer, it will be packed.  Therefore, our clerk in the packing department is in a position to deny that the goods sent to you were in any way inferior to the sample sent by us to you earlier along with quotation.  As regards the color, your complaint that it is much darker is only an overstated.  We have again compared your sample piece with reference to sample taken from consignment sent to you and found that the color is exactly the same.  In view of the above facts, we desire to know from you why we shall be called upon to make any allowance when we have delivered the goods exactly to your order.  However, in every respect, we are required to come to conclusion that someone at your side is not acting honestly with an intention to cause trouble to us and claim an allowance from us.  We are sorry to inform you that we are not satisfied with the manner in which you treat mandates as we have to allow some claim or suffer some loss on every mandate sent to you.  We are afraid to think what would be our ultimate loss on this business with you if we go on in this way.  However, we look forward to better understanding between us in future.  Better, better, yours, faithfully.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 80 words per minute. Passage B. Ready. Start. Dear sir, para, we are in receipt of your complaint about the low quality of the goods supplied to you. We must, however, state that it has caused us considerable surprise because such complaint about the quality of our product has been received from you only in our smooth business. With regard to our mandate sent to you by railway parcel, we are definitely of a different opinion to that stated in your letter. It is our practice to examine the products carefully prior to packing and only after confirmation that it is exactly the same as required by the customer. It will be packed. Therefore, our clerk in the packing department is in a position to deny that the goods sent to you were in any way inferior to the sample sent by us to you along with quotation. As regards the color, your complaint that it is much darker is only an overstated. We have again compared your sample piece with reference to sample taken from consignment sent to you and found that the color is exactly the same. In view of the above facts, we desire to know from you why we shall be called upon to make any allowance when we have delivered the goods exactly to your order in every respect. We are required to come to conclusion that someone at your side is not acting honestly with an intention to cause trouble to us and claim an allowance from us. We are sorry to inform you that we are not satisfied with the manner in which you treat mandates as we have to allow some claim or suffer some loss on every mandate sent to you. We are afraid to think what would be our ultimate loss on this business with you if we go on in this way. However, we look forward to better understanding between us in future, para, yours, faithfully.</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 80 words per minute.  Trial passage.  Ready?  Start.  As you have moved into our new offices over one week end last May and on the Monday morning, we were operating in our new surroundings as planned.  The whole exercise was a great credit to the chief office staff and such was their cooperation that there was no hold up in the normal running of our business.  Tara. Now that we have been in occupation for some months, it is a great pleasure to report our complete satisfaction with the new office.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 80 words per minute. Trial passage. Ready, start. As you have moved into our new offices over one week and last May and on the Monday morning, we were operating in our new surroundings as planned. The whole exercise was a great credit to the chief office staff and such was their cooperation that there was no hold up in the normal running of our business. Tara. Now that we have been in occupation for some months, it is a great pleasure to report our complete satisfaction with the new office.</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1791,7 @@
       <c r="P13" s="2" t="n"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute, passage A. Ready? Start.  Dear friends, Para, it is my privilege once again to welcome you all to the 10th Annual General Meeting of the company today.  As the director's report and accounts of your company for the year ended 30th June have been in your hands for some time.  I should like with your approval to take them before I touch on the present economic conditions in the country.  I feel it would be helpful as a background to refer to some of the points in my speech last year.  I had expressed certain fears on that occasion and made a reference to the drop in our agricultural output.  Progressing inflation, growing shortage of working capital, the difficulties faced by textile industry and last but not the least, conditions arising from new oil prices.  I also mentioned on that occasion that a tendency was developing for under-utilization of installed capacities and increasing unemployment,  particularly among the qualified class.  Power cuts imposed at that time resulted in sharp fall in production as they do so even at present in some parts of the country.  The effect of all these factors naturally led to so many events and had already shown the bad results.  We have now put our hopes on few point economic program brought about by the Prime Minister under conditions which are definitely better than what they were earlier.  I hope that conditions will improve rapidly in the coming year.  However, you will have observed that the said program is a real approach to our economic condition and lays down for the first time in our history economic priorities for achieving social justice  so that we can confer on weaker sections of the society a hope of better opportunities than the mere privilege of a vote which independence had brought forth for them.  Para, coming now to our own operations, I am sure you are pleased with the results of our company which have been substantially better than those reflected during the last year.  In fact, on the whole, the tyre industry has had a successful year of operation in spite of number of difficulties.  This happy position can be attributed to decontrol of prices of tyres from April and other favourable factors,  excise duty and other indirect taxes which were imposed on the industrial output in order to cover up the margins during the days of inflation are today affecting off-take.</t>
+          <t>English shorthand, 100 words per minute, passage A. Ready, start. Dear friends, Para, it is my privilege once again to welcome you all to the 10th annual general meeting of the company today. As the director's report and accounts of your company for the year ended, 30th June have been in your hands for some time. I should like, with your approval, to take them. Before I touch on the present economic conditions in the country, I feel it would be helpful as a background to refer to some of the points in my speech last year. I had expressed certain fears on that occasion and made a reference to the drop in our agricultural output. Progressing inflation, growing shortage of working capital, the difficulties faced by textile industry, and last but not the least, conditions arising from new oil prices. I also mentioned on that occasion that a tendency was developing for underutilization of installed capacities and increasing unemployment, particularly among the qualified class. Power cuts imposed at that time resulted in sharp fall in production, as they do so even at present in some parts of the country. The effect of all these factors naturally led to so many events and had already shown the bad results. We have now put our hopes on few points. Economic program brought about by the Prime Minister under conditions which are definitely better than what they were earlier. I hope that conditions will improve rapidly in the coming year. You will have observed that the saidID program is a real approach to our economic condition and lays down for the first time in our history. Economic priorities for achieving social justice so that we can confer on weaker sections of the society a hope of better opportunities than the mere privilege of a vote which independence had brought forth for them. Para, coming now to our own operations, I am sure you are pleased with the results of our company, which have been substantially better than those reflected during the last year. In fact, on the whole, the tire industry has had a successful year of operation in spite of number of difficulties. This happy position can be attributed to decontrol of prices of tires from April and other favorable factors, exercise duty and other indirect taxes which were imposed on the industrial output in order to cover up the margins during the days of inflation are today affecting of tech.</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
@@ -1618,22 +1801,37 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute, passage B. Ready? Start.  Ladies and gentlemen, para, I am happy to be with you this morning and to associate myself with this pleasant function.  On this occasion, I would like to state that every person who is not dealing with a specific subject in an expert way would naturally like to go in for generalizations.  I am not an expert in any subject and so I can say many things about many subjects.  Looking at this institute from a distance and going through its publications, it seems to me that it has been making good progress.  We have been informed that similar institutes in other countries have begun to appreciate the work of this institute.  There can be no doubt about the importance of the work which you are called upon to do.  I am glad that from a small annual business session, this gathering of so many distinguished persons will spread out into a conference on a specific subject matter, namely recruitment for the public services.  I feel that this is something really solid and worthwhile and would bring definitely good results.  It may be that results are not very obvious, but it will be in any case an earnest discussion of subjects of high importance.  Tara, I often wonder how we should approach these subjects.  There are several possible approaches to them.  I hope most of you here are either of the administrator type with actual experience or the professor type.  Both having fund of knowledge are very important.  I do not think the man-in-the-street approach is likely to be well-informed or even helpful.  However, it is obviously an important approach because the administration is ultimately meant to serve such people.  You must remember that aspect otherwise you will have no solid ground under your feet.  The administration not only has to be felt to be good by the people affected.  That should always be so, but it is all the more necessary in fully democratic set-up.  Tara, an administrator who is doing honest work, who knows that he is doing his utmost, often does not receive the recognition that is due to him.  In fact, he meets with severe criticism and feels hurt.  An able administrator will always do the right thing and also make the people feel that he reflects their wishes.  A feeling must come to the people that he is reflecting their wishes.  A feeling must come to the people that he is reflecting their wishes.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, hundred words per minute, passage B. Ready, start. Ladies and gentlemen, para, I am happy to be with you this morning and to associate myself with this pleasant function. On this occasion, I would like to state that every person who is not dealing with a specific subject in an expert way would naturally like to go in for generalizations. I am not an expert in any subject, and so I can say many things about many subjects. Looking at this institute from a distance and going through its publications, it seems to me that it has been making good progress. We have been informed that similar institutes in other countries have begun to appreciate the work of this institute. There can be no doubt about the importance of the work which you are called upon to do. I am glad that from a small annual business session, this gathering of so many distinguished persons will spread out into a conference on a specific subject matter, namely recruitment for the public services. I feel that this is something really solid and worthwhile and would bring definitely good results. It may be that results are not very obvious, but it will be in any case an earnest discussions of subjects of high importance. Para, I often wonder how we should approach these subjects. There are several possible approaches to them. I hope most of you here are either of the administrator type with actual experience or the professor type. Both having fund of knowledge are very important. I do not think the man in the streets approach is likely to be well-informed or even helpful. However, it is obviously an important approach because the administration is ultimately meant to serve such people. You must remember that, aspect, otherwise, you will have no solid ground under your feet. The administration not only has to be felt to be good by the people affected. That should always be so, but it is all the more necessary in fully democratic setup. Para, an administrator who is doing honest work, who knows that he is doing his utmost often does not receive the recognition that is due to him. In fact, he meets with severe criticism and feels hurt. An able administrator will always do the right thing and also make the people feel that he reflects their wishes. A feeling must come to the people that he is reflecting their wishes.</t>
         </is>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute, trial passage.  Ready? Start.  Ladies and gentlemen,  Para, I have great pleasure in welcoming you all to the 12th annual general meeting of the company.  The 12th annual report covers 9 months of commercial operation.  I am sure you must have gone through the accounts for the year under review and I take them as read.  The operation of the plant has now established and a capacity utilization of percent has been achieved in the first 6 months period.  It is expected that the whole year we would be able to achieve a capacity utilization in excess of 9%.  Thank you.  Thank you.  Thank you.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 100 words per minute, trial passage. Ready, start. Ladies and gentlemen, para, I have great pleasure in welcoming you all to the 12th annual general meeting of the company. The 12th annual report covers nine months of commercial operations. I am sure you must have gone through the accounts for the year under review and I take them as red. The operation of the plant has now established and a capacity utilization of percent has been achieved in the first six months period. It is expected that the whole year we would be able to achieve a capacity utilization in excess of 9%.</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1898,7 @@
       <c r="P14" s="2" t="n"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute.  Passage A.  Ready?  Start.  Ladies and gentlemen,  Pyara,  It gives me great pleasure to welcome you to this annual general meeting of your company.  It is with regret that I have to report that the profits of this year have not been as good as last year's, of course.  Last year's were record profits.  The sales have continued to show an upward trend and were better than the last year's mark.  Your directors have recommended to maintain the dividend at 15% on equity share capital.  The performance of any company is naturally conditioned by environment in which it operates.  Last year, Indian industry was overtaken by recession and a number of enterprises suddenly found themselves confronted with fall in demand.  Rising costs and increase in stocks and eventually were forced to cut down production.  Commercial vehicles, automobiles, tire, paper, textile were some of major industries which came directly under the spell of recession.  Major company operations like textiles units in Rajasthan were affected not only recession but also by sever power cuts.  We are not only country which has been attacked by recessionary forces.  As a matter of fact, in last two years, almost all industrialist countries have been facing recession.  We have been saved so far partly because our economy is somewhat covered from such international trends and partly because growth to us is compelling necessity.  There is something wrong somewhere which has disturbed the balance and force the industry to move backward instead of going forward.  I am aware that the present industrial situation cannot be adequately described by a single phenomenon like recession.  There are many other factors in operation which have made the problem little complex.  For instance, there have been excessive imports which can be described as dumping following our liberalized import policy and the recession abroad.  Power storage continues in most of the states.  Our foreign exchange earnings have not increased and the reserves have come down to an alarming low level.  Industrial relations are disturbing and have taken a gigantic form in Mumbai.  We have to view these trends in the perspective of the development set out in the 6-5 year plan.  It was hoped that the average rate of growth of industrial production would be little over 8%.  I was the opinion at that time that even this growth was small in comparison with both our needs as also probabilities.</t>
+          <t>English shorthand, 100 words per minute. Passage A. Ready? Start. Ladies and gentlemen. Piarra, it gives me great pleasure to welcome you to this annual general meeting of your company. It is with regret that I have to report that the profits of this year have not been as good as last years, of course. Last years were record profits. The sales have continued to show an upward trend and were better than the last year's mark. Your directors have recommended to maintain the dividend at 15% on equity share capital. The performance of any company is naturally conditioned by environment in which it operates. Last year, Indian industry was overtaken by recession and number of enterprises suddenly found themselves confronted with fall in demand. Rising costs and increase in stocks and eventually were forced to cut down production. Commercial vehicles, automobile tire paper textile were some of major industries which came directly under the spale of recession. Major company operations like textiles units in Rajasthan were affected not only recession, but also by saver power cuts. We are not only country which has been attacked by recessionary forces. As a matter of fact, in last years, almost all industrialist countries have been facing recession. We have been saved so far, partly because our economy is somewhat covered from such international trends and partly because growth to us is compelling necessity. There is something wrong somewhere which has disturbed the balance and force the industry to move backward instead of going forward. I am aware that the present industrial situation cannot be adequately described by a single phenomenon like recession. There are many other factors in operation which have made the problem little complex. For instance, there have been excessive imports which can be described as dumping following our liberalized import policy and the recession abroad. Power storage continues in most of the states. Our foreign exchange, earnings have not increased and the reserves have come down to an alarming law level. Industrial relations are disturbing and have taken a gigantic form in Mumbai. We have to view these trends in the perspective of the development set out in the six-five-year plan. It was hoped that the average rate of growth of industrial production would be little over 8%. I was the opinion at that time that even this growth was small in comparison with both our needs as also probabilities.</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
@@ -1710,22 +1908,37 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute.  Passage B.  Ready?  Start.  Ladies and gentlemen,  Pyara,  it gives me great pleasure to welcome you to this annual general meeting of your company.  The 31st annual general meeting of your company is for me a very special occasion.  I have been working throughout my life in this company.  The Board of Directors has rightly taken a decision that I should retire as a managing director  from the end of March making way for the younger generation.  The Board has decided that Mr. Joshi be appointed as the chairman  and Mr. Fatih, the managing director, from April onwards.  I will be addressing you for the last time as chairman.  Being a man of sentiment, I cannot help recalling the joy and the toil that I have shared in  steering the affairs of this company for more than four decades.  The 60s was a period when we initiated major diversification in this company  from textiles and sugar to fertilizers and tires.  The 70s was a period when our emphasis shifted towards building a new generation of managers  who could bring both stability and growth to the company.  Achieving such balance between stability and growth, I believe, is the perpetual challenge before top management.  Some have handled it better than others and those who have handled it better have taken their corporations to new heights.  In this respect, I believe that our company on the whole has been eminently successful.  Despite the fact that it has been weighed down by an aging textile industry,  it has succeeded in launching new ventures with growth potential for the future.  Having made these general remarks, I would like to underscore the central theme of my speech,  which I shall call the management of transition.  I would like to take you into my confidence by saying that your present top management  had prepared for this transition well in advance by exposing both of them to various areas of responsibility  within and outside the company.  The result is that they will be taking over as a team of seasoned and experienced business leaders.  I have full faith in them and I am sure you will extend to them the same support and cooperation  as I have been receiving from you during all these years.  At any point of time in the history of enterprise,  there always remains some unfinished business despite the handsprings of hope and confidence.  Para, thanking you, yours faithfully.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 100 words per minute. Passage B. Ready? Start. Ladies and gentlemen, Paira, it gives me great pleasure to welcome you to this annual general meeting of your company. The 31st annual general meeting of your company. The 31st annual general meeting of your company. The 31st annual general meeting of your company is for me a very special occasion. I have been working throughout my life in this company. The Board of Directors has rightly taken a decision that I should retire as a managing director from the end of March Making Way for the younger generation. The board has decided that Mr. Joshi be appointed as the chairman and Mr. Fatil, the managing director from April onwards. I will be addressing you for the last time as chairman. Being a man of sentiment, I cannot help recalling the joy and the toil that I have shared in steering the affairs of this company for more than four decades. The 60s was a period when we initiated major diversification in this company from textiles and sugar to fertilizers and tyres cord. The 70s was a period when our emphasize shifted towards building a new generation of managers who could bring both stability and growth to the company. Achieving such balance between stability and growth, I believe, is the perpetual challenge before top management. Some have handled it better than others, and those who have handled it better have taken their corporations to new heights. In this respect, I believe that our company on the whole has been imminently successful. Despite the fact that it has been weighed down by an aging textile industry, it has succeeded in launching new ventures with growth, potential for the future. Having made the general remarks, I would like to underscore the central theme of my speech, which I shall call the management of transition. I would like to take you into my confidence by saying that your present top management had prepared for this transition well in advance by exposing both of them to various areas of responsibility within and outside the company. The result is that they will be taking over as a team of seasoned and experienced business leaders. I have full faith in them and I am sure you will extend to them the same support and cooperation as I have been receiving from you during all these years. At any point of time in the history of Enterprise, there always remains some unfinished business, despite the handsprings of hope and confidence. Pera, thanking you yours faithfully.</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute. Trial passage. Ready? Start.  Ladies and gentlemen, Vera, I have great pleasure in welcoming you all to the 12th annual general meeting of the company.  The 12th annual report covers 9 months of commercial operation. I am sure you must have gone through the accounts for the year under review, and I take them as read.  The operation of the plant has now established and a capacity utilization of percent has been achieved in the first six months period.  It is expected that of the whole year, we would be able to achieve a capacity utilization in excess of nine percent.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 100 words per minute, trial passage. Ready? Start. Ladies and gentlemen, Paira, I have great pleasure in welcoming you all to the 12th annual general meeting of the company. The 12th annual report covers nine months of commercial operation. I am sure you must have gone through the accounts for the year under review and I take them as read. The operation of the plant has now established and a capacity utilization of percent has been achieved in the first six months period. It is expected that of the whole year we would be able to achieve a capacity utilization in excess of 9%.</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1792,7 +2005,7 @@
       <c r="P15" s="2" t="n"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute. Passage A. Ready? Start.  Gentlemen, Farrah, I have great pleasure to welcome you to this 33th annual general meeting of the company.  The director's report and the accounts have been with you for some time.  Now, and with your permission, I take them as read. I am sure you have read the report and the accounts for the last year and found them interesting and satisfactory.  As I told you, this time last year, the year commenced with a comfortable order book.  The flow of orders during the year was even and adequate.  This was despite the fact that conditions in markets for most of your company's products were extremely competitive.  A notable achievement was that the exports increased to a greater extent and crossed Rs. 1 crore mark for the first time.  Although, as you must have noticed from the accounts, the volume of sales more than its rate of increase, the increase in profits was less than proportionate.  In fact, the increase has been only marginal.  The factors responsible for this lower profitability were mainly competitive, prices, higher cost of inputs, particularly in the case of important projects undertaken by your company,  which involve a large percentage of bought-out materials and last but not least unsettled labor conditions.  One of the side effects of which was go slow tactics resulting in the last few months of the year in lower recovery from your company's plant.  In spite of these adverse factors, I am happy to inform you that your company has performed well and has been able to plug back a good sum to its resources.  I am sure you will appreciate the performance and join me in extending hearty congratulations to our beloved managing director and his excellent team.  The current year commenced with a full order book and position and with plans for a higher sales.  However, the sales during the first five months of this year are only slightly higher than in the corresponding period of the previous year.  The developments on the labor front in the past few months have caused serious concern to your management.  Your company has always believed in harmonious industrial relations and has been taking steps for promoting the interests of the workers.  This will be borne out by the fact that since the inception, the management has excellent and cordial relations with the workers except for a very brief period.</t>
+          <t>English shorthand, hundred words per minute. Passage A. Ready. Start. Gentleman, Farah, I have great pleasure to welcome you to this 33 annual general meeting of the company. The director's report and the accounts have been with you for some time. Now and with your permission, I take them as read. I am sure you have read the report and the accounts for the last year and found them interesting and satisfactory. As I told you, this time, last year, the year commenced with a comfortable order book. The flow of orders during the year was even and adequate. This was despite the fact that conditions in markets for most of your companies' products were extremely competitive. A notable achievement was that the exports increased to a greater extent and crossed rupees one-crower mark for the first time. Although, as you must have noticed from the accounts, the volume of sales more than its rate of increase, the increase in profits was less than proportionate. In fact, the increase has been only marginal. The factors responsible for this lower profitability were mainly competitive prices, higher cost of inputs, particularly in the case of important projects undertaken by your company, which involve a large percentage of bought-out materials and last but not least unsettled labor conditions. One of the side effects of which was go slow. Tactics resulting in the last few months of the year in lower recovery from your company's plant. In spite of these adverse factors, I am happy to inform you that your company has performed well and has been able to plug back a good sum to its resources. I am sure you will appreciate the performance and join me in extending hearty congratulations to our beloved managing director and his excellent team. The current year commenced with a full-order book and position and with plans for a higher sales. However, the sales during the first five months of this year are only slightly higher than in the corresponding period of the previous year. The developments on the labor front in the past few months have caused serious concern to your management. Your company has always believed in harmonious industrial relations and has been taking steps for promoting the interest of the workers. This will be borne out by the fact that since the inception, the management has excellent and cordial relations with the workers, except for a very brief period.</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
@@ -1802,22 +2015,37 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>English shorthand 100 words per minute. Passage B. Ready? Start. Ladies and gentlemen, Tara,  I am happy to be here and speak to you a few words on this important occasion. Let me at  the outset offer my congratulations to the graduates of the year who by hard work and  discipline effort have attained their degrees and some of whom have achieved distinctions also.  Today you have honored some distinguished sons and daughters of the country. They have  rendered dedicated services in their respective fields and as such they have beloved themselves  to one and all. The university has a sense of satisfaction in having honored such eminent  persons whose contribution to the nation is unique. Your university has grown from strength  to strength during the past 40 years. It has been considered as one of the most beautiful  universities of India. It is situated on an evergreen hill. The main building of the university  which is raising its head to the sky is a symbol of man's aspiration for higher and higher knowledge.  The building is surrounded by a very well maintained garden. Many distinguished visitors have admired this  university as an ideal place for academic life and higher education. In this university you have conditions  which make it possible to develop true university life. You do not suffer from blockage. I am glad that you pay  attention to research work. No teacher can inspire his students or win their respect if he is not himself  interested in extending the range of knowledge. The ability to teach pupils, to teach themselves, to inspire  students, to new lines of enquiry are rare gifts. The work and reputation of a university depend on the  presence of such teachers. One of the first objects of the universities all over the world is to produce a class of  men who would devote themselves to research and scholarship on the highest plane. Many of us are apt to think that those  who loom largely in the eyes of the public are the only ones that lead really youthful lives, which sometimes talk and write as  as though only one or two individuals were really doing youthful work and the rest doing nothing. It is, however, a mistake to think so. A nation's true greatness depends upon its average man and woman. It is the life, thoughts and action of the average man and woman  of the average man and woman that the solid strength of a nation really lights.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 100 words per minute. Passage B. Ready Start. Ladies and gentlemen. Tara, I am happy to be here and speak to you a few words on this important occasion. Let me at the outset offer my congratulations to the graduates of the year who, by hard work and discipline, effort have attained their degrees and some of whom have achieved distinctions also. Today, you have honored some distinguished sons and daughters of the country. They have rendered dedicated services in their respective fields, and as such, they have beloved themselves to one and all. The university has a sense of satisfaction in having honored such imminent persons whose contribution to the nation is unique. Your university has grown from strength to strength during the past 40 years. It has been considered as one of the most beautiful universities of India. It is situated on an ever-green hill. The main building of the university, which is raising its head to the sky, is a symbol of man's aspiration for higher and higher knowledge. The building is surrounded by a very well-maintained garden. Many distinguished visitors have admired this university as an ideal place for an academic life and higher education. In this university, you have conditions which make it possible to develop true university life. You do not suffer from blockage. I am glad that you pay attention to research work. No teacher can inspire his students or win their respect if he is not himself interested in extending the range of knowledge. The ability to teach pupils to teach themselves to inspire students to new lines of inquiry are rare gifts. The work and reputation of a university depend on the presence of such teachers. One of the first objects of the universities all over the world is to produce a class of men who would devote themselves to research and scholarship on the highest plane. Many of us are apt to think that those who loom largely in the eyes of the public are the only ones that lead really youthful lives, which sometimes talk and write as though only one or two individuals were really doing useful work and rest doing nothing. It is, however, a mistake to think so. A nation's true greatness depends upon its average man and woman. It is the life, thoughts, and action of the average man and woman that the solid strength of a nation really lies.</t>
         </is>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand 100 words per minute. Trial Passage. Ready? Start. Ladies and gentlemen,  para, I have great pleasure in welcoming you all to the 12th annual general meeting of the company.  The 12th annual report covers nine months of commercial operation. I am sure you must have  gone through the accounts for the year under review and I take them as real. The operation  of the plant has now established and a capacity utilization of percent has been achieved in  the first six months period. It is expected that the whole year we would be able to achieve  a capacity utilization in excess of nine percent.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 100 words per minute. Trial passage. Ready, start. Ladies and gentlemen, para, I have great pleasure in welcoming you all to the 12th annual general meeting of the company. The 12th annual report covers nine months of commercial operation. I am sure you must have gone through the accounts for the year under review and I take them as real. The operation of the plant has now established any capacity utilization of percent has been achieved in the first six months period. It is expected that the whole year we would be able to achieve a capacity utilization in excess of 9%.</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1884,7 +2112,7 @@
       <c r="P16" s="2" t="n"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand 100 Words Per Minute. Passage A. Ready? Start.  Para. I am deeply touched by the kind thoughts and sentiments that you have expressed.  In fact, I feel overwhelmed. You and me are not strangers to each other.  We have met before and you already know how deeply I value and esteem your friendship.  You also know how high you are in the esteem of my people.  We know you as a great and tireless fighter for the freedom of your country, as a symbol of the energies, the hopes and the aspirations of your people.  We have watched with admiration how you have led your people through years of joyful and we hope satisfactory that you will continue to lead them in their steady progress towards the glorious future that is their destiny.  Both of our people have drawn inspiration from our common struggle for freedom.  Representatives of both our countries have in the deliberations of various international organizations, in which our countries participated, lent their support to the demand for freedom and independence of dependent people, particularly in Asia and Africa, who were or still are under foreign domination.  We are living in a dynamic though difficult period.  The advances made in science and technology in our lifetime have been surprising.  Only evolution of our moral and spiritual ideals have not kept pace with these tremendous advances in science and technology.  The world is passing through terrible stress and strains.  Are the advances in science and technology to be harnessed to the economic and social development of the world and removed of hunger, poverty and disease for all men and thus make their contribution to the increase of human happiness and fulfillment?  Or are these advances to be used for destruction of the human race?  These are the questions facing us and the world today.  Both our governments have been doing all they can to secure that those in authority all over the world make the right choice and instead of warming away the great gains of science on destructive purposes, put them to constructive use for the benefit of all men regardless of race.  Basically, our national problems are also similar.  Having gained freedom, our countries are engaged in the more complex and difficult task of giving economic and social content to our freedom.  Without these essential developments which improve the lot of the common man, liberty and freedom have little meaning.  Thanking you once again.</t>
+          <t>English shorthand, 100 words per minute. Passage A. Ready? Start. Pera. I am deeply touched by the kind thoughts and sentiments that you have expressed. In fact, I feel overwhelmed. You and me are not strangers to each other. We have met before, and you already know how deeply I value and esteem your friendship. You also know how high you are in the esteem of my people. We know you as a great and tireless fighter for the freedom of your country, as a symbol of the energies, the hopes, and the aspirations of your people. We have watched with admiration how you have led your people through years of joyful and we hope satisfactory that you will continue to lead them in their steady progress towards the glorious future, that is their destiny. Both of our peoples have drawn inspiration from our common struggle for freedom. Representatives of both our countries have in the deliberations of various international organizations in which our countries participated lent their support to the demand for freedom and independence of dependent people, particularly in Asia and Africa, who were or still are under foreign domination. We are living in a dynamic, though difficult, period. The advances made in science and technology in our lifetime have been surprising. Only evolution of our moral and spiritual ideals have not kept pace with these tremendous advances in science and technology. The world is passing through terrible stress and strengths are the advances in science and technology to be harnessed to the economic and social development of the world and removed of hunger, poverty, and disease for all men and thus make their contribution to the increase of human happiness and fulfillment? Or are these advances to be used for destruction of the human race? These are the questions facing us and the world today. Both our governments have been doing all they can to secure that those in authority all over the world make the right choice and instead of warming away the great gains of science on destructive purposes, put them to constructive use for the benefit of all men regardless of race. Basically, our national problems are also similar. Having gained freedom, our countries are engaged in the more complex and difficult task of giving economic and social content to our freedom. Without these essential developments which improve the lot of the common man, liberty, freedom have little meaning. There are thanking you once again.</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
@@ -1894,22 +2122,37 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute.  Passage B. Ready? Start.  Ladies and gentlemen, para, it is a matter of gratification that this state is forging ahead with schemes  for provision of medical relief, sanitation and other necessary services.  In a wide country like India, with a large population, much of it ill-maintained and with ill-held,  it is more or less inevitable and necessary consequence.  We are therefore trying our best to tackle this question from both ends,  while on one side efforts are being made to improve the living conditions,  to raise the general living standard of our people, which will include also improvement in their health.  On the other side, attempts are being made to provide medical facilities and service on as large a scale  as we can possibly do in our present conditions.  I am therefore happy to learn that in this state, you have made good progress already  and that deficiencies, I have various services are being made good very quickly.  In modern medicine, for detecting testing facilities and also for electric treatment,  various kinds of drugs are an absolute necessity.  It is found by experience that there are several diseases which can be controlled.  They have been controlled in other countries and to the extent we have been able to use old methods and facilities,  we have been able to control them in our country too.  It is therefore essential that each state should have all the necessary equipments  for the purpose of supplying the drugs, the tonics and the boosters which are required for the purpose.  I know that in some states, we have got up to date and very good laboratories which are doing this work  but as they are not sufficient for this country, you are going in for more by expanding the laboratory here  as well as by establishing regional laboratories.  In modern days, everyone who goes to a doctor finds that a doctor by himself is not able to detect his illness.  He needs the help and assistance of a laboratory and each laboratory requires scientific instruments  and other kinds of equipment besides a staff of trained men.  Unless all these are provided, the medical facilities cannot be said to be complete  and how your good, efficient and experienced a doctor may be,  he will very often find himself more or less helpless in the absence of all these facilities.  It is therefore absolutely necessary that these facilities should be provided.  Also, let's talk to you about the counselor</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 100 words per minute. Passage B. Ready Start. Ladies and gentlemen, Paira, it is a matter of gratification that this state is forging ahead with schemes for provision of medical relief, sanitation and other necessary services. In a wide country like India, with a large population, much of it ill-maintained and with ill health it is more or less inevitable and necessary consequence. We are therefore trying our best to tackle this question from both ends, while on one side efforts are being made to improve the living conditions to raise the general living standard of our people, which will include also improvement in their health. On the other side, attempts are being made to provide medical facilities and service on as large a scale as we can possibly do in our present conditions. I am therefore happy to learn that in this state you have made good progress already and that deficiencies I have various services are being made good very quickly. In modern medicine for detecting testing facilities and also for electric treatment, various kinds of drugs are an absolute necessity. It is found by experience that there are several diseases which can be controlled. They have been controlled in other countries and to the extent we have been able to use old methods and facilities. We have been able to control them in our country too. It is therefore essential that each state should have all the necessary equipments for the purpose of supplying the drugs, the tonics, and the boosters, which are required for the purpose. I know that in some states we have got up to date and very good laboratories which are doing this work, but as they are not sufficient for this country, you are going in for more by expanding the laboratory here, as well as by establishing regional laboratories. In modern days, everyone who goes to a doctor finds that a doctor by himself is not able to detect his illness. He needs the health and assistance of a laboratory and each laboratory requires scientific instruments and other kinds of equipment besides a staff of trended men. Unless all these are, provided the medical facilities cannot be said to be complete and how your good efficient and experience a doctor may be, he will very often find himself more or less, helpless in the absence of all these facilities. It is therefore absolutely necessary that these facilities should be provided.</t>
         </is>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 100 words per minute. Trial passage. Ready? Start.  Ladies and gentlemen, Vera, I have great pleasure in welcoming you all to the 12th annual general meeting of the company.  The 12th annual report covers 9 months of commercial operation. I am sure you must have gone through the accounts for the year under review, and I take them as read.  The operation of the plant has now established and a capacity utilization of percent has been achieved in the first six months period.  It is expected that of the whole year, we would be able to achieve a capacity utilization in excess of nine percent.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 100 words per minute, trial passage. Ready? Start. Ladies and gentlemen, Paira, I have great pleasure in welcoming you all to the 12th annual general meeting of the company. The 12th annual report covers nine months of commercial operation. I am sure you must have gone through the accounts for the year under review and I take them as read. The operation of the plant has now established and a capacity utilization of percent has been achieved in the first six months period. It is expected that of the whole year we would be able to achieve a capacity utilization in excess of 9%.</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -1976,7 +2219,7 @@
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand, 120 words per minute. Passage A. Ready? Start.  Ladies and gentlemen, Para, it gives me great pleasure to welcome you all to this ancient city of Pune and particularly to this historic hall.  You will find history staring at you from the front and also from the back. We have retained these pictures on the walls so that we may sometimes feel the change that has taken place.  Sometimes it is necessary to remember the past also. That is why we have retained these pictures in this hall.  Many of you are perhaps visiting Pune for the first time and some of you would have come here on many occasions.  A few amongst you belong to the Pune and it is coming back to their own home for them.  We are particularly grateful to the chairman for having agreed to have the board meeting here.  For some time past, the meetings have been held only at Mumbai. I suppose from now on, the various states will get their chance and the board meetings will be held in all the states.  There are certain advantages in having these meetings outside Mumbai.  It gives one an intimate pictures of things happening in the various states.  The officers and others concerned are greatly benefited by the visit of eminent educationalists from outside the state.  And I am sure the visitors also would be benefited in the same way by having a look at things in the particular state.  It is through this process of mutual consultation that it would be possible for us to make progress.  The occasion we are meeting now is of some significance, particularly in growing and developing country.  We are just now going through the process of the completion of the second five-year plan.  There are only two years more and we have to think of the third five-year plan.  Therefore, it is appropriate that we should take into account the experiences we have gained and the lessons we have learnt in the formulating the working of the second five-year plan.  I am sure these experiences and lessons would guide us properly for the purpose of formulating the third five-year plan.  And more than that, in successfully implementing them, we are all aware that when the second five-year plan was being formulated,  persons particularly interested in the development of education were disappointed.  To the extent as regards the allocation of resources for the educational development.  But I do not think we can blame the planning commission for this.  I say that we ourselves are to be blamed because we did not formulate the plan.  With reference to fiscal targets and what do you mean in terms of finances?  We did not place before the planning commission perhaps the proper picture.  We had the benefit of very valuable reports, one in respect of university education and the other in respect of secondary education.</t>
+          <t>English shorthand, 120 words per minute, passage A. Ready, start. Ladies and gentlemen, para, it gives me great pleasure to welcome you all to this ancient city of Pune and particularly to this historic hall. You will find history staring at you from the front and also from the back. We have retained these pictures on the walls so that we may sometimes feel the change that has taken place. Sometimes it is necessary to remember the past also. That is why we have written these pictures in this hall. Many of you are perhaps visiting Pune for the first time, and some of you would have come here on many occasions. A few amongst you belong to the Pune, and it is coming back to their own home for them. We are particularly grateful to the chairman for having agreed to have the board meeting here. For some time past, the meetings have been held only at Mumbai. I suppose from now on the various states will get their chance and the board meetings will be held in all the states. There are certain advantages in having these meetings outside Mumbai. It gives one and intimate pictures of things happening in the various states. The officers and others concerned are greatly benefited by the visit of eminent educationalists from outside the state, and I'm sure the visitors also would be benefited in the same way by having a look at things in the particular state. It is through this process of mutual consultation that it would be possible for us to make progress. The occasion we are meeting now is of some significance, particularly in growing and developing country. We are just now going through the process of the completion of the second five-year plan. There are only two years more, and we have to think of the third five-year plan. There are only two years more and we have to think of the third five year plan. Therefore, it is appropriate that we should take into account the experiences we have gained and the lessons we have learned in the formulating, the working ofthe second five-year plan. I am sure these experiences and lessons would guide us properly for the purpose of formulating the third five-year plan and more than that in successfully implementing them. We are all aware that when the second five-year plan was being formulated, persons particularly interested in the development of education were disappointed. To the extent as regards the allocation of resources for the educational development. But I do not think we can blame the Planning Commission for this. I say that we ourselves are to be blamed because we did not formulate the plan with reference to fiscal targets and what do you mean in terms of finances? We did not place before the Planning Commission perhaps the proper picture. We had the benefit of very valuable reports, one in respect of university education and the other in respect of secondary education.</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -1986,22 +2229,37 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>English Shorthand, 120 words per minute, Passage B.  Ready? Start!  Mr. Speaker, a large number of Honorable Members have participated in this debate and have made useful suggestions.  Since I was interested with the responsibility of this ministry in the first trade conference,  I made it clear that the food problem has to be tackled as a national problem.  It should not be treated as a party question and no attempt should be made to take advantage for party purposes of a serious situation in one part of the country or the other.  It should be the joint effort of the central government and the state governments to meet the serious situation that is facing the country.  Unless we make a joint endeavor in this matter, I fear that the problem will continue to challenge us.  Therefore, joint effort is necessary.  The joint effort should be not only by the governments but also by the people in every state  because the problem is such that the entire country will have to be mobilized to face this situation.  Sir, the suggestions that have been made divide the entire issue into four broad aspects.  The four important aspects on which emphasis has been laid for the various sides of the house are the aspects of procurement, distribution, production and price.  In other words, procurement will help us to some extent.  Some of the state governments have their own systems of procurement and in some states the procurement policies have been quite successful.  By and large, it will have to be left to the state governments as to what system they will follow for the successful procurement of the surplus food grains in their respective states.  In some states it may be the levy system while in some others it may be directly from the cultivators or from the millers.  It will all depend upon the circumstances existing in each state.  So, it will be difficult to have a uniform policy so far as procurement is concerned.  But, it will have to be an effort of the state governments to have some system of procurement so that whatever surplus is available in the surplus state is made available to the deficit states.  The system of distribution also differs in various states.  At certain places we have rationing and in many rural areas in the deficit states we have fair price shops.  It will require a bold person to say that in any of these systems of distribution there is no scope for leakages.  So, it should be the endeavor of those who are in charge of all these distribution systems to see that in view of the scarcity we are faced with all channels of leakages are efficiently plugged.  So, if there is any leakage, the people for whom the food grains are mint would not get the food grains.  Instead, the food grains would go to a class of people who have a better purchasing capacity.  Para, thanking you, yours faithfully.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 120 words per minute, passage B. Ready, start. Mr. Speaker, a large number of honourable members have participated in this debate and have made useful suggestions. Since I was interested with the responsibility of this ministry in the first trade conference, I made it clear that the food problem has to be tackled as a national problem. It should not be treated as a party question and no attempt should be made to take advantage for party purposes of a serious situation in one part of the country or the other. It should be the joint effort of the central government and the state governments to meet the serious situation that is facing the country. Unless we make a joint endeavor in this matter, I fear that the problem will continue to challenge us. Therefore, joint efforts is necessary. The joint effort should be not only by the governments, but also by the people in every state, because the problem is such that the entire country will have to be mobilized to face this situation. Sir, the suggestions that have been made divide the entire issue into four broad aspects. The four important aspects on which emphasis has been laid for the various sides of the house are the aspects of procurement, distribution, production, and price. Procurement will help us to some extent. Some of the state governments have their own systems of procurement, and in some states, the procurement policies have been quite successful. By and large, it will have to be left to the state governments as to what system they will follow for the successful procurement of the surplus food grains in their respective states. In some states, it may be the levy system, while in some others it may be directly from the cultivators or from the millers. It will all depend upon the circumstances existing in each state. So it will be difficult to have a uniform policy so far as procurement is concerned. But it will have to be an effort of the state governments to have some system of procurement so that whatever surplus is available in the surplus state is made available to the deficit states. The system of distribution also differs in various states. At certain places, we have rationing and in many rural areas in the deficit states we have fair price shops. It will require a bold person to say that in any of these systems of distribution there is no scope for leakages. So it should be the endeavor of those who are in charge of all these distribution systems. To see that, in view of the scarcity, we are faced with all channels of leakages are efficiently plugged. If there is any leakage, the people for whom the food grains are mint would not get the food grains. Instead, the food grains would go to a class of people who have a better purchasing capacity. Param, thanking you, yours, faithfully.</t>
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 120 words per minute, trial passage.  Ready? Start.  Communicating with a person who is in front of you is face-to-face communication  and this is mostly oral in nature.  Communicating with a person who is away from you is communicating over a distance  and is called distance communication.  It may be either oral or written in nature.  In this unit, you are going to look at distance communication  and some of the ways in which it is managed.  Para.  One of the most common modes of distance communication is male.  It is also one of the earliest systems of such communication.  In its simplest form, mail means a letter which sent by post.  Mail is cheapest form of communication.  A new development in this field of communication is speed post.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 120 words per minute, trial passage. Ready, start. Communicating with a person who is in front of your is face-to-face communication, and this is mostly oral in nature. Communicating with a person who is away from you is communicating over a distance and is called distance communication. It may be either oral or written in nature. In this unit, you are going to look at distance communication and some of the ways in which it is managed. Param, one of the most common modes of distance communication is male. It is also one of the earliest systems of such communication. In its simplest form, mail means a letter which sent by post. Mail is cheapest form of communication. A new development in this field of communication is speed post.</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2326,7 @@
       <c r="P18" s="2" t="n"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 120 words per minute. Passage A. Ready? Start. Sir, para, at the outset,  I would like to express my gratitude to the honorable members on both sides of the house  for participating in the discussion and making very valuable suggestions. They have expressed  their views in their own way. But at the same time, they have touched on some of the issues  which are very important from the point of view of the national economy. I would not say that the  views that they have expressed are due to any political consideration. But they were  really expressed in the national interest. In this connection, I was happy that there was  at least one honorable member who said that we should face the question of economy from  a national point of view. Last year, if we go through the budget speech, we will find that  the basic aims are national growth and social justice. This is the thrust of the budget that  we have prepared and it may be seen whether it is reflected in the budget provisions or not.  I am sure that if the honorable members go through the budget, they will find that there are a number of  new ideas which have been incorporated in the present budget as this is the last year of the current  five-year plan. I have no doubt that the honorable members will be trying to find whether we have been able to  achieve the plan targets for this purpose. I would like to draw the attention of the house to the fact that we have been able to exceed the financial provisions.  So, no ministry can say that sufficient funds were not available and that is the reason why it is not able to achieve the target set for itself.  But at the same time, I agree that merely spending money is not adequate.  On the other hand, there should be adequate return in physical terms.  That is why we have been making provisions every year with a view to seeing that the various sectors are able to achieve the targets that they have set for themselves.  If the honorable members go through the documents which have been presented to the house, they will find that there are two or three things which are very important.  The first is the rate of growth. I do not understand why the leader of the opposition was very angry about the rate of growth because of the fact that somehow or other, this time on account of the favorable monsoon, we were able to achieve almost million tons of food grains production.  There is still one more year left and if we have normal monsoon, I am sure we will be able to achieve more next year.  There's still one more year.  Let's listen to HN</t>
+          <t>English shorthand 120 words per minute. Passage A. Ready. Start. Sir, para. At the outset, I would like to express my gratitude to the honorable members on both sides of the House for participating in the discussion and making very valuable suggestions. They have expressed their views in their own way, but at the same time they have touched on some of the issues which are very important from the point of view of the national economy. I would not say that the views that they have expressed are due to any political consideration, but they were really expressed in the national interest. In this connection, I was happy that there was at least one honorable member who said that we should face the question of economy from a national point of view. Last year, if we go through the budget speech, we will find that the basic aims are national growth and social justice. This is the thirst of the budget that we have prepared and it may be seen whether it is reflected in the budget provisions or not. I am sure that if the honorable members go through the budget, they will find that there are a number of new ideas which have been incorporated in the present budget, as this is the last year of the current five-year plan. I have no doubt that the Honorable Members will be trying to find whether we have been able to achieve the plan targets for this purpose. I would like to draw the attention of the House to the fact that we have been able to exceed the financial provisions. It is for the first time that we are going to achievement of the target. This is in regard to the financial provisions. So no ministry can say that sufficient funds were not available and that is the reason why it is not able to achieve the target set for itself. But at the same time, I agree that merely spending money is not adequate. On the other hand, there should be adequate return in physical terms. That is why we have been making provisions every year with a view to seeing that the various sectors are able to achieve the targets that they have set for themselves. If the honorable members go through the documents which have been presented to the house, they will find that there are two or three things which are very important, the first is the rate of growth. I do not understand why the leader of the opposition was very angry about the rate of growth because of the fact that somehow or other this time on account of the favorable monsoon. We were able to achieve almost million tons of food grains production. There is still one more year left and if we have normal monsoon, I'm sure we will be able to achieve more next year.</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
@@ -2078,22 +2336,37 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 120 words per minute. Passage B. Ready? Start.  Mr. Chairman, Para, I am glad to participate in the discussion on the railway budget.  At the outset, I must say that I have every praise for the railwaymen who are doing their best to improve the efficiency of the Indian railways.  It is only because of their clear efforts that we are having a surplus budget.  But I am sorry that the second class fare has been increased in this year's budget.  We were expecting that at least in this budget, our new minister would not increase the second class fare.  I would request him to reconsider the decision and see whether the second class passengers can be exempted for this levy.  Coming to the various aspects of the railways, I must say that the work regarding electrification of the railways has been done very effectively.  But at the same time, the employees who are doing this work have submitted a memorandum to the railway administration.  I would request that something should be done in their case to redress their genuine complaints.  I would request the railway minister to hold a meeting with the representatives of the All India Railway Men's Federation and also with the representatives of railway electrification workers to decide this issue by talking across the table.  Now, I would like to draw the attention of the Honourable Minister to another important point, namely the appointment of a wage board.  This demand has been supported by the National Federation of Railway Men's Federation and also I happen to the President of Southeastern Railway Men's Union, which is affiliated to the All India Railway Men's Federation.  We requested the appointment of a wage board with full powers because all the complaints of the railway men cannot be bitted out by sitting across the table or sitting around the table.  The time has come when the recommendations of the pay commission have no relation with the rising cost of living today because it was thought by the pay commission that prices would stabilize somewhere.  But unfortunately, it has not been possible to hold the price line.  I know the railway ministry will say that the appointed committee and its recommendations have also been implemented, though in certain cases the committee's report was accepted in two by the railway board with slight modifications.  It has not been implemented in certain places.  I would request the Honourable Minister to see that recommendations of the committee are implemented fully.  Then appointment of wage board has become question of life and death for railway employees throughout the country.  I am sure railway minister will see that wage board is appointed.  The railway employees do not want an immediate increase but they want an objective analysis of their jobs where the correct man is doing the correct job.  I request that wage board may be appointed soon and the government should not have any hesitation in appointing wage board.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand 120 words per minute. Passage B. Ready Start. Mr. Chairman, Para, I am glad to participate in the discussion on the railway budget. At the outset, I must say that I have every phrase for the railway men who are doing their best to improve the efficiency of the Indian railways. It is only because of their clear efforts that we are having a surplus budget. But I am sorry that the second class fare has been increased in this year's budget. We were expecting that at least in this budget our new minister would not increase the second class fare. I would request him to reconsider the decision and see whether the second class passengers can be exempted for this levy. Coming to the various aspects of the railways, I must say that the work regarding electrification of the railways has been done very effectively, but at the same time, the employees who are doing this work have submitted a memorandum to the railway administration. I would request that something should be done in their case to redress their genuine complaints. I would request the railway minister to hold a meeting with the representatives of the All India Railway Mainz Federation and also with the representative of railway electrification workers to decide this issue by talking across the table. Now I would like to draw the attention of the Honorable Minister to another important point, namely the appointment of a wage board. This demand has been supported by the National Federation of Railwaymen also. I happen to the President of South Eastern Railwaymen's Union which is affiliated to the All India Railwaymen's Federation. We requested the appointment of a wage board with full powers because all the complaints of the railwaymen cannot be beated out by sitting across the table or sitting around the table. The time has come when the recommendations of the Pay Commission have no relation with the rising cost of living today because it was thought by the pay commission that prices would stabilize somewhere but unfortunately it has not been possible to hold the price line. I know the railway ministry will say that they appointed committee and its recommendations have also been implemented, though in certain cases the committee's report was accepted in two by the railway board with slight modifications. It has not been implemented in certain places. I would request the Honorable Minister to see that recommendations of the committee are implemented fully. Then appointment of wage board has become question of life and depth for railway employees throughout the country. I'm sure railway minister will see that wage board is appointed. The railway employees do not want an immediate increase, but they want an objective analysis of their jobs, where the correct man is doing the correct job. I request that wage board may be appointed soon and the government should not have any hesitation in appointing wage board.</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
         <is>
-          <t>English shorthand. 120 words per minute. Trial passage. Ready? Start. Para. Communicating  with a person who is in front of your face to face. Communication and this is mostly oral  in nature. Communicating with a person who is away from you is communicating over a distance  and is called distance communication. It may be either oral or written in nature. In this unit,  you are going to look at distance communication and some of the ways in which it is managed. Para.  One of the most common modes of distance communication is mail. It is also one of the  earliest systems of such communication. In its simplest form, mail means a letter which  sent by post. Mail is the cheapest form of communication. A new development in this field  of communication is speed post.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 120 words per minute, trial passage, ready, start, para, communicating with a person who is in front of your, is face to face, communication and this is mostly oral in nature. Communicating with a person who is away from you is communicating over a distance and is called distance communication. It may be either oral or written in nature. In this unit you are going to look at distance, communication and some of the ways in which it is managed. Para. One of the most common modes of distance communication is male. It is also one of the earliest systems of such communication. In its simplest form, male means a letter which sent by post, male is cheapest form of communication. A new development in this field of communication is speedpost.</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2433,7 @@
       <c r="P19" s="2" t="n"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 120 words per minute. Passage A. Ready? Start.  Mr. Speaker, Para, I have been in charge of finance for the last two years. Now, I may assure the members of the House  that we have been able to manage the financial affairs of this state successfully during a very  critical period. If honorable members would go through the budget proposals for the previous  two years, I am sure they will agree with me that we have got over a very difficult period,  even if it was necessary to get assistance from the central government also.  Honorable members have said that we have not been able to meet their demands in respect of  their nations and also some other general demands. As I have already stated on another occasion,  the things that we have got to achieve are so many and so great that it will not be possible  to meet all these demands within a short period of time because those needs have been accumulating  for many years. But I should like to add that they can be achieved within a few years. That is why  we have now formulated a plan with reference to the resources available and the achievements which  we can make with reference to these resources. So, if the honorable gentleman has made a charge on the floor  of the House that in spite of the fact that for the last two years, honorable members have been making demands  in respect of their nations. They have not been met properly. I plead guilty to that charge. It would have meant spending further crores of rupees. If we had got another rupees two crores from center, perhaps we would have been able to meet a major portion of the demands made on the floor of the house.  We have been able to get on all these years. I may assure the honorable members that we have got over the crisis. And I think I will not be wrong if I say that we are entering a period of uniformity.  I hope and pray that in this year we will have a normal year and our expectations will be fulfilled. I am sure that in the next year, whoever is called upon to present the budget, he will have more comfortable time.  I am sure the present sacrifices will have the way for the future generations. That is my hope. And with this satisfaction, I may tell this house that I have carried on as finance minister to the best of my ability.  My only prayer is that hereafter droughts and floods may not occur. We cannot prevent these things occurring even if they occur. They may not occur on the same scale.  And I am sure that our people will be able to face all these difficulties. While we are prepared for the worst, I am hoping for the best. Thank you once again. Yours faithfully.  Thank you.</t>
+          <t>English shorthand 120 words per minute. Passage A. Ready? Start. Mr. Speaker, Para. I have been in charge of finance for the last two years. Now, I may assure the members of the house that we have been able to manage the financial affairs of this state successfully during a very critical period. If honourable members would go through the budget proposals for the previous two years, I am sure. They will agree with me that we have got over a very difficult period, even if it was necessary to get assistance from the central government also. Honorable members have said that we have not been able to meet their demands in respect of their nations and also some other general demands, as I have already stated on another occasion. The things that we have got to achieve are so many and so great that it will not be possible to meet all these demands within a short period of time because those needs have been accumulating for many years. But I should like to add that they can be achieved within a few years. That is why we have now formulated a plan with reference to the resources available and the achievements which we can make with reference to these resources. So if the Honorable Gentleman has made a charge on the floor of the house, that in spite of the fact that for the last two years, Honorable Members have been making demands in respect of their nations, they have not been met properly. I plead guilty to that charge. It would have meant spending further croars of rupees. If we had got another rupees to cross from center, perhaps we would have been able to meet a major portion of the demands made on the floor of the house. We have been able to get on all these years. I may assure the Honorable Members that we have got over the crisis, and I think I will not be wrong if I say that we are entering a period of uniformity. I hope and pray that in this year we will have a normal year and our expectations will be fulfilled. I'm sure that in the next year whoever is called upon to present the budget, he will have more comfortable time. I am sure the present sacrifices will have the way for the future generations. That is my hope, and with this satisfaction, I may tell this house that I have carried on as finance minister to the best of my ability. My only prayer is that hereafter draughts and flurts may not occur. We cannot prevent these things occurring even if they occur. They may not occur on the same scale and I'm sure that our people will be able to face all these difficulties while we are prepared for the worst I'm hoping for the best. Thanking you once again, you respectfully.</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
@@ -2170,22 +2443,37 @@
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 120 words per minute. Passage B. Ready? Start. Mr. Speaker, Sir,  Para, at the outset, I thank the Honorable Members for the constructive suggestions they have made  in the course of the debate. I shall now reply to some of the points raised by them. First of all,  with reference to the small surplus on the revenue side, the leader of the opposition said that I had  done this by decreasing the expenditure. I do not know whether there is any other method of balancing  a budget. So far as I know, we can do it only by adjusting the expenditure to the income and this  is the only way in which we can do it. But I have to point out that we have still to meet our capital  expenditure and for this purpose, we require the assistance of the center. As far as revenue  expenditure is concerned, we cannot go on having deficits year after year. As Honorable Members  are aware, for the last three years, we are having deficits and it is necessary to balance our budget.  In this connection, I am glad to say that the Finance Commission has gone into the question of the  revenue expenditure on account of the development expenditure of the states. So, it has made some revenue  resources available to the states. There was money which was available to the center. Now, it has been  allocated to the states by the Finance Commission. To that extent, I will be able to cut the assistance  which we have to give under the plan. If this is done, we will gain to some extent by the recommendations  of the Finance Commission. Then, I come to the taxation measures which I have proposed in my budget speech.  It is really unfortunate that even those who are not members of the House say that the court fee  should not have been increased. As far as this criticism is concerned, I am sorry that a wrong view has been  taken of the proposal. I am sure the members who are lawyers will realize the anomalies which exist in the  Present Court Fees Act. We want to remove these exceptions and in that way, we will also be able to get some money.  It is not as if we want to make the poor people suffer on account of this. Then, with regard to the  Tobacco Tax, it has been said that we are taxing luxury of poor men and that it should not be taxed. Now, I was really  surprised to see speech made by a person connected with commerce to the effect that government which had been  adopting the policy of prohibition should not levy tax on tobacco. It seems to me that he thinks the excites revenue  we will be getting by selling toddy comes from people who are not poor. I am not able to appreciate the stand taken by him.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 120 words per minute, passage B. Ready, start. Mr. Speaker, Sir, Para, at the outset, I thank the Honourable Members for the constructive suggestions they have made in the course of the debate. I shall now reply to some of the points raised by them. First of all, with reference to the small surplus on the revenue side. The leader of the opposition said that I had done this by decreasing the expenditure. I do not know whether there is any other method of balancing a budget. So far as I know we can do it only by adjusting the expenditure to the income and this is the only way in which we can do it. But I have to point out that we have still to meet our capital expenditure and for this purpose we require the assistance of the center. As far as revenue expenditure is concerned, we cannot go on having deficits year after year. As honourable members are aware for the last three years, we are having deficits and it is necessary to balance our budget. In this connection, I am glad to say that the Finance Commission has gone into the question of the revenue expenditure on account of the developmental expenditure of the states, so it has made some revenue resources available to the states. There was money which was available to the center. Now, it has been allocated to the states by the Finance Commission. To that extent, I will be able to cut the assistance which we have to give under the plan. If this is done, we will gain to some extent by the recommendations of the Finance Commission. Then I come to the taxation measures which I have proposed in my budget speech. It is really unfortunate that even those who are not members of the house say that the court fee should not have been increased. As far as this criticism is concerned, I am sorry that a wrong view has been taken of the proposal. I am sure the members who are lawyers will realize the anomalies which exist in the present Court Fees Act. We want to remove these exceptions and in that way we will also be able to get some money. It is not as if we want to make the poor people suffer on account of this. Then with regard to the tobacco tax, it has been said that we are taxing luxury of poor man and that it should not be taxed. Now, I was really surprised to see speech made by a person connected with commerce to the effect that government, which had been adopting the policy of prohibition should not levy tax on tobacco. It seems to me that he thinks the excites revenue we will be getting by selling toddy comes from people who are not poor. I am not able to appreciate the stand taken by him.</t>
         </is>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>English shorthand. 120 words per minute. Trial passage. Ready? Start. Para. Communicating  with a person who is in front of your face to face. Communication and this is mostly oral  in nature. Communicating with a person who is away from you is communicating over a distance  and is called distance communication. It may be either oral or written in nature. In this unit,  you are going to look at distance communication and some of the ways in which it is managed. Para.  One of the most common modes of distance communication is mail. It is also one of the  earliest systems of such communication. In its simplest form, mail means a letter which  sent by post. Mail is the cheapest form of communication. A new development in this field  of communication is speed post.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 120 words per minute, trial passage, ready, start, para, communicating with a person who is in front of your, is face to face, communication and this is mostly oral in nature. Communicating with a person who is away from you is communicating over a distance and is called distance communication. It may be either oral or written in nature. In this unit you are going to look at distance, communication and some of the ways in which it is managed. Para. One of the most common modes of distance communication is male. It is also one of the earliest systems of such communication. In its simplest form, male means a letter which sent by post, male is cheapest form of communication. A new development in this field of communication is speedpost.</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2540,7 @@
       <c r="P20" s="2" t="n"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 120 words per minute. Passage A. Ready, start. Sir, para, I thank you for giving  me an opportunity to say a few words on this occasion. I did not want to intervene in this  debate, but there seems to be a serious discussion on the issue of sales tax. I did not expect this  in the debate on this demand for grants. I thought that we could deal with it in the budget debate  for the whole year to be discussed in a short time. But the remarks that have been made compelled me  to say a few words. In this occasion, we may discuss this problem of sales tax not from the point of  view of party politics, but from the point of view of the welfare of the state and the requirements  of the government to carry on their functions. There is no doubt that this tax forms the most  important part of the state revenues in these days. So, I would like to say that we may take  into consideration this question and discuss the issues involved. One of the most important things  that we should consider with reference to this matter is this. The question is whether we should  tax only those who drink and get a large amount of revenue to carry on our functions or whether we should  tax all the people and get the same amount by indirect taxation. It seems to me that it is better to  to levy a tax upon all the people than to levy a tax upon an unfortunate section of the people only. There is no  reason why it should not be done when we know that the source of revenue is bad and that the victims are only an  an unfortunate section of the people. It seems to me clear that we should find a way out. I am sure that one  indirect tax on all the people will be the right thing so far as this matter is concerned. At the same time, I do not  say that it is a good thing to all people. I do not say that foodstuffs should be taxed. But in this  connection, one point that must be borne in mind is this. When we want some revenue and when we have to decide whether  whether we should tax a few unfortunate people who are poor or whether we should tax everybody, we have to take into  the incidence of the incidence of the tax so that it may fall on everybody. It is right on the part of the  honorable members to say that foodstuffs should not be taxed. It may seem to be alright, but we are aware of the  of the poverty of our people. The consumption is mostly of essentials. The trade is mostly in essential articles. So, we  cannot get a large amount of revenue by taxing everybody unless we take into account what everybody consumes.  the vaccines.</t>
+          <t>English shorthand, 120 words per minute. Passage A. Ready. Start. Sir, Para. I thank you for giving me an opportunity to say a few words on this occasion. I did not want to intervene in this debate, but there seems to be a serious discussion on the issue of sales tax. I did not expect this in the debate on this demand for grants. I thought that we could deal with it in the budget debate for the whole year to be discussed in a short time. But the remarks that have been made compelled me to say a few words. In this occasion, we may discuss this problem of sales tax, not from the point of view of party politics, but from the point of view of the welfare of the state and the requirements of the government to carry on their functions. There is no doubt that this tax forms the most important part of the state revenues in these dates. So I would like to say that we may take into consideration this question and discuss the issues involved. One of the most important things that we should consider with reference to this matter is this. The question is whether we should tax only those who drink and get a large amount of revenue to carry on our functions or whether we should tax all the people and get the same amount by indirect taxation. It seems to me that it is better to levy a tax upon all the people than to levy a tax upon an unfortunate section of the people only. There is no reason why it should not be done. When we know that the source of revenue is bad and that the victims are only an unfortunate section of the people, it seems to me clear that we should find a way out. I'm sure that one indirect acts on all the people will be the right thing so far as this matter is concerned. At the same time, I do not say that it is a good thing to all people. I do not say that foodstuffs should be taxed. But in this connection, one point that must be borne in mind is this. When we want some revenue and when we have to decide whether we should tax a few unfortunate people who are poor or whether we should tax everybody. We have to take into account the incidence of the tax so that it may fall on everybody. It is right on the part of the honorable members to say that food stops should not be taxed. It may seem to be all right, but we are aware of the poverty of our people. The consumption is mostly of essentials. The trade is mostly in essential articles. So we cannot get a large amount of revenue by taxing everybody unless we take into account what everybody consumes.</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
@@ -2262,22 +2550,37 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>English shorthand 120 words per minute. Passage B. Ready? Start. Mr. Chairman, Para, I intervene in this debate for a few minutes in order that I may explain the position with reference to certain questions dealt with by Honorable Members.  I would like to deal with the question relating to food prices. There is no doubt that the position of high prices of food grains is really a matter for worry for all of us. As a matter of fact, the prices have been rising and there has been fluctuation in the prices of food grains for some time.  As has been pointed out by an Honorable Member, perhaps this food problem is a result of the war.  Ever since the last war, we have been facing the question of high prices and sometimes scarcity of food.  In this connection, I would like to point out that before the war, we had reserve stocks which were built up year after year.  But on the other hand, during the war, production was affected by the failure of the monsoons and there was scarcity.  So, all the reserve stocks were consumed year after year.  Then, after the war, there were no reserve stocks and there was less production.  Not only that, but our requirements of food also were going up year after year.  Of course, we have taken some steps to increase the production of rice and millets.  One thing should be noted here.  People have been taking more and more of rice now.  Those who were eating millets have taken to rice.  We are trying to cope with the demand and production has been going up.  I am glad that we have been lucky in having good monsoons.  In addition to that, I am happy that the cultivators have come forward to adopt improved methods of cultivation and have increased production.  Of course, I am aware that we have to step up production still further.  We have to meet not only the needs of the increased population, but also we should be able to meet situation where there is a failure of the monsoon.  So, we are taking all steps to see that production is further increased to a great extent.  It is also the only way in which we can improve the economic condition of the agriculturist in this state.  Of course, I may claim that we have been producing as much as is necessary to meet the food requirements of the state.  In spite of that, the prices have been going up from time to time.  That is the problem that we have to face so far as the question of food prices is concerned.  It is not merely question of supply and demand.  I wish to point out that there is adequate rice.  I have been inquiring district after district and there is no complaint of scarcity of food grains anywhere, but at the same time, the prices have been rising.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 120 words per minute. Passage B. Ready. Start. Mr. Chairman. Para, I intervene in this debate for a few minutes in order that I may explain the position with reference to certain questions dealt with by honorable members. I would like to deal with the question relating to food prices. There is no doubt that the position of high prices of food grains is really a matter for worry for all of us. As a matter of fact, the prices have been rising and there has been fluctuation in the prices of food grains for some time. As has been pointed out by an honorable member, perhaps this food problem is a result of the war. Ever since the last war, we have been facing the question of high prices and sometimes scarcity of food. In this connection, I would like to point out that before the war, we had reserve stocks which were built up year after year. But on the other hand, during the war, production was affected by the failure of the monsoons and there was scarcity. So all the reserve stocks were consumed year after year. Then after the war, there were no reserve stocks and there was less production. Not only that, but our requirements of food also were going up year after year. Of course, we have taken some steps to increase the production of rice and millets. One thing should be noted here. People have been taking more and more of rice now. Those who were eating millets have taken to rice. We are trying to cope with the demand and production has been going up. I am glad that we have been lucky in having good monsoons. In addition to that, I am happy that the cultivator have come forward to adopt improved methods of cultivation and have increased production. Of course, I am aware that we have to step up production still further. We have to meet not only the needs of the increased population, but also we should be able to meet situation where there is a failure of the monsoon. So we are taking all steps to see that production is further increased to a great extent. It is also the only way in which we can improve the economic condition of the agriculturalist in this state. Of course, I may claim that we have been producing as much as is necessary to meet the food requirements of the state. In spite of that, the prices have been going up from time to time. That is the problem that we have to face so far as the question of food prices is concerned. It is not merely question of supply and demand. I wish to point out that there is adequate rice. I have been inquiring, district after district, and there is no complaint of scarcity of food grains anywhere but at the same time the prices have been rising.</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>English shorthand. 120 words per minute. Trial passage. Ready? Start. Para. Communicating  with a person who is in front of your face to face. Communication and this is mostly oral  in nature. Communicating with a person who is away from you is communicating over a distance  and is called distance communication. It may be either oral or written in nature. In this unit,  you are going to look at distance communication and some of the ways in which it is managed. Para.  One of the most common modes of distance communication is mail. It is also one of the  earliest systems of such communication. In its simplest form, mail means a letter which  sent by post. Mail is the cheapest form of communication. A new development in this field  of communication is speed post.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 120 words per minute, trial passage, ready, start, para, communicating with a person who is in front of your, is face to face, communication and this is mostly oral in nature. Communicating with a person who is away from you is communicating over a distance and is called distance communication. It may be either oral or written in nature. In this unit you are going to look at distance, communication and some of the ways in which it is managed. Para. One of the most common modes of distance communication is male. It is also one of the earliest systems of such communication. In its simplest form, male means a letter which sent by post, male is cheapest form of communication. A new development in this field of communication is speedpost.</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2647,7 @@
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 130 words per minute, passage A. Ready? Start.  In Companies Act provides that every company shall cause minutes of all proceedings of general meetings, all proceedings at meetings of its directors and where there are managers, all proceedings at meetings of its managers to be entered in books kept for that purpose.  Any such minute, if purporting to be signed by the chairman of the meeting at which the proceedings were held or by the chairman of the next succeeding meeting, shall be evidence of the proceedings.  Where minutes have been made in accordance with the provision of the section, then until the contrary is proved, the meeting shall be deemed to have been duly held and convened and all the proceedings threat to have been duly held and all appointments of directors, managers or liquidators shall be deemed to be valid.  Failure to prepare minutes as required by the section renders, the company and every officer of the company in default liable to a default fine.  As will be noticed, the minutes of a meeting are not required to be read at a subsequent meeting of the board of directors or of the shareholders.  In the case of a general meeting and they require no approval from the directors or the shareholders before they are signed by the chairman.  It is customary, however, for minutes of a board meeting to be read by the secretary at the next board meeting of the company or for the minutes to be copied and circulated to the directors for their approval before the next meeting, in which case there is no necessity to have then read.  But if the chairman considered fit, we could decide that the minutes of a meeting drafted by the secretary should be submitted only to him for approval and signature and that his colleagues should not be acquainted with the actual wording of the decisions arrived at before the minutes were written up.  He could not, however, he could not, however, he could not, however, prevent his colleagues from inspecting the minute book of the company, provided they were doing so in the interest of the company as a whole and not in their individual interest.  Para, it is to avoid any possibility of subsequent legal action that the practice of reading the minutes of obtaining the approval of the body thereto has sprung up.  The word confirmation used in that connection is not correct.  As minutes require no confirmation, the decisions having once been made stand without further confirmation.  If the necessity for altering minutes arises before they are signed by the chairman but subsequent to the writing up in the minute book,  the alterations may be inserted and initialed by the chairman when he signs but when once minutes have been signed by should not under any circumstance be altered.  If it becomes necessary to vary a resolution previously adopted, that variation should always be carried out by means of a minute passed at subsequent meeting.  Para, some companies keep their minutes on the loose leaf principle and if proper safeguards are provided, there is nothing against this practice.  Now, the modern loose leaf minute book is provided with the locking device.  Then as long as it is located, it is not short for the timely reason.  Thank you.  And finally buy the new leafนะ.</t>
+          <t>English shorthand, 130 words per minute, passage A. Ready, start. In Companies Act provides that every company shall cause minutes of all proceedings of general meetings, all proceedings at meetings of its directors and where there are managers, all proceedings at meetings of its managers, all proceedings at meetings of its managers, to be entered in books kept for that purpose. Any such minute is purporting to be signed by the chairman of the meeting at which the proceedings were held or by the chairman of the next succeeding meeting shall be evidence of the proceedings, where minutes have been made in accordance with the provision of the section, then until the contrary is proved, the meeting shall be deemed to have been duly held and convened and all the proceedings threat to have been duly held and all appointments of directors, managers or liquidators shall be deemed to be valid. Failure to prepare minutes as required by the section renders the company and every officer of the company in default liable to a default fine. As will be noticed, the minutes of a meeting are not required to be read at a subsequent meeting of the board of directors or of the shareholders in the case of a general meeting and they require no approval from the directors or the shareholders before they are signed by the chairman. It is customary, however, for minutes of a board meeting to be read by the secretary at the next board meeting of the company or for the minutes to be copied and circulated to the directors for their approval before the next meeting, in which case there is no necessity to have then read. But if the chairman considered fit, we could decide that the minutes of a meeting drafted by the secretary should be submitted only to him for approval and signature, and that his colleagues should not be acquainted with the actual wording of the decisions arrived at before the minutes were written up. He could not however prevent his colleagues from inspecting the minute book of the company provided they were doing so in the interest of the company as a whole and not in their individual interest. Param, it is to avoid any possibility of subsequent legal action that the practice of reading the minutes of obtaining the approval of the body there too has sprung up. The world confirmation used in that connection is not correct. As minutes require no confirmation, the decisions having once been made stand without further confirmation. If the necessity for altering minutes arises before they are signed by the chairman, but subsequent to their writing up in the minute book. The alterations may be inserted and initial by the chairman when he signs, but when once minutes have been signed by should not under any circumstance be altered. If it becomes necessary to vary a resolution previously adopted, that variation should always be carried out by means of a minute passed at subsequent meeting. There are some companies keep their minutes on the loose leaf principle and if proper safeguards are provided, there is nothing against this practice. Now the modern loose leaf minute book is provided with the locking device.</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
@@ -2354,22 +2657,37 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 130 words per minute, passage B. Ready? Start.  With reference to the cooperative societies, as far as the cooperative societies are concerned, I can realize the anxiety of the Honorable Minister that if cooperative societies are employing less than 50 people and if they are not employing power, it is desirable that this obligation should not be imposed on these cooperative societies in view of the fact that it is our individual.  intention to encourage cooperative societies. These cooperative societies might not have the necessary resources and therefore may not be in a position to contribute to the provident fund. On the other hand, there is another aspect of the question which it is also necessary to take into consideration and in this behalf, it is necessary because this type of protection and many other types of  protection are given by way of encouragement to the cooperative societies. Again, there are many unscrupulous people who form some sort of cooperative society which is a cooperative society only in name and which in fact is merely a proprietary concern and then they take advantage of these particular provisions.  Sir, we have realized that there were owners and employers who were taking advantage of the fact that the number was kept at 50. It was only when the employees were more than 50 that this particular act was applicable so far.  They were partitioning their establishment into various departments and into various units and thereby they were trying to escape from the provisions of this act.  Fortunately, the government has now made it clear in this bill that no such partitioning will be useful to the employer because even if there is partitioning now they will all be considered as one consolidated establishment and if there were more than 20 people employed then this particular law will be applicable to them.  Some such trick is likely to be resorted to by the employer by calling his concern a cooperative society and thereby trying to escape the extension of the benefits that are being provided for the employees in this particular bill.  Now, sir, there are cooperative societies acts and there are cooperative constitutions where it is made compulsory that after a particular employee has worked for a certain number of years in a given establishment which is a cooperative establishment that employee automatically becomes member of the cooperative society.  Constitutions of this type where the right of membership in the cooperative society is granted to the employees who are working for a particular number of years in that particular society.  I can understand that if this particular bill exempts such societies which permits their own employees to become members of those cooperative societies, it would be quite fair because in that case these employees themselves will become members and therefore they will have dual role of employers being members of the cooperative society and also of employees.  If, however, if, however, particular constitutions does not provide for such compulsory registration of its employees who have worked for particular number of years in that concern as members, then that kind of relationship is as between an employer and an employee.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>English shorthand, 130 words per minute, passage B. Ready, start. With reference to the cooperative societies, as far as the cooperative societies are concerned, I can realize the anxiety of the Honorable Minister that if cooperative societies are employing less than 50 people, and if they are not employing power, it is desirable that this obligation should not be imposed on these cooperative societies in view of the fact that it is our intention to encourage cooperative societies. These cooperative societies might not have the necessary resources and therefore may not be in a position to contribute to the provident fund. On the other hand, there is another aspect of the question which it is also necessary to take into consideration and in this behalf it is necessary because this type of protection and many other types of protection are given by way of encouragement to the cooperative societies. Again, there are many unscrupulous people who form some sort of cooperative society which is a cooperative society only in name and which in fact is merely a proprietary concern and then they take advantage of this particular provision. Sir, we have realized that there were owners and there were employers who were taking advantage of the fact that the number was kept at 50. It was only when the employees were more than 50 that this particular act was applicable so far. They were partitioning their establishment into various departments and into various units and thereby they were trying to escape from the provisions of this act. Fortunately, the government has now made it clear in this bill that no such partitioning will be useful to the employer because even if there is partitioning, now they will all be considered as one consolidated establishment and if there were more than 20 people employed, then this particular law will be applicable to them. Some such trick is likely to be resorted to buy the employer by calling his concern a cooperative society and thereby trying to escape the extension of the benefits that are being provided for the employees in this particular bill. Now, sir, there are cooperative societies acts and there are cooperative constitutions where it is made compulsory that after a particular employee has worked for a certain number of years in a given establishment which is a cooperative establishment that employee automatically becomes member of the cooperative society. Constitutions of this type where the right of membership in the cooperative society is granted to the employees who are working for particular number of years in that particular society. I can understand that if this particular bill exempts such societies which permits their own employees to become members of those cooperative societies. It would be quite fair because in that case, these employees themselves will become members and therefore they will have dual role of employers being members of the cooperative society and also of employees. If, however, particular constitutions does not provide for such compulsory registration of its employees who have worked for a particular number of years in that concern as members, then that kind of relationship is as between and employer and an employee.</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 130 words per minute, trial passage. Ready? Start.  Sir, I must thank the Honorable Mover of this Bill for the opportunity that he gave to the House and to myself on behalf of the Government  to discuss this very important measure as several Honorable Members have more or less unanimously projected the object of this Bill is that  in a vast country of our size, it is essential that as many articles as are essential to life are brought under a system of price discipline  which ultimately reflects into a label being fixed to a community on the basis of a reasonable profit and return to the producer and the seller.  One can easily see that there cannot be any objection to it. As a matter of fact, on behalf of Government and myself, I wholeheartedly welcome this objective.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>English shorthand, 130 words per minute, trial passage. Ready, start. Sir, I must thank the honorable mover of this bill for the opportunity that he gave to the house and to myself on behalf of the government to discuss this very important measure as honourable members have more or less unanimously projected, the object of this bill is that in a vast country of our size, it is essential that as many articles as are essential to life are brought under a system of price discipline which ultimately reflects into a label being fixed to a community on the basis of a reasonable profit and return to the producer and the seller. One can easily see that there cannot be any objection to it. As a matter of fact, on behalf of government and myself, I wholeheartedly welcome this objective.</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2754,7 @@
       <c r="P22" s="2" t="n"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>English shorthand, 130 words per minute, passage A, ready, start, a glacier is a large body  of ice and snow, it forms because the snow is an area does not all melt in summer, each  winter more snow is added, the weight of all the snow creates pressure, this pressure turns  the lower parts of snow into ice, after this happens for many years, the glacier will start  growing large, it becomes so heavy that gravity causes the ice to move, it flows downwards  like water but very slow, the glacier only move about 50 meters per year, new snowfalls  replace the parts that flow away, glaciers are the largest sources of fresh water on earth,  the largest bodies of salt water are the oceans, glaciers will only form in places that are cold  enough and get enough snow over time, this can take a long time, it often takes tens or hundreds  of years for a glacier to form, there are two kinds of glaciers, continental glaciers and  alpine glaciers, alpine glaciers are also called mountain glaciers, continental glaciers are glaciers  that spread out over a large area of land, they were created mostly during the ice ages a long  time, there are still some continental glaciers in Greenland and Antarctica, they often flow  downwards into the sea and break up, the broken parts that float in the sea are called icebergs,  alpine glaciers form in mountain areas, they are smaller than continental glaciers, alpine glaciers  usually flow until they reach a point where the temperature is warm enough that ice melts completely  during the summer para, glaciers are very important, they have a large effect on the environment, they do this  because they are very large and heavy, when they move they erode mountains and land, since they froze  the ice, long ago snow crystals and air bubbles inside are kept in good condition, these can provide a large  amount of information for scientists, recently glaciers have been melting more than they did in the past,  many scientists think this is happening because global warming is changing the climate, glaciers are blue in  color, this is because water is very good at absorbing light, only the strongest light with the most energy is  able to escape, blue is the color of light that has the most energy, because of this blue is the only color of  light that can escape without being absorbed, a glacier is a persistent body of dense ice that is constantly  owing under its own weight, glaciers slow deform and flow under stresses induced by their weight creating and  other distinguishing features, glaciers form only on land and are distinct from the much thinner sea ice and  lake ice that forms on the surface of bodies of water, many glaciers from temperature alpine and seasonal  polar climates store water as ice during the colder seasons and release it later in the form of melt  water as warmer summer temperatures because the glacier to melt creating a water source that is specially  important for plants, animals and human uses when other sources may be scanned.</t>
+          <t>English shorthand. 130 words for a minute. Passage A. Ready. Start. A glacier is a large body of ice and snow. It forms because the snow is an area, does not all melt in summer. Each winter, more snow is added. The weight of all, the snow creates pressure. This pressure turns the lower parts of snow into ice. After this happens for many years, the glacier will start growing large. It becomes so heavy that gravity causes the ice to move. It flows downwards like water, but very slow the glacier only move about 50 meters per year. New snowfalls replace the parts that flow away. Glaciers are the largest sources of fresh water on earth. The largest bodies of salt water are the oceans. Glaciers will only form in places that are cold enough and get enough snow over time. This can take a long time. It often takes tens or hundreds of years for a glacier to form. There are two kinds of glaciers, continental glaciers and alpine glaciers. Alpine glaciers are also called mountain glaciers. Continental glaciers are glaciers that spread out over a large area of land. They were created mostly during the ice ages a long time. There are still some continental glaciers in Greenland and Antarctica. They often flow downwards into the sea and break up. The broken parts that float in the sea are called icebergs. Alpine glaciers form in mountain areas. They are smaller than continental glaciers. Alpine glaciers usually flow until they reach a point where the temperature is warm enough that ice melts completely during the summer. Glaciers are very important. They have a large effect on the environment. They do this because they are very large and heavy. When they move, they erode mountains and land. Since they froze long ago, snow crystals and air bubbles inside are kept in good condition. These can provide a large amount of information for scientists, sir. Recently glaciers have been melting more than they did in the past. Many scientists think this is happening because global warming is changing the climate. Glaciers are blue in color, this is because water is very good at absorbing light. Only the strongest light with the most energy is able to escape blue is the color of light that has the most energy. Because of this blue is the only color of light that can escape without being absorbed. A glacier is a persistent body of dense ice that is constantly owing under its own weight. Glaciers slow, deform and flow under stresses induced by their weight, creating and other distinguishing features. Glaciers form honoly on land and are, distinct from the much thinner sea ice and lake ice that forms on the surface of bodies of water. Many glaciers from temperature alpine and seasonal polar climates store water as ice during the colder seasons and release it later in the form of melt water as warmer summer temperatures because the glacier to melt creating a water source that is specially important for plants, animals and human uses when other sources may be scantle.</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -2446,22 +2764,37 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>Are you ready? English shorthand, 130 words per minute. Are you ready for the passage B?  Start. Mr. Deputy Chairman, I have a few brief remarks to make, if I may say so. I think in  this Honourable House, when we discuss such a matter as this, it would be better and in the  fitness of things if we discuss it in terms of principle instead of introducing names  of individuals. How many rupees who get are the names of individual firms? I am not in  the least interested to defend high salaries paid by any business firm either in Civil Street  Calcutta or in any other street anywhere else. But I think as a matter of principle, we should  avoid mentioning names of individuals and firms because it seems to be unjust and unfair. We  in this house are a privileged group of people. But we should be very careful about using our  privilege. Otherwise, we might do damage to the prestige of authority of Parliament in  the eyes of the public. Now, sir, I think we should discuss this measure in terms of principles  and policies. And the two important basic points that are involved in this are a question of  investment and a question of incentives. We have decided to bring about what we call a socialist  society in this country. And a socialist society does not mean that we should engage ourselves in  working out a just distribution of poverty. The main purpose of a socialist society is to produce  a sufficiently large volume of wealth so that we can provide our people with at least the minimum  requirements of civilized human existence in terms of food, cloth, housing, health, education and so on.  Obviously, this wealth production and the volume of it that we require in terms of our situation requires  investment on a massive scale. A socialist society has to invest capital in order to produce wealth.  It may interest my honourable friend to know that in the planning commission in Russia,  there is a whole-time member whose designation is member in charge of capital investment. It sounds  rather odd that a socialist country has to appoint man whose principal anxiety is to work out the  best way of capital use. Sir, in any kind of society such as ours, it is possible to work out the amount of  savings that the society can possibly make in terms of its own situation and the amount of investment that  is necessary in order to produce the volume of wealth that we have got to produce if we are going to achieve  our social objectives. The difference between what we have got to invest and what we can possibly save  in terms of our own society is very wide gap in our situation and that gap has to be filed obviously by  for importing capital from wherever we can get from socialist or communist society. By all means,  we should take it. If we cannot get enough from them, we have to take from other kinds of society whether  we agree or disagree with the social purposes or the kind of political organization that they believe in.</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>We ready. English shorthand. 130 words per minute. We ready for the passage B. Start. Mr. Deputy Chairman. I have a few brief remarks to make. If I may say so, I think in this Honorable House House when we discuss such a matter as this, it would be better and in the fitness of things if we discuss it in terms of principle instead of introducing names of individuals. How many rupees who get are the names of individual firms? I am not in the list interested to defend high salaries paid by any business firm either in Civil Street, Calcutta or in any other street anywhere else. But I think as a matter of principle, we should avoid mentioning names of individuals and firms because it seems to be unjust and unfair. We in this house are a privileged group of people. But we should be very careful about using our privilege, otherwise we might do damage to the prestige of authority or parliament in the eyes of the public. Now, sir, I think we should discuss this major in terms of principles and policies and the two important basic points that are involved in this are a question of investment and a question of incentives. We have decided to bring about what we call a socialist society in this country and a socialist society does not mean that we should engage ourselves in working out a just distribution of poverty. The main purpose of a socialist society is to produce a sufficiently large volume of wealth so that we can provide our people with at least the minimum requirements of civilized human existence in terms of food cloth, housing, health, education and so on. Obviously this wealth production and and a volume of it that we require in terms of our situation requires investment on a massive scale. A socialist society has to invest capital in order to produce wealth. It may interest my honourable friend to know that in the Planning Commission in Russia, there is a whole-time member whose designation is member in charge of capital investment, it sounds rather odd that a socialist country has to appoint man whose principal anxiety is to work out the best way of capital use, para. Sir, in any kind of society such as ours, it is possible to work out the amount of savings that the society can possibly make in terms of its own situation and amount of investment that is necessary in order to produce the volume of wealth that we have got to produce if we are going to achieve our social objectives. The difference between what we have got to invest and what we can possibly save in terms of our own society is very wide gap in our situation and that gap has to be filed obviously by importing capital from wherever we can get it if we can get from socialist or communist society by all means we should take it if we cannot get enough from them we have to take from other kinds of society whether we agree or disagree with the social purposes or the kind of political organization that they believe in.</t>
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
         <is>
-          <t>We are ready, English shorthand, 130 words per minute, ready for the trial passage, start.  Sir, I must thank the honorable mover of this bill for the opportunity that he gave to the  House and to myself on behalf of the government to discuss this very important measures, as  several honorable members have more or less unanimously projected. The object of this  bill is that in a vast country of our size, it is essential that as many articles are  essential to life are brought under a system of price discipline, which ultimately reflects  into a label being fixed to a commodity on the basis of reasonable profit and return.  to the producer and seller. One can easily see that there cannot be any objection to it.  As a matter of fact, on behalf of the government and myself, I wholeheartedly welcome this objective.</t>
+          <t>en</t>
         </is>
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>We are ready. English shorthand. 130 words per minute. Ready for the trial passage. Start. Sir, I must thank the honourable mover of this bill for the opportunity that he gave to the House and to myself on behalf of the government to discuss this very important measures. As several honourable members have more or less unanimously projected, the object of this bill is that in a vast country of our size, it is essential that as many articles are essential to life are brought under a system of price discipline which ultimately reflects into a label being fixed to a commodity on the basis of reasonable profit and return to the producer and seller. One can easily see that there cannot be any objection to it as a matter of fact. On behalf of government and myself, I wholeheartedly welcome this objective.</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2861,7 @@
       <c r="P23" s="2" t="n"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन, साथ शब्ट प्रतिमिनीट  पैसेज ए, रेडी?  स्टार्ट  भारत हा एक कुरुशी प्रधान देश आहे  भारताचा या खाद्य संपन्न ते मागे  शेतकर्यांचे योगदान मोलाचे आहे  भारत ही शेतकर्याची भूमी आहे  अपल्या देशाची बरीच शी लोकसंख्या गावा मध्ये रहाते  व शेती करते  भारतीय शेतकर्याचा सगली कडे सन्मान होतो  कारण शेतकरीच संपूर्ण देशा साथी खाद्य उगवतो  शेतकर्याचे जीवन अतीशे व्यस्त अस्ते  शेत नांगर्णे बी लावने  रात्रंदिवस शेताची राखन कर्णे इत्यादी कारिया मध्ये  शेतकरी कायम गुंतलेला अस्तो  शेतकरी सकाली लवकर उड़तो  आपले बैल आणी इतर सर्व सामान घेवन  शेता कडे निगतो  तासन तास शेताच तो काम करतो  शेतकर्याचा घरचे  इतर लोक सुधा  शेताच त्याची मदद करताच  शेतकर्याचे जेवन अतीशे साधे अस्ते  बरेच शेतकरी  चटनी भाकर खावन  दिवस काड़त अस्तात  दुपारी शेतकर्याचा घरचे त्याची पत्नी  किम्मा दुसरे कोणी तरी  जेवन गेवन येते  शेतकरी जेवन करून  काही मिन्तांचा  विशरांती नंतर  पुन्हा अपल्या कामाला लागतो  तो कठील परिशरम करतो  पण एवड्या परिशरमा नंतर देखिल  त्याला जास्त लाब होत नाही परिशेत  शेतकर्याचे जीवन  खूपच साधे अस्ते  त्याचा पहराव ग्रामीन अस्तो  बरेज शेतकरी  कच्चा घरात रहतात  शेतकर्याची संपत्ती  बैल आणी काही एकर जमीन अस्ते  शेतकरी हा देशाचा आत्मा अस्तो  आज शेतकर्याला  सरकार द्वारे अधिक-अधिक मदत मिलाईला हवी  त्याला शेतीचे सर्व अधुनीक यंत्र  वकितक नाशके उपलप्थ करून द्याईला हवेत  स्वातेंत्र प्राप्तीचा अनेक वर्षानंतर ही  शेतकर्याची स्थिती जशीचा तशी आहे  असे महणाईला हरकत नाही  झाला हरकत नाही</t>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनट पसेज ए रेडी स्टार्ट भारत हा एक कृषीपधान देश आहे भारताच्या या खाद्य संपन्नतेमागे शेतकऱ्यांचे योगदान मोलाचे आहे भारत ही शेतकऱ्याची भूमी आहे आपल्या देशाची बरीचशी लोकसंख्या गावामध्ये राहते व शेती करते भारतीय शेतकऱ्याचा सगळीकडे सन्मान होतो कारण शेतकरीच संपूर्ण देशासाठी खाद्य उगवतो शेतकऱ्याचे जीवन अतिशय व्यस्त असते शेत नांगरणे बी लावणे रात्रंदिवस शताची राखण करणे इत्यादी कार्यामध्ये शेतकरी कायम गुंतलेला असतो शेतकरी सकाळी लवकर उठतो आपले बैल आणि इतर सर्व सामान घेऊन शेताकडे निघतो तासन तास शेतात तो काम करतो शेतकऱ्याच्या घरचे इतर लोक सुद्धा शेतात त्याची मदत करतात शेतकऱ्याचे जेवण अतिशय साधे असते बरेच शेतकरी चटणी भाकर खाऊन दिवस काढत असतात दुपारी शेतकऱ्याच्या घरून त्याची पत्नी किंवा दुसरे कोणी तरी जेवण घेऊन येते शेतकरी जेवण करून काही मिनिटांच्या विश्रांती नंतर पुन्हा आपल्या कामाला लागतो तो कठीण परिश्रम करतो पण एवढ्या परिश्रमा नंतर देखील त्याला जास्त लाभ होत नाही परिचछेत शेतकऱ्याचे जीवन खूपच साधे असते त्याचा पेहराव ग्रामीण असतो बरेच शेतकरी कच्च्या घरात राहतात शेतकऱ्याची संपत्ती बैल आणि काही ए जमीन असते शेतकरी हा देशाचा आत्मा असतो आज शेतकऱ्याला सरकार दवारे अधिकाधिक मदत मिळायला हवी त्याला शेतीचे सर्व आधुनिक यंत्र व कीटकनाशके उपलब्ध करून द्यायला हवेत स्वातंत्र्य प्राप्तीच्या अनेक वर्ष नंतरही शेतकऱ्यांची स्थिती जशीच्या तशी आहे असे म्हणायला हरकत नाही</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
@@ -2538,22 +2871,37 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन साथ शब्द प्रतिमिनीट, पैसेज बी, रेडी, स्टार्ट  भारताला क्रुशी प्रधान डेश मटले जाते, भारती य अर्थ व्यवस्थेचा कणा शेती हाच आहे  शेतात काम करनार्या व्यक्तिला शेतकरी मटले जाते, शेतकरी हाँ संपूर्ण डिवस शेतात काम करतो  उन वारा पाउस इत्या दिनची परवा न करता आपले कार्य करीत अस्तो  शेतकरी कठीन परिश्रमाचे प्रतीक आहे त्याचात फार सैयम अस्तो  वर्ष भर शेतात काम करून तो आपल्या कश्टाचा फडाची वाट पहात अस्तो  आपले जीवन सन्मानाने जकतो  आपले संपूर्ण आयुष निसरगाचा सानिध्यात गालवतो  शेतकर्याचे जीवन संतूलित अस्ते तो दररोज सकाली लवकर उठतो  डिवस भरात त्याला अनेक कामे कराईची अस्तात  सकाली लवकर उठून तयारी वगैरे करून तो शेताकडे निकतो  तो आपला संपूर्ण दिवस शेतातील पिकांचा कालजी मध्ये घालोतो  शेत नांगर्णे पीक पेर्णे पिकाला पाणी देने उन वार्या पासून आपल्या पिकाचे रक्षन करणे  इत्यादी अनेक कामे शेतकर्याला करावी लागतात परिछेद  शेतकरी त्याचे पीक अनेक नैसर्गीक आपत्ती पासून संरक्षित करतो  पशु पक्षी गिडे मुंग्या इत्यादीन पासून तो आपल्या पिकाचे रक्षन करतो  शेतात सुन्दर बहर लेल्या पिकामागे शेतकर्याची शेती विशयीची भक्ती प्रेम आणी कठीन परिश्रम अस्ते  एक शेतकरी संपूर्ण जगातिल मानवाला अन्न पुरविण्या साथी आपले जीवन व्यतीत करतो  दिवस भर शेतात काम केल्यावर संध्या काली सूर्य मावल्या नंतर शेतकरी अपल्या घरी पहोचतो  जावेली तो घरी पहोचतो तेम्हा तो अत्यंत ठकलेला व समाधानी अस्तो</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट भारताला कृषी प्रधान देश म्हटले जाते भारतीय अर्थव्यवस्थेचा कणा शेती हाच आहे शेतात काम करणाऱ्या व्यक्तीला शेतकरी म्हटले जाते शेतकरी हा संपूर्ण दिवस शेतात काम करतो ऊन वारा पाऊस इत्यादीची परवा न करता आपले कार्य करीत असतो शेतकरी कठीण परिश्रमाचे प्रतीक आहे त्याच्यात फार संयम असतो वर्षभर शेतात काम करून तो आपल्या कष्टाच्या फळाची वाट पाहत असतो आपले जीवन सन्मानाने जगतो आपले संपूर्ण आयुष्य निसर्गाच्या सानिध्यात घालवतो शेतकऱ्याचे जीवन संतुलित असते तो दररोज सकाळी लवकर उठतो दिवसभरात त्याला अनेक कामे करायची असतात सकाळी लवकर उठून तयारी वगैरे करून तो शेताकडे निघतो तो आपला संपूर्ण दिवस शेतातील पिकांच्या काळजीमध्ये घालवतो शेत नांगरणे पीक पेरणे पिकाला पाणी देणे ऊन वाऱ्यापासून आपल्या पिकाचे रक्षण करणे इत्यादी अनेक कामे शेतकऱ्याला करावी लागतात परिच्छद शेतकरी त्याचे पीक अनेक नैसर्गिक आपत्तीपसून संरक्षित करतो पशु पक्षी किडे मुंग्या इत्यादीपसून तो आपल्या पिकाचे रक्षण करतो शेतात सुंदर बहरलेल्या पिकामागे शेतकऱ्याची शेती विषयीची भक्ती प्रेम आणि कठीण परिश्रम असते एक शेतकरी संपूर्ण जगातील मानवाला अन्न पुरविण्यासाठी आपले जीवन व्यतीत करतो दिवसभर शेतात काम केल्यावर संध्याकाळी सूर्य मावळल्यानंतर शेतकरी आपल्या घरी पोहोचतो ज्या वेळी तो घरी पोहोचतो तेव्हा तो अत्यंत थकलेला व समाधानी असतो</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U23" s="2" t="inlineStr">
-        <is>
-          <t>मराथी लगुलेखन, साथ शब्द प्रतिमिनेट, ट्रायल पैसेज, सरावाचा उतारा, रेडी, स्टार्ट, महाशे, आज, जगात, लोक संख्या वाढ़ीचा,  प्रश्ण, तोंड, वासून, उभा आहे, वेलीच, त्याला, पाय बंद, न, घातल्यास, विपरीद, परिडाम, जाल्या शिवाय, रहाणार नाही,  भारताची 31 मार्च, एकोणिशे 55 परियंत, लोक संख्या 44 कोटी होती, एवडी लोक संख्या, असन्याची मुख्य 3 कारणे आहेद,  वाडते, जन्म प्रमाण, घडते, मुरुत्यू प्रमाण, व, अशिक्षित पड़ा,</t>
-        </is>
-      </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट ट्रायल पॅसेज सरावाचा उतारा रेडी स्टार्ट महाशय आज जगात लोकसंख्या वाढीचा प्रश्न तोंड वासून उभा आहे वेळीच त्याला पायबंद न घातल्यास विपरीत परिणाम झाल्याशिवाय राहणार नाही भारताची एकतीस मार्च एकोणीशे पंच्याऐंशी पर्यंत लोकसंख्या चौऱतर कोटी होती एवढी लोकसंखण्याची मुख्य त कारणे आहेत वाढते जन्मप्रमाण घटते मृत्यू प्रमाण व अशिक्षित पणा</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2968,7 @@
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन, साठ शब्द प्रती मिनिट, पैसेज ए, रेडी, स्टार्ट, बंधुन्नो, परिचेद, माजापुर्वी या ठिकानी वैद्यकिय वेवसायतेल, अनेक अनुभवी व नामवंत लोकांची मार्गदर्शन पर भाशने जालेली आहेत,  तेनचा भाशनातुन, तेननी स्वताचे जे अनुभव अतिशे स्पष्टपने सांगित लेले आहेत, ते आपना सर्वाना भावी आयुश्यात बहु मोलाचे थरतील यात शंका नाही.  तथापी या सबेचा अध्यक्ष या नातैने मला आपनाशी काही शब्द बोलावयाचे आहेत परिचे.  आपल्या सार्ख्या वेद्यकिय पद्विधरान समोर भाशन करन्याची माजी ही पहिलीच वेड आहे.  सादारन तहा कोठे ही अध्यक्ष मनुन जबाबदारी स्विकारतानना त्या सबेचा विशयाशी माजा काही संबंध असेल.  क्युवा त्या सबेच्या विशयाशे मला काही द्ञान असेल.  अगर त्या बद्दल काही माहिती असेल तरच मी ती जबाबदारी स्विकारतो.  उद्देश एकच अस्तो की माजा अश्या सभातिल उपस्थिती मुले संबंधित जनतेला.  काही मदत होँ शक्ते व काही मार्गदर्शन मी त्यानना करू शक्तो.  मी व्यवसायाने कारखानदार व जातीने मागा स्वर्गिय आहे.  त्या मुले कारखान्याचे अगर उद्द्योग धंद्यांचे उद्गाठन समारंभ मजूर संगटनांचा सभा दलित बांधवांचे मिलावे.  आणी तैंचे विवित कारेक्रम अशाच कारेक्रमात मी भाग घेत अस्तू.  माजा सामाजिक जिवनाचे क्षेत्र यवडेच मर्यादित असतान्ना मी आपल्या या चर्चा सत्राचा समारोपाचे निमंत्रन का स्विकारले असाही प्रश्ण त्या मुले निर्मान हूँ शकेल.  तसा वैद्यगिय व्यवसायाशी माजा काही ही संबंद नाही हे खरे आहे.  परेंटु मला या क्षेत्राची आवड आहे मनुन मी हे निमंत्रन स्विकारले आहे.  परिच्चेद कड़ावे आपला.</t>
+          <t>मराठी लघुलेखन साठ शब्द प्र्रतिमिनिट पॅसेज ए रेडी स्टार्ट बंधून नो परिच्छेद माझ्यापूर्वी या ठिकाणी वैद्यकीय व्यवसायातील अनेक अनुभवी व नामवंत लोकांची मार्गदर्शनपर भाषणे झालेली आहेत त्यांच्या भाषणातून त्यांनी स्वतचे जे अनुभव अतिशय स्पष्टपणे सांगितलेले आहेत ते आपणा सर्वांना भावी आयुष्यात बहुमलाचे ठरतील यात शंका नाही तथापि या सभेचा अध्यक्ष या नात्याने मला आपणाशी काही शब्द बोलावयाचे आहेत परिच्छेद आपल्यासारख्या वैद्यकीय पदवीधरांसमोर भाषण करण्याची माझी ही पहिलीच वेळ आहे साधारणत कुठेही अध्यक्ष म्हणून जबाबदारी स्वीकारताना त्या सभेच्या विषयाशी माझा काही संबंध असेल किंवा त्या सभेच्या विषयाचे मला काही ज्ञान असेल अगर त्याबद्दल काही माहिती असेल तरच मी ती जबाबदारी स्वीकारतो उद्देश एकच असतो की माझ्या अशा सभातील उपस्थितीमुळे संबंधित जनतेला काही मदत होऊ शकते व काही मार्गदर्शन मी त्यांना करू शकतो मी व्यवसायाने कारखानदार व जातीने मागासवर्गीय आहे त्यामुळे कारखान्याचे अगर उद्योगधंद्यांचे उद्घाटन समारंभ मजूर संघटनांच्या सभा दलित बांधवांचे मिळावे आणि त्यांचे विविध कार्यक्रम अशाच कार्यक्रमात मी भाग घेत असतो माझ्या सामाजिक जीवनाचे क्षेत्र एवढेच मर्यादित असताना मी आपल्या या चर्चासत्राच्या समारोपाचे निमंत्रण का स्वीकारले असाही प्रश्न त्यामुळे निर्माण होऊ शकेल तसा वैद्यकीय व्यवसायाशी माझा काहीही संबंध नाही हे खरे आहे परंतु मला या क्षेत्राची आवड आहे म्हणून मी हे निमंत्रण स्वीकारले आहे परिच्छेद कळावे आपला</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -2630,22 +2978,37 @@
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन, साठ शब्द प्रती मिनिट, पैसेज बी, रेडी, स्टार्ट, परिछेद, आजच्या काडात, जाहिरातीन ना, हे जे महत्व आले आहे, ते विक्रेते, आनी ग्राहक यांच्या, गर्जे तुम आले आहे,  जाहिरात, ही केवल, विक्रेतेंच्याच, फैद्या साठी असते, असे नवे, जाहिरात, हा, विक्रेता, उत्पादक, आनी ग्राहक, यांच्या तिल, सववाद आहे, उत्पादनाच्या, क्षेत्रात, अध्योगी करना मुले,  एवधी, विविधता, आनी प्रचंड स्पर्धा, निर्मान जालेली आहे, की ग्राहकाला, आपल्या, गर्जे च्या, पूर्ती साथी, योग्य वस्तुची, निवड करने, अउघड जालेले आहे,  एकच वस्तु, अनेक उत्पादक, तयार करू लागले मुले, तैंचा तही, अंतर्गत स्पर्धा, शुरू जाली आहे,  अन्य उत्पादना होन, आपल्याच उत्पादनाची गुनवत्ता, उपयुक्तता, कशी मोटी आहे, हे ग्राहकान्ना, पटोन, देन्यात, तैंचा मद्धे, चड़ा ओड, लागली आहे,  कुठली ही जाहिरात, ही विक्रेता आनी ग्राहक, यांचा मधिल उत्पादक सववाद असलाने, ती अधिकाधिक वेधक असने अवश्यक असते,  त्या मुले, जाहिरातीचा मथला, त्या मथलात समाविष्ट जालेल्या, वर्ननाचा तपशील, कंपनीचे बोध चिन्ह, क्युवा मुद्रा,  कंपनीचे नाव वपत्ता आनी घोश वाक्य, अशा सर्व गोश्टी कडे लक्ष दैवे लागते, ती सोपी सर्वानना समझेल अशी असावी लागते,  जाहिरातीत, जे काही सांगित ले आहे, ते आपले आहे, विश्वासार्ह आहे, असे ही वाटनाची गरज असते,  सभोव तालची परिस्थिती, त्या परिस्थिती मधिल वास्तवतेचे भाण आनी जाण दोनी असावे लागते,  जाहिरात, ही मन आकर्षुन घेनारी त्याच बरोबर अंतक करनावर ठसे उमट विनारी असली पाहिजे,  स्पर्धेच्या युगात जाहिरातीला महत्व प्राप्त जालेले आहे,  जाहिराती मुले ग्राहकांची पसंती वस्तुन्ना मिलत अस्ते,</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट परिच्छेद आजच्या काळात जाहिरातींना हे जे महत्त्व आले आहे ते विक्रेते आणि ग्राहक यांच्या गरजेतून आले आहे जाहिरात ही केवळ विक्रेत्यांच्याच फायद्यासाठी असते असे नव्हे जाहिरात हा विक्रेता उत्पादक आणि ग्राहक यांच्यातील संवाद आहे उत्पादनाच्या क्षेत्रात औद्योगकरणामुळे एवढी विविधता आणि प्रचंड स्पर्धा निर्माण झालेली आहे की ग्राहकाला आपल्या गरजेच्या पूर्तीसाठी योग्य वस्तूची निवड करणे अवघड झालेले आहे एकच वस्तू अनेक उत्पादक तयार करू लागल्यामुळे त्यांच्यातही अंतर्गत स्पर्धा सुरू झाली आहे अन्य उत्पादनाहून आपल्याच उत्पादनाची गुणवत्ता उपयुक्तता कशी मोठी आहे हे ग्राहकांना पटवून देण्यात त्यांच्यामध्ये चढा ओढ लागली आहे कुठलीही जाहिरात ही विक्रेता आणि ग्राहक यांच्यामधील उत्पादक संवाद असल्याने ती अधिकाधिक वेधक असणे आवश्यक असते त्यामुळे जाहिरातीचा मथळा त्या मथळ्यात समाविष्ट झालेल्या वर्णनाचा तपशील कंपनीचे बोधचिन्ह किंवा मुद्रा कंपनीचे नाव व पत्ता आणि घोषवाक्य अशा सर्व गोष्टीकडे लक्ष द्यावे लागते ती सोपी सर्वांना समजेल अशी असावी लागते जाहिरातीत जे काही सांगितले आहे ते आपले आहे विश्वासार्ह आहे असेही वाटण्याची गरज असते सभोवतालची परिस्थिती त्या परिस्थितीमधील वास्तवतेचे भण आणि जाण दोन्ही असावे लागते जाहिरात ही मनआकर्षून घेणारी त्याचबरोबर अंतःकरणावर ठसे उमटविणारी असली पाहिजे स्पर्धेच्या युगात जाहिरातीला महत्त्व प्राप्त झालेले आहे जाहिरातीमुळे ग्राहकांची पसंती वस्तूंना मिळत असते</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U24" s="2" t="inlineStr">
-        <is>
-          <t>मराथी लगुलेखन, साट शब्द प्रती मिनिट, ट्रायल पैसेज, रेडी, स्टार्ट, माशे परिच्छेद, आज, जगात, लोक संक्या वाडीचा, प्रश्न, तोंड वासुन, उबा आहे,  वेलिच, त्याला, पायबंध, न, गातल्यास, विपरित परिणाम, जाल्या शिवाय, राहनार नाही, भारताची, 31 मार्च, एकोनाविश्य, पंचैंची परियंत, लोक संक्या, शवर्यात्तर कोटी होती,  योडी, लोक संक्या, असन्याची, मुख्य, तीन, कारणे आहेत, वाड़ते, जन्म प्रमान, घटते, वृत्यु प्रमान, व, अशिक्षीत पना,</t>
-        </is>
-      </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट ट्रायल पॅसेज रेडी स्टार्ट महाशय परिच्छेद आज जगात लोकसंख्या वाढीचा प्रश्न तोंड वासून उभा आहे वेळीच त्याला पायबंद न घातल्यास विपरीत परिणाम झाल्याशिवाय राहणार नाही भारताची एकतीस मार्च एकोणावीशे पंच्याऐंशी पर्यंत लोकसंख्या चौऱ्यातर कोटी होती एवढी लोकसंख्या असण्याची मुख्य तन कारणे आहेत वाढते जन्म प्रमाण घटते मृत्यू प्रमाण व अशिक्षितपणा</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2712,7 +3075,7 @@
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>मराठी लगूलेखन साठ शब्द प्रती मिनिट पैसेज ए रेडी स्टार्ट पैरा भारतीय महिलानी प्रगती आणी आउवाने दोनी अनोभवली आहेत  पुर्वीचा कालात महिलानना भेद भावाचा सामना करावा लागत होता विशेश ताहा शिक्षन आणी नोकरी मदे तथापी वाढत्या जानी वे सह आता बरेच लोग विभीद क्षेत्रात काम करतात  आणी नेत्रुत्वाची पदे भुशवतात असे असु नहीं लिंग आधारित हिमसाचार आणी असमानता या सारखे प्रश्न अजु नहीं कायम आहेत्  निरोगी समाजा साथी महिलान साथी समानता आणी आदर सु निस्चीत करणे आवशक आहे  गेल्या काही वर्शात भारत आतिल महिलांची स्थिती बदल्ली आहेत्  पुर्वी त्यांचा भुमिका मुख्यत्वे घरा पुर्त्या मर्यादित होत्या आणी त्यान्ना मर्यादित अधीकार होते्  स्वातंत्र्य आणी आधोनिक शिक्षणा सह अधीक मुली शालेत जात आहेत् आणी महिला कामाचा ठिकानी सामील होत आहेत्  काई द्यान मुले महिलांची सुरक्षा आणी अधीकार सुधारले आहेत् तरी ही भेदभाव आणी हिंसा चार हे प्रमूख चिंतेचे विशय आहेत्  प्यारा शिक्षणा आणी संधीत वारे महिलाना सक्षम बनवने हे भारताचा विकासा साथी महत्वाचे आहे  भारतातिल महिलांची बदलती स्थिती समान तेचा दिशेने एक सकारात्मक पावूल आहे  खरी प्रगती साध्य करणया साथी त्याना आदर सौरक्षण आणी समान संधीना प्रोच्षाहन देने अत्यांत महत्वाचे आहे  प्राचीन काला पासुन आधुनिक भारतात महिलांचे स्थान कसे विकसीत जाले आहे यावर जास्त भर तेतो  वैदीक कालात महिलांना काही स्वातंत्रय होते परंतु सामाजिक रिती रिवाजान मुले हलु हलु त्यांचे अधिकार गमावले गेले  आज महिला शिक्षण, राजकारण आणी व्यवसायात पुन्ना स्थान मिलवत आहेत।  मुलीनचा शिक्षणाला प्रोच्चाहन देनारे उपक्रम हे सकारात्मक पावुल आहे।</t>
+          <t>मराठी लघुलेखन साठ शब्द प्रति मिनिट पॅसेज ए रेडी स्टार्ट पॅरा भारतीय महिलांनी प्रगती आणि आव्हाने दोन्ही अनुभवली आहेत पूर्वीच्या काळात महिलांना भेदभावाचा सामना करावा लागत होता विशेषत शिक्षण आणि नोकरीमध्ये तथापि वाढत्या जाणीवेसह आता बरेच लोक विविध क्षेत्रात काम करतात आणि नेतृत्वाची पदे भूषवतात असे असूनही लिंग आधारित हिंसाचार आणि असमानता यासारखे प्रश्न अजूनही कायम आहेत निरोगी समाजासाठी महिलांसाठी समानता आणि आदर सुनिश्चित करणे आवश्यक आहे गेल्या काही वर्षात भारतातील महिलांची स्थिती बदलली आहे पूर्वी त्यांच्या भूमिका मुख्यत्वे घरापुरत्या मर्यादित होत्या आणि त्यांना मर्यादित अधिकार होते स्वातंत्र्य आणि आधुनिक शिक्षणासह अधिक मुली शाळेत जात आहेत आणि महिला कामाच्या ठिकाणी सामील होत आहेत कायद्यांमुळे महिलांची सुरक्षा आणि अधिकार सुधारले आहेत तरीही भेदभाव आणि हिंसाचार हे प्रमुख चिंतेचे विषय आहेत पॅरा शिक्षण आणि संधीद्वारे महिलांना सक्षम बनवणे हे भारताच्या विकासासाठी महत्त्वाचे आहे भारतातील महिलांची बदलती स्थिती समानतेच्या दिशेने एक सकारात्मक पाऊल आहे खरी प्रगती साध्य करण्यासाठी त्यांना आदर संरक्षण आणि समान संधीना प्रोत्साहन देणे अत्यंत महत्त्वाचे आहे प्राचीन काळापासून आधुनिक भारतात महिलांचे स्थान कसे विकसित झाले आहे यावर जास्त भर देतो वैदिक काळात महिलांना काही स्वातंत्र्य होते परंतु सामाजिक रीतीरिवाजांमुळे हळूहळू त्यांचे अधिकार गमावले गेले आज महिला शिक्षण राजकारण आणि व्यवसायात पुन्हा स्थान मिळवत आहेत मुलींच्या शिक्षणाला प्रोत्साहन देणारे उपक्रम हे सकारात्मक पाऊल आहे</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -2722,22 +3085,37 @@
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>मराठे लगुलेखन साठ शब्द प्रती मिनिट, पैसेज बी, रेडी, स्टार्ट, पैरा, महिलांचा हक, प्रगती आणी सततचा समस्या या दोन्नी गोष्टिनचा विचार केला आहे,  प्राचेन भारतात बाल विवाह आणी सती या सार्ख्या सामाजिक गईर क्रुत्यान्नी त्यांचे अधिकार मर्यादीत केले होते, त्या पैक्षा महिलांचे स्थिती सांगली होती,  स्वातंत्र्या नंतर सुधार्णा जसेकी मतदानाचा अधिकार आणी समान वेतन काईदे, परिस्तिती सुधार्णाचे उद्धिष्ट होते,  आज महिला डॉक्टर अभी अंते, आणी राजकी य नेत्या आहेक्ट, परन्तु अनेकाना अजु नहीं घरगूती हिउंसाचार,  आणी सेक्षणिक अड्थल्यां चार्ख्या आउवानाना तोंड द्यावे लागते, ग्रामेन भागातिल मुली ना अनेकदा शालान मधे प्रवेश नस्तो,  जा मुले मुलान पेक्षा साक्षरता दर कमी होतो, मुली वाचवा, मुली शिकवा, सार्ख्या योजना या अंतराना भरून काडणयाचा उद्देश ठेवतात,  विवीध क्षेत्रात, नावाज लेल्या नामवंत महीला, तैंचा कामगिरीने राष्ट्राला प्रेरणा देतात,  समान संधी देन्याचा सकारात्मक परिणाम दर्शवितात, शतकानू शतके महीलाना, कुटुम्ब आनी समाजात,  आदर आणी स्वातंत्र्य होते, कालांतराने हुंडा, छल आणी लिंग भेद या सार्ख्या प्रथान मदे त्यांचे स्वातंत्र्य मर्यादित होते,  तथा पी आधुनीक युगात सकारात्मक बदल जाले आहेत,  शिक्षन रोजगाराचा संधी आणी काईदेशिर हक्क वाधले आहेत,  तरी ही अनेक महिलानना अजु नहीं भेद भाव आणी हिंसाचाराचा सामना करावा लागतो,  अचा समस्या जा, खर्या, लिंग, समान तेला, अडथला आनितात,  सक्षम महिला भारताचा विकासा साथी आवश्यक आहेत,  त्या आरोग्य, शिक्षन, अर्थ व्यवस्ता आणी संस्कृतीत योगदान देतात,  घरगूती हिंसाचार, प्रती बंधक काईडा, आणी स्वच्छ भारत,  सार्ख्या मोही माननी महिलानना अनेक योजने द्वारे मदद केली आहे,</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट पॅरा महिलांच्या हक्क प्रगती आणि सततच्या समस्या या दोन्ही गोष्टींचा विचार केला आहे प्राचीन भारतात बालविवाह आणि सती यासारख्या सामाजिक गैरकृत्यांनी त्यांचे अधिकार मर्यादित केले होते त्यापेक्षा महिलांची स्थिती चांगली होती स्वातंत्र्यानंतर सुधारणा जसे की मतदानाचा अधिकार आणि समान वेतन कायदे परिस्थिती सुधारण्याचे उद्दिष्ट होते आज महिला डॉक्टर अभियंते आणि राजकीय नेत्या आहेत परंतु अनेकांना अजूनही घरगुती हिंसाचार आणि शैक्षणिक अडथळ्यांसारख्या आव्हानाना तोंड द्यावे लागते ग्रामीण भागातील मुलींना अनेकदा शाळांमध्ये प्रवेश नसतो ज्यामुळे मुलांपेक्षा साक्षरता दर कमी होतो मुली वाचवा मुली शिकवा सारख्या योजना या अंतरांना भरून काढण्याचा उद्देश ठेवतात विविध क्षेत्रात नावाजलेल्या नामवंत महिला त्यांच्या कामगिरीने राष्ट्राला प्रेरणा देतात समान संधी देण्याचा सकारात्मक परिणाम दर्शवितात शतकानुशतके महिलांना कुटुंब आणि समाजात आदर आणि स्वातंत्र्य होते कालांतराने हुंडा छळ आणि लिंगभेद यासारख्या प्रथांमध्ये त्यांचे स्वातंत्य मर्यादित होते तथापि आधुनिक युगात सकारात्मक बदल झाले आहेत शिक्षण रोजगाराच्या संधी आणि कायदेशीर हक्क वाढले आहेत तरीही अनेक महिलांना अजूनही भेदभाव आणि हिंसाचाराचा सामना करावा लागतो अशा समस्या ज्या खऱ्या लिंग समानतेला अडथळा आणतात सक्षम महिला भारताच्या विकासासाठी आवश्यक आहेत त्या आरोग्य शिक्षण अर्थव्यवस्था आणि संस्कृतीत योगदान देतात घरगुती हिंसाचार प्रतिबंधक कायदा आणि स्वच्छ भारत सारख्या मोहिमांनी महिलांना अनेक योजनेद्वारे मदत केली आहे</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U25" s="2" t="inlineStr">
-        <is>
-          <t>मराथी लगुलेखन, साथ शब्द प्रती मिनिट, ट्रायल पैसेज, रेडी, स्टाट, महाशय पैरा, आज जगात लोकसंख्या वाडीचा प्रश्न तोन वासून उभा आहे,  वेडीच त्याला पाईबंध न घातल्यास, विपरित परिणाव, जाल्या शिवाय, राहनार नाही, भारताची एक्तिस माज एकुनिश्चे पंच्याईशी परियंत लोकसंख्या चाउर्यात्तर कोटी हुती,  एवडी लोकसंख्या असन्याची मुख्य तीन कारणे आहेत्ट, वाडते जन्म प्रमान, घटते मृत्यु प्रमान, व अशिक्षिती पणा,</t>
-        </is>
-      </c>
       <c r="V25" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट ट्रायल पॅसेज रेडी स्टार्ट महाशय पारा आज जगात लोकसंख्या वाढीचा प्रश्न तोंड वासून उभा आहे वेळीच त्याला पायबंद न घातल्यास विपरीत परिणाम झाल्याशिवाय राहणार नाही भारताची एकतीस मार्च एकोणीशे पंच्याऐंशी पर्यंत लोकसंख्या चौऱ्याहत्तर कोटी होती एवढी लोकसंख्या असण्याची मुख्य तीन कारणे आहेत वाढते जन्म प्रमाण घटते मृत्यू प्रमाण व अशिक्षतीपणा</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2804,7 +3182,7 @@
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुले खन, साथ शब्द प्रतिमिनीट, पैसेज ए, रेडी, स्टार्ट, शेतकरी हे निस संशय पणे आपल्या देशाचा कणा आहेत,  मानवी अस्तित्वा साथी आवश्यक असलेल्या, सरवात आवश्यक उत्पादनांचे उत्पादन करण्या साथी तेच काम करतात,  एकाद्या व्यक्ती कडे, अमर्याद संपत्ति असुशक्ते, परंथु दिवसाचा शेवटी, त्याचा ताटात अन्न आहे की नाही, हे महत्वाचे आहे,  अपल्याकडे इतके पैसे असले तरी, आपन अन्न उत्पादन करू शक्तो असे नाही, परिछेद बाजारात उपलप्ध असलेली, धान्ये आणी डाली,  आणी आणी बाज़ात्स खरेदी करू शक्तो जेम्हा, आपन अवश्यक असलेले धान्य, आणी डाली खरेदी करू शक्तो,  अन्य था लोक भयानक दुशकाडाला सामोरे जातील, आणी उपास मारीने मरतील,  बंगालचा दुशकाडाची सर्वात वाईट अठवण अठवते, लाखो लोक खाण्या साथी, अन्य नसल्याने मरण पावले,  आज आपन अपल्याकडे असलेल्या, अन्य बद्दल कृतद्न्य असले पाहिजे,  कारण कुठे तरी एक शेतकरी समाजाचे पोट भर्ण्या साथी अठक परिश्रम करत आहे,  शेतकरी खूप महतवाचे आहेद, कारण ते अपल्याला आपन खातो ते अन्य पुरवताद परिशेद,  संपूर्ण देश याच कारणा मुले, त्यांचा वर अवलंबून आहे, आपन नेहमीच शेतकर्यान बद्दल बोलतो,  आणि फक्त शब्दान नी त्यांचे कवतू करतो, शेतकर्यान ना मदद करण्या साथी, आपन कदी ही उड़ाकार घेत नाही,  बहुतेक शेतकरी गहू आणि तांदूल कापणीवर अवलंबून अस्तात, कारण ते आपल्या देशात सर्वात जास्त वापरले जानारे अन्न आहे,  मोठ्या प्रमानात, शेतकरी असोत, किम्वा, लहान प्रमानात, असोत, ते सर्वजन, खूप, कमी नफ्या साथी, काम करतात, आणि समाधानी राहतात.</t>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट पॅसेज ए रेडी स्टार्ट शेतकरी हे निःसंशयपणे आपल्या देशाचा कणा आहेत मानवी अस्तित्वासाठी आवश्यक असलेल्या सर्वात आवश्यक उत्पादनांचे उत्पादन करण्यासाठी तेच काम करतात एखाद्या व्यक्तीकडे अमर्याद संपत्ती असू शकते परंतु दिवसाच्या शेवटी त्याच्या ताटात अन्न आहे की नाही हे महत्त्वाचे आहे आपल्याकडे इतके पैसे असले तरी आपण अन्न उत्पादन करू शकतो असे नाही परिचछद बाजारात उपलब्ध असलेली धान्य आणि डाळी आपण फक्त तेव्हाच खरेदी करू शकतो जेव्हा आपण आवश्यक असलेले धान्य आणि डाळी खरेदी करू शकतो अन्यथा लोक भयानक दुष्काळाला सामोरे जातील आणि उपासमारीने मरतील बंगालच्या दुष्काळाची सर्वात वाईट आठवण आठवते लाखो लोक खाण्यासाठी अन्न नसल्याने मरण पावले आज आपण आपल्याकडे असलेल्या अन्नाबद्दल कृतज्ञ असले पाहिजे कारण कुठेतरी एक शेतकरी समाजाचे पोट भरण्यासाठी अथक परिश्रम करत आहे शेतकरी खूप महत्वाचे आहेत कारण ते आपल्याला आपण खातो ते अन्न पुरवतात परिच्छेद संपूर्ण देश याच कारणामुळे त्यांच्यावर अवलंबून आहे आपण नेहमीच शेतकऱ्यांबद्दल बोलतो आणि फक्त शब्दांनी त्यांचे कौतुक करतो शेतकऱ्यांना मदत करण्यासाठी आपण कधीही पुढाकार घेत नाही बहुतेक शेतकरी गहू आणि तांदूळ कापणीवर अवलंबून असतात कारण ते आपल्या देशात सर्वात जास्त वापरले जाणारे अन्न आहे मोठ्या प्रमाणात शेतकरी असोत किंवा लहान प्रमाणात असोत ते सर्वजण खूप कमी नफ्यासाठी काम करतात आणि समाधानी राहतात</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -2814,22 +3192,37 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन साथ शब्द प्रतिमिनीट  पैसेज बी रेडी स्टार्ट  शेती ही शेतकरी आणी शेतकर्यांचे मुले  व शेतात काम करनारे मजूर यांचा साथीचा विशय आहे  व शेती शी निगडीत माहीती  ही संकल्पना अशी का रूढ जाली असावी  तसे बगितले तर शेती हा व्यापक आणी प्रत्येक मानव सब्धतेचा विशय आहे  हे सर्वान्नाच कल्डे पाही जे  कारण असे नेहमी प्रकरशाने दिसून येते की  कुणालाही शेती साथी माहीती गेन्याची विशेश रूची नाहीच  असा समज लोकान मध्ये दिसून येतो की  शेती मंजे फार मेहनतीचे व अउघण काम आहे सर्वान्ना यां गोश्टी समजल्या पाही जेत  आपन जो भाजी पाला फले धान्य पिके इतर आपन रोजचा दैनंदीन जीवनात खातो  ते जमीनीत येते कसे या बद्दल उच्छुकता व माहीती असली पाही जे  वर्तमानातली तरून पिड़ी जेवा या कड़े एक रूची संथी आणी उत्तम व्यवसाई  मणून पाहन्यास सुर्वात करेल तेमा शेती या क्षेत्राचे स्वरूप बदललेले व उत्तम जालेले असेल  शेती हा विशे फक्त शेतकर्यान साथी नाही  हा विशे सर्व पृत्वी तलावरिल प्रत्येक मानव सभ्यतेचा आहे  शेती असे क्षेत्र आहे ज्या मद्ये सर्वान साथीच मोठ्या व उत्तम संधी दडलेल्या आहेद  हे सर्वानना माहीत असेल तसेच सर्वच क्षेत्रातिल शिक्षन संपादन केलेल्या सर्वान साथी शेती मद्ये संधी आहेद  शेती मद्ये विविध पद्धती चे संशोधन व संशोधक होण्यास संधी आहे जसे पिकान मद्ये बियाण्यान मद्ये इत्यादी ठिकाणी संशोधन होत अस्तात्  व खोण्यास मोठा वाव आहे तसेच शेतीत नवीन तंत्रद्न्यानाला देखील चांगला वाव आहे</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनीट पॅसेज बी रेडी स्टार्ट शेती ही शेतकरी आणि शेतकऱ्यांचे मुले व शेतात काम करणारे मजूर यांच्यासाठीचा विषय आहे व शेतीशी निगडीित माहिती ही संकल्पना अशी का रूढ झाली असावी तसे बघितले तर शेती हा व्यापक आणि प्रत्येक मानव सभ्यतेचा विषय आहे हे सर्वांनाच कळले पाहिजे कारण असे नेहमी प्रकर्षाने दिसून येते की कुणालाही शेतीसाठी माहिती घेण्याची विशेष रुची नाहीच असा समज लोकांमध्ये दिसून येतो की शेती म्हणजे फार मेहनतीचे व अवघड काम आहे सर्वांना या गोष्टी समजल्या पाहिजेतेत आपण जो भाजीपाला फळे धान्य पिके इतर आपण रोजच्या दैनंदिन जीवनात खातो ते जमिनीत येते कसे याबद्दल उत्सुकता व माहिती असली पाहिजे वर्तमानातली तरुण पिढी जेव्हा याकडे एक रुची संधी आणि उत्तम व्यवसाय म्हणून पाहण्यास सुरुवात करेल तेव्हा शेती या क्षेत्राचे स्वरूप बदललेले व उत्तम झालेले असेल शेती हा विषय फक्त शेतकऱ्यांसाठी नाही हा विषय सर्व पृथ्वी तलावरील प्रत्येक मानव सभ्यतेचा आहे शेती असे क्षेत्र आहे ज्यामध्ये सर्वांसाठीच मोठ्या व उत्तम संधी दडलेल्या आहेत हे सर्वांना माहत असेल तसेच सर्वच क्षेत्रातील शिक्षण संपादन केलेल्या सर्वांसाठी शेतीमध्ये संधी आहेत शेतीमध्ये विविध पद्धतीचे संशोधन व संशोधक होण्यास संधी आहे जसे पिकांमध्ये बियाण्यामध्ये इ्या ठिकाणी संशोधन होत असतात व होण्यास मोठा वाव आहे तसेच शेतीत नवीन तंत्रज्ञानाला देखील चांगला वाव आहे</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U26" s="2" t="inlineStr">
-        <is>
-          <t>मराथी लगुलेखन, साथ शब्द प्रतिमिनेट, ट्रायल पैसेज, सरावाचा उतारा, रेडी, स्टार्ट, महाशे, आज, जगात, लोक संख्या वाढ़ीचा,  प्रश्ण, तोंड, वासून, उभा आहे, वेलीच, त्याला, पाय बंद, न, घातल्यास, विपरीद, परिडाम, जाल्या शिवाय, रहाणार नाही,  भारताची 31 मार्च, एकोणिशे 55 परियंत, लोक संख्या 44 कोटी होती, एवडी लोक संख्या, असन्याची मुख्य 3 कारणे आहेद,  वाडते, जन्म प्रमाण, घडते, मुरुत्यू प्रमाण, व, अशिक्षित पड़ा,</t>
-        </is>
-      </c>
       <c r="V26" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन साठ शब्द प्रतिमिनिट ट्रायल पॅसेज सरावाचा उतारा रेडी स्टार्ट महाशय आज जगात लोकसंख्या वाढीचा प्रश्न तोंड वासून उभा आहे वेळीच त्याला पायबंद न घातल्यास विपरीत परिणाम झाल्याशिवाय राहणार नाही भारताची एकतीस मार्च एकोणीशे पंच्याऐंशी पर्यंत लोकसंख्या चौऱतर कोटी होती एवढी लोकसंखण्याची मुख्य त कारणे आहेत वाढते जन्मप्रमाण घटते मृत्यू प्रमाण व अशिक्षित पणा</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2896,7 +3289,7 @@
       <c r="P27" s="2" t="n"/>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>मराठी लगुलेखन आइशी शब्द प्रतिमिनेट पैसेज ए रेडी स्टार्ड परिछेत कोन त्याही देशाचे नागरीक हेच त्या देशाची संपत्ती अस्तार जर देशाचे नागरीक अदर्ष मेहनती आनी सज्जन अस्तील तरस देश प्रगती करतो  एक अदर्ष नागरीक सर्वात अधी एक अदर्ष व्यक्ती अस्तो तो निहमी देशाचा आनी समाजाचा प्रगती साथी कारियर अस्तो  असा व्यक्ती अपल्या नियमांचे काटेकोर पने पालन करतो  आपल्या भारत देशाथ अनेक प्रसिद्ध असे अदर्ष नागरीक हून गेले अहे परिछेत अदर्ष नागरीकाचे अनेक गुन अस्तात  एक अदर्ष नागरीक इमांदार करतव्य निस्ठ आनी सत्यमार्गावर चालनारा अस्तो  तो अपल्या देशाची संस्कृती इतिहास आनी भुमिशी प्रेम करतो  अदर्ष नागरीकाचा मनात देश प्रेम भरलेले अस्ते  तो देशा विशई आपल्या करतव्य ना पुरेपूर बजावतो  आनी निहमी आपल्या करतव्या प्रती जागरूक अस्तो  असा नागरीक वेव प्रसंगी देशा साथी आपले प्रान देन्या सही तयार अस्तो  एक सांगला नागरीक स्वच्छेने नियमांचे पालन करतो  तो राष्ट्राचा उन्नती साथी सकरात्मक योगदान देतो  अदर्ष नागरीक राष्ट्र प्रगतीचा कार्यक्रमात उत्साहाने सामिल होतो  तो समाजाचा अदर्ष मुल्यान्ना सन्मान देतो  आनी समाजात असलेल्या कूरिती समाप्त करन्या साथी लोकान मधे जागरूकता निर्मान करतो  अदर्ष नागरीका चे संपूर्ण जिवन समाजा साथी आनी देशा साथी अरपीत अस्ते  परंतु दुसरी कडे काही असे ही नागरीक अस्तात जे स्वतहाचा स्वार्था साथी देश आनी समाजाचा बली देन्या साथी देखेल मागे पुडे पहात नाही  आज अपल्या समाजात असे अनेक लोक आहेत, जे धोके बाजी करून देशाला नुकसान पोचवतात, हे लोक अपल्या देशा साथी हनी कारक असतात,  परिछेत, एक अदर्ष नागरी हाथ देशाची शान असतो, तो सर्वांशी प्रेम करतो, आनी समाजात असलेले वाईट लोकांचे सत्य सर्वांसमोर अनतो,  मनुन अपन सर्वांचे करतव्य आहे की, अपन देशाचे अदर्ष नागरीक बनायला हवे, आनी देशा विशई आपली जबाबदारी समझून देश सेवेचे कारिय करायला हवे,  आपली सम्षूती आनी इतिहास कायव जतन करून थेवावा</t>
+          <t>मराठी लघुलेखन ऐशी शब्द प्रतिमिनेट पसेज हे रेडी स्टार्ट परिच्छद कोणत्याही देशाचे नागरिक हेच त्या देशाची संपत्ती असतात जर देशाचे नागरिक आदर्श मेहनती आणि सज्जन असतील तरच देश प्रगती करतो एक आदर्श नागरिक सर्वात आधी एक आदर्श व्यक्ती असतो तो नेहमी देशाच्या आणि समाजाच्या प्रगतीसाठी कार्यरत असतो असा व्यक्ती आपल्या नियमांचे काटेकोरपणे पालन करतो आपल्या भारत देशात अनेक प्रसिद्ध असे आदर्श नागरिक होऊन गेले आहेत परिछद आदर्श नागरिकाचे अनेक गुण असतात एक आदर्श नागरिक इमानदार कर्तव्यनिष्ठ आणि सत्य मार्गावर चालणारा असतो तो आपल्या देशाची संस्कृती इतिहास आणि भूमीशी प्रेम करतो आदर्श नागरिकाच्या मनात देशप्रेम भरलेले असते तो देशाविषयी आपल्या कर्तव्यांना पुरेपूर बजावतो आणि नेहमी आपल्या कर्तव्याप्रती जागरूक असतो असा नागरिक वेळ प्रसंगी देशासाठी आपले प्राण देण्यासही तयार असतो एक चांगला नागरिक स्वच्छेने नियमांचे पालन करतो तो राष्ट्राच्या उन्नतीसाठी सकारात्मक योगदान देतो आदर्श नागरिक राष्ट्र प्रगतीच्या कार्यक्रमात उत्हाने सामील होतो तो समाजाच्या आदर्श मूल्याना सन्मान देतो आणि समाजात असलेल्या कुरीती समाप्त करण्यासाठी लोकांमध्ये जागरूकता निर्माण करतो आदर्श नागरिकाचे संपूर्ण जीवन समाजासाठी आणि देशासाठी अर्पित असते परंतु दुसरीकडे काही असे ह नागरिक असतात जे स्वतःच्या स्वार्थासाठी देश आणि समाजाचा बळी देण्यासाठी देखील मागे पुढे पाहत नाही आज आपल्या समाजात असे अनेक लोक आहेत जे धोकेबाजी करून देशाला नुकसान पोहचवतात हे लोक आपल्या देशासाठी हानिकारक असतात परिछद एक आदर्श नागरिक हाच देशाची शण असतो तो सर्वांशी प्रेम करतो आणि समाजात असलेले वाईट लोकांचे सत्य सर्वां समोर आणतो म्हणून आपण सर्वांचे कर्तव्य आहे की आपण देशाचे आदर्श नागरिक बनायला हवे आणि देशाविषयी आपली जबाबदारी समजून देश सेवेचे कार्य करायला हवे आपली संस्कृती आणि इतिहास कायम जतन करून ठेवावा</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -2906,22 +3299,37 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन अईशी शब्द प्रतिमिनेट पैसेज बी रेडी स्टार्ट परिछेद स्त्री पुरूष समानता महंजे स्त्री आनी पुरूष यान्ना समान हक्क संधी आनी आदर मिलवून देन्याचा मुलुबूत विचार होई  एक सुद्रूड प्रगत आनी सशक्त समाज निर्मान करन्या साथी स्त्री पुरूष समानता ही आत्यावश्यक आहे परंतु आजही अनेक समाजात लिंग भिताचा प्रश्न गंभीर आहे  समानते साथी प्रत्यकाने एकत्री तपने प्रयत्न केले पहिजे  स्त्री पुरूष समानता ही आदुनेक समाजाची अत्यांत महत्वाची गरच आहे  समानता महंजे स्त्री आने पुरूषान्ना समान हक संधी आने आदर मिलने परंतु आपल्या समाजात अनेक स्यतकान पासून स्त्रीयां सा दर्जा दुयम समजला जातो  सिक्षन नोकरी संपत्तीवर हक आने सामाजीत अधिकार या बाबतीत स्त्रीयांना पुरूषांचा तुलनेत कमी मानले गेले आहे  समाजात प्रगती घडवन्या साथी स्त्री पुरूष समानता अत्यावश्यक आहे  स्त्री ही केवल कुटुमबाची जबाबदारी अपार पाड़नारी नसून ती समाजाचा प्रते क्षेत्रात योगदान देवु शक्ते  शिक्षन, विद्न्यान, तंत्रद्न्यान, राजकारन, क्रिडा, अनिकला, अशा विवीद क्षेत्रान, स्त्री या चमकत आहे  परंतु त्यानना खर्या अर्थाने समान तेचा अनुबव देन्या साथी मानसी कतेत बदल होने गर्जेचे आहे  रिछेत समाजात समान तेची भावना रुजवन्या साथी स्त्री पुरुष दोगान नीही एक मेकान्ना आदराने वागवाईला हवे  शिक्षन आने जनजागरुती चा माध्यमातून मुलानवर लहान पना पासून समान तेचे संस्कार होने महत्वाचे आहे  घरकाम मुलांची जबाबदारी आनी निर्ने भेन्याचा प्रक्रियेद दोगानचा समान सहभाग असायला हवा  स्त्री पुरुष समानता ही केवल महिलांचा प्रश्ण नाही  ती संपुर्ण समाजाचा प्रगती साथे अवश्यक आहे  समान तेचा मारगाने अपन अधेक न्याईय सू संस्क्रूत आनी शांततामय समाज निर्मान करू शक्तो  स्त्री आनी पुरुष एकत्र हतात हात घालून चालल्यासच एक सशक्त आनी सुन्दर समाज घडेल  परिछेत स्त्री आनी पुरुष यानना समान हक्क अधिकार आनी जबाबदार्या मिलाव्याद यालाच समानता महनताद  यामदे शिक्षन, रोजगार, कुटुम्ब, राजकारन इत्या दिनचा समावेश होतो  समानतेचा अर्थ, समानतेचा आधारावर समाज घडवने आहे  समानतेचा डाद मिलावगार आने चान्सार आना जबएपब यावर्पrर के लिक्षन, रर्ड़ारâte, कि मैंप्ता आन इन आपई यावर्पब, या यावर्फ, या यावर्वर्ण</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन ऐंशी शब्द प्रतिमिनेट पॅसेज बी रेडी स्टार परिच्छेद स्त्री पुरुष समानता म्हणजे स्त्री आणि पुरुष यांना समान हक्क संधी आणि आदर मिळवून देण्याचा मूलभूत विचार होय एक सुदृढ प्रगत आणि सशक्त समाज निर्माण करण्यासाठी स्त्री पुरुष समानता ही अत्यावश्यक आहे परंतु आजही अनेक समाजात लिंग भिदाचा प्रश्न गंभीर आहे समानतेसाठी प्रत्येकाने एकत्रितपणे प्रयत्न केले पाहिजे स्त्री पुरुष समानता ही आधुनिक समाजाची अत्यंत महत्त्वाची गरज आहे समानता म्हणजे स्त्री आणि पुरुषांना समान हक्क संधी आणि आदर मिळणे परंतु आपल्या समाजात अनेक शतकांपासून स्त्रियांचा दर्जा दुयम समजला जातो शिक्षण नोकरी संपत्तीवर हक्क आणि सामाजिक अधिकार या बाबतीत स्त्रियाना पुरुषांच्या तुलनेत कमी मानले गेले आहे समाजात प्रगती घडवण्यासाठी स्त्री पुरुष समानता अत्यावश्यक आहे स्त्री ही केवळ कुटुंबाची जबाबदारी अार पाडणारी नसून ती समाजाच्या प्रत्येक क्षेत्रात योगदान देऊ शकते शिक्षण विज्ञान तंत्रज्ञान राजकारण क्रीडा आणि कला अशा विविध क्षेत्र स्त्रिया चमकत आहेत परंतु त्यांना खऱ्या अर्थाने समानतेचा अनुभव देण्यासाठी मानसिकतेत बदल होणे गरजेचे आहे परिच्छद समाजात समानतेची भावना रुजवण्यासाठी स्त्री पुरुष दोघांनीही एकमेकांना आदराने वागवायला हवे शिक्षण आणि जनजागृतीच्या माध्यमातून मुलावर लहानपणापासून समानतेचे संस्कार होणे महत्वाचे आहे घरकाम मुलांची जबाबदारी आणि निर्णय घेण्याच्या प्रक्रियेत दोघांचा समान सहभाग असायला हवा स्त्री पुरुष समानता हि केवळ महिलांचा प्रश्न नाही ती संपूर्ण समाजाच्या प्रगतीसाठी आवश्यक आहे समानतेच्या मार्गानेच आपण अधिक न्याय सुसंस्कृत आणि शांततामय समाज निर्माण करू शकतो स्त्री आणि पुरुष एकत्र हातात हात घालून चालल्यासच एक सशक्त आणि सुंदर समाज घडेल परिच्छद स्त्री आणि पुरुष यांना समान हक्क अधिकार आणि जबाबदाऱ्या मिळाव्यात यालाच समानता म्हणतात यामध्ये शिक्षण रोजगार कुटुंब राजकारण इत्यादीचा समावेश होतो समानतेचा अर्थ समानतेच्या आधारावर समाज घडवणे आहे</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U27" s="2" t="inlineStr">
-        <is>
-          <t>मराठी लुगुलेखन अइशी शब्द प्रतिमनेट  ट्रायल पैसेज रेडी स्टाट  परिछेद माननिय सदस्यन्नी अपला प्रस्ताव मांडताना विनानुदान तत्वावर चालनार्या शालांचा बाबतीत  जा सेवाशर्ती वह नियम आहेत त्या बद्दल सहनुबुती या ठिकानी व्यकत केली आहे  जा शाला अनुदान तत्वावर चालतात त्यातील शिक्षकान्ना सेवाशर्ती चे जे नियम लागू आहेत  तेच विना अनुदान तत्वावर चालनार्या शिक्षकान नाही लागू केलेले आहेत आनी कर्ण्यात एतील वेतनाचा प्रश्नांचा थोडासा विचार करावा लागेल कारण या शालानना शासन अनुदान देत नाही</t>
-        </is>
-      </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लुघुलेखन ऐंशी शब्द प्रतिमिनेिट ट्रायल पॅसेज रेडी स्टार्ट परिच्छद माननीय सदस्यांनी आपला प्रस्ताव मांडताना विनानुदान तत्त्वावर चालणाऱ्या शाळांच्या बाबतीत ज्या सेवा शर्ती व नियम आहेत त्याबद्दल सहानुभूती या ठिकाणी व्यक्त केली आहे ज्या शाळा अनुदानतत्वावर चालतात त्यातील शिक्षकांना सेवा शर्तीचे जे नियम लागू आहेत तेच विनाअनुदान तत्त्वावर चालणाऱ्या शिक्षकांनाही लागू केलेले आहेत आणि करण्यात येतील वेतनाच्या प्रश्नांचा थोडासा विचार करावा लागेल कारण या शाळांना शासन अनुदान देत नाही</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -2988,7 +3396,7 @@
       <c r="P28" s="2" t="n"/>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>मराथी लोगुलेखन आइशी शब्द प्रतिमिनेट  पैसेज ए, रिडी, स्टार्ट  स्री पुरुष हो परिच्छेत आपल्या कम्पनीचा सर्वसाधरन सभेत  आपले स्वागत करताना मला अतिशे अनंद होत आहे  हिशोब तपासलेल्या हिशोब आचे निवेदन अपनास मिलाले असेल  आनी संचा लकांचा अहवाल अपन वाचला असेलच असे मी आपल्या परवानगिने गुरुहीत धरून चालतो  चालू साली मुख्य तहा कच्चा मालाचा वाधनार्या किम्ती कामगाराचे सुधारीत वेतन  आनी इतर खर्चा मदे भरम साथ वाड या कारनामुले कंपनीचा नफ्यावर परिनाम जाला आहे  उद्योक धंद्यातील वाधनारी तिवरस परधा व बाजार पेठेत दिवसेन दिवस उत्पादक वस्तु साथी जाहराती साथी खर्च करन्याची गरज निर्मान जाली आहे  परिछ संचालक मंडलाने वेडो वेडी बदल लेल्या दोरना मुलेच वाटा घाटी मदे उड़ा तान न करता काम गारांचा होनार्या संपास वेडीच उपाय योजना केल्या मुले उत्पादनात वाड जहली  कम्पनीने आता पावेतो पुषकलच प्रगती किली आहे  कम्पनीने आखलेल्या अउद्योगीक धुरनांचा अम्मल बजावनी साथी जलत गतीने वास्तव वादी दुरुष्टिकोन स्विकार्न्यात अला ही अत्यंत अनंदाची गोष्ट आहे  मागिल साली कम्पनीची परिस्थिती महनावी तितकी समाधान कारक नवती  कच्चा मालाचा किमती विजेचे वाड ते दर कामकाजाचा खर्च वगसारा यांची तर्तूद केल्यानंतर कम्पनीला जास्त नफा मिलाला नाही  परंतू कम्पनीची परिस्थिती समाधान कारक आहे हे मान्यकराल अशी मी आशा करतो  परिछेत मागिल साली कम्पनीचा उतकर्षा साथी ची महत्वाची पावुले अपन उचललीत व जा विवीद योजना अखल्या त्या मुले कारकान्याचा उत्पादनात वाड जाली  व एकंदर कम्पनीची परिस्थिती सर्व बाजुनी सुधारली अपन केलेल्या उपाई योजने मुले आपल्या कम्पनीने आता पावेतो लक्षनिय प्रगती केली आहे  मालाची किम्मत व वाडिव मागने संबंदीचा कम्पनीने स्विकार लेल्या दोरना बाबत्चा दुरुष्टि कोन संचालक मंडला कडून तसेज कामगार प्रतिनी दीकडून स्विकारन्यात आला  ही कम्पनीचा दुरुष्टिने व आउद्योगेक शांतता टिकवन्या साथी अत्यांत अनंदाची गोष्ट आहे  परिचे आपनास कल्पना असेलच की कम्पनीने गेल्या वर्षा पासून काटे कोर पने व्यवहरा मदेल उदले पनाला प्रिनाम कारक आला घातला आहे</t>
+          <t>मराठी लघुलेखन ऐंशी शब्द प्रतिमिनेिट पॅसेज ए रेडी स्टार्ट श्री पुरुष हो परिच्छद आपल्या कंपनीच्या सर्वसाधारण सभेत आपले स्वागत करताना मला अतिशय आनंद होत आहे हिशोब तपासलेल्या हिशोबाचे निवेदन आपणास मिळाले असेल आणि संचालकांचा अहवाल आपण वाचला असेलच असे मी आपल्या परवानगीने गृहीत धरून चालतो चालू साली मुख्यत कच्च्या मालाच्या वाढणाऱ्या किंमती कामगाराचे सुधारित वेतन आणि इतर खर्चामध्ये भरमसाठ वाढ या कारणामुळे कंपनीच्या नफ्यावर परिणाम झाला आहे उद्योगधंद्यातील वाढणारी तीव्र स्पर्धा व बाजारपेठेत दिवसेंदिवस उत्पादक वस्तूसाठी जाहिरातीसाठी खर्च करण्याची गरज निर्माण झाली आहे परिच्छेद संचालक मंडळाने वेळोवेळी बदललेल्या धोरणामुळेच वाटाघाटीमध्ये ओढा ताण न करता कामगारांच्या होणाऱ्या संपास वेळीच उपाययोजना केल्यामुळे उत्पादनात वाढ झाली कंपनीने आता पावेतो पुष्कळच प्रगती केली आहे कंपनीने आखलेल्या औद्योगिक धोरणांच्या अंमलबजावणीसाठी जलदगतीने वास्तववादी दृष्टकोन स्वीकारण्यात आला ही अत्यंत आनंदाची गोष्ट आहे मागील साली कंपनीची परिस्थिती म्हणावी तितकी समाधानकारक नव्हती कच्च्या मालाच्या किंमती विजेचे वाढते दर कामकाजाचा खर्च व घसारा यांची तरतूद केल्यानंतर कंपनीला जास्त नफा मिळाला नाही परंतु कंपनीची परिस्थिती समाधानकारक आहे हे मान्य कराल अशी मी आशा करतो परिच्छेद मागील साली कंपनीच्या उत्कर्षासाठीची महत्त्वाची पावले आपण उचललीत व ज्या विविध योजना आखल्या त्यामुळे कारखान्याच्या उत्पादनात वाढ झाली व एकंदर कंपनीची परिस्थिती सर्व बाजूनी सुधारली आपण केलेल्या उपाययोजनेमुळे आपल्या कंपनीने आता पावेतो लक्षणीय प्रगती केली आहे मालाची किंमत व वाढीव मागणी संबंधीच्या कंपनीने स्वीकारलेल्या धोरणाबाबतचा दृष्टकोन संचालक मंडळाकडून तसेच कामगार प्रतिनिधीकडून स्वीकारण्यात आला ही कंपनीच्या दृष्टीने व औद्योगिक शांतता टिकवण्यासाठी अत्यंत आनंदाची गोष्ट आहे परिच्छद आपणास कल्पना असेलच की कंपनीने गेल्या वर्षापासून काटेकोरपणे व्यवहारामधील उदळेपणाला परिणामकारक आळा घातला आहे</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
@@ -2998,22 +3406,37 @@
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>मराथी लुगुलेखन आइशी शब्द प्रतिमनेट, पैसेज बी, रेडी, स्टार्ट  सन्माननिय सहकारी सभासद बंदू भगिनेनो  अपल्या सहकारी साखर कार्खाना सोलापूर लिमेटेड  याचा वार्षिक सर्वसादरन सभेत अपना सर्वांचे हार्दीक स्वागत करताना मला अनंद होत आहे  परिछेत अपल्या साखर कार्खन्याचा मार्च अखेरचा वर्षाचा वार्षिक अहवाल अपना कडे आहे  तो अपन वाचला असेलच असे में अपल्या परवानगी ने गुरुहीत धरून चालतो  तसेच वार्शिक अहवाल ताले बंद व नफा तोटा पत्रके संचालक मंड़ाचा वतिने अपनास साधर करताना मला अनंद होत आहे  परिछेच अपना सर्वनना कल्पना असेलच की हा साकर कार्खना सहकार तत्वावर लहनातल्या लहान शेद कर्याचा हिता साथी स्थापन कर्ण्याद अलेला आहे  तसेच समाजातील सर्व धरातील सामान्य मानसाचे जीवन सुजलाम सुफलाम वावे या साथी आपल्या कार्खन्याने प्रयत्नांची पराकास्टा केली आहे  तसेच कार्खना निर्निरालया माध्यमातुन सर्व धरातील लोकांचे जीवन सम्रुद्ध वावे प्रगतिशील वावे व कृषी आउध्योगीक नव समाज निर्मान वावा व सहकारी चल्वल भक्कम शक्तिशाली वावी व ग्रामिन जनतेचा उन्नतीचे व दुर्बल  समाज परिवर्तनाचे कार्य कर्ण्या साथी स्थापन जालेला आहे  परिछेत भारताचे सर्वांचे लाड़के पंत प्रधान याननी अलपा वधितत सर्व थरातील जनतेचा तसेच शेतकरी मजुर वर्ग, कामगार वर्ग, भुमी हीन शेतकरी, मागास वर्गिय यांचा आशा अकांग्षांची पुरती कर्न्यासाठी सतत प्रयतनशील आहेत  अउद्योगिक, सामाजिक, शैक्षनिक, शिती विशयक कार्यक्रमानना चालना दिली आहे असे नमूद कर्न्यास अभिमान वाटतो परिछेत अपल्या कार्खन्यातून पाजर तलाव उपसा जलसिंचन योजना इत्यादी साथी सरकार कडे मंजुरी साथी व ग्रामीन यो  विद्यूत पुरवठा, पानी पुरवठा, ग्रामीन रस्ते, सुधारना, कुकुट पालन, व शितीवर अवलंबुन असनारे लगु उद्योग व त्यांचा विकास, इत्यादी विवीद, कल्यानकारी, योजनान द्वारे, परिश्रमाची पराकाष्ठा करीत आहेत।  काही तालुक्यातील गावांचा नवैनेच समावेश कर्ण्यात आला आहे। अपल्या कार्खण्याची व्याप्ती वाधत जाईल या पद्धतीची योजना आखली गेली आहे।</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन ऐंशी शब्द प्रतिमनेट पॅसेज बी रेडी स्टार्ट सन्माननीय सहकारी सभासद बंधू भगिनींनो आपल्या सहकारी साखर कारखाना सोलापूर लिमिटेड याचा वार्षिक सर्वसाधारण सभेत आपणा सर्वांचे हार्दिक स्वागत करताना मला आनंद होत आहे परिच्छेद आपल्या साखर कारखान्याचा मार्च अखेरच्या वर्षाचा वार्षिक अहवाल आपणाकडे आहे तो आपण वाचला असेलच असे मी आपल्या परवानगीने गृहीत धरून चालतो तसेच वार्षिक अहवाल ताळेबंद व नफ तोटा पत्रके संचालक मंडळाच्या वतीने आपणास सादर करताना मला आनंद होत आहे परिच्छद आपणा सर्वांना कल्पना असेलच की हा साखर कारखाना सहकार तत्वावर लहानातल्या लहान शेतकऱ्याच्या हितासाठी स्थापन करण्यात आलेला आहे तसेच समाजातील सर्व थरातील सामान्य माणसाचे जीवन सुजलाम सुफलाम व्हावे यासाठी आपल्या कारखान्याने प्रयत्नांची पराकाष्ठा केली आहे तसेच कारखाना निरनिराळ्या माध्यमातून सर्व थरातील लोकांचे जीवन समृद्ध व्हावे प्रगतिशील व्हावे व कृषी औद्योगिक नव समाज निर्माण व्हावा व सहकारी चळवळ भक्कम शक्तिशाली व्हावी व ग्रामीण जनतेच्या उन्नतीचे व दुर्बल घटकाच्या कल्याणाचे समाज परिवर्तनाचे कार्य करण्यासाठी स्थापन झालेला आहे परिच्छेद भारताचे सर्वांचे लाडके पंतप्रधान यांनी अल्पावधीतच सर्व थरातील जनतेच्या तसेच शेतकरी मजूरवर्ग कामगार वर्ग भूमिहीन शेतकरी मागासवर्गीय यांच्या आशा आकांक्षांची पूर्ती करण्यासाठी सतत प्रयत्नशील आहेत तसेच महाराष्ट्रातील औद्योगिक सामाजिक शैक्षणिक शेतीविषयक कार्यक्रमांना चालना दिली आहे असे नमूद करण्यास अभिमान वाटतो परिच्छेद आपल्या कारखान्यातून पाझर तलाव उपसा जलसिंचन योजना इत्यादीसाठी सरकारकडे मंजुरीसाठी व ग्रामीण युवकांसाठी स्वयंरोजगार योजना विद्युत पुरवठा पाणी पुरवठा ग्रामीण रस्ते सुधारणा कुक्कुटपालन व शेतीवर अवलंबून असणारे लघुउद्योग व त्यांचा विकास इत्यादी विविध कल्याणकारी योजनाद्वारे परिश्रमाची पराकाष्ठा करीत आहेत परिच्छेद आपल्या कारखान्याच्या कार्यक्षेत्रात मागच्या वर्षी सोलापूर जिल्ह्यातील काही तालुक्यातील गावांचा नव्यानेच समावेश करण्यात आला आहे आपल्या कारखान्याची व्याप्ती वाढत जाईल या पद्धतीची योजना आखली गेली आहे</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U28" s="2" t="inlineStr">
-        <is>
-          <t>मराठी लुगुलेखन अइशी शब्द प्रतिमनेट  ट्रायल पैसेज रेडी स्टाट  परिछेद माननिय सदस्यन्नी अपला प्रस्ताव मांडताना विनानुदान तत्वावर चालनार्या शालांचा बाबतीत  जा सेवाशर्ती व नियम आहेत त्या बद्दल सहनु भूती या ठिकानी व्यक्त केली आहे  जा शाला अनुदान तत्वावर चालतात त्यातील शिक्षकानना सेवाशर्ती चे जे नियम लागु आहेत तेच विना अनुदान तत्वावर चालनार्या शिक्षकानना ही  लागू केलेले आहेत, आनी कर्ण्यात एतील, वेतनाचा प्रश्नांचा थोडासा विचार करावा लागेल, कारण या शालानना शासन अनुदान देत नाही.</t>
-        </is>
-      </c>
       <c r="V28" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लुघुलेखन ऐंशी शब्द प्रतिमिनेिट ट्रायल पॅसेज रेडी स्टार्ट परिच्छद माननीय सदस्यांनी आपला प्रस्ताव मांडताना विनानुदान तत्त्वावर चालणाऱ्या शाळांच्या बाबतीत ज्या सेवा शर्ती व नियम आहेत त्याबद्दल सहानुभूती या ठिकाणी व्यक्त केली आहे ज्या शाळा अनुदानतत्वावर चालतात त्यातील शिक्षकांना सेवा शर्तीचे जे नियम लागू आहेत तेच विनाअनुदान तत्त्वावर चालणाऱ्या शिक्षकांनाही लागू केलेले आहेत आणि करण्यात येतील वेतनाच्या प्रश्नांचा थोडासा विचार करावा लागेल कारण या शाळांना शासन अनुदान देत नाही</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3503,7 @@
       <c r="P29" s="2" t="n"/>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>मराठी लगुलेखन शंभर शब्द प्रती मिनिट  पैसेज ए  रेडी स्टाट पैरा  स्त्री पुरुष समानता मनजे समाजात स्त्री आणी पुरुषाना समान हक्क संधी आणी स्तन्मान मिलने  या समानतेचा विचार शिक्षन, नोकरी, कउटुम्बिक जबाबदार्या, राजकारण, तसेच समाजिक व सांस्कृतिक शेत्रान मदे होतो  समानतेचे तत्व हे मानवतेचा मुलभूत तत्वान पैकी एक आहे  प्राचिन कालात स्त्रियाना समाजात उच्च स्थान होते, पन कालांतराने सामाजिक, सांस्कृतिक आणी धार्मिक कार्णान मुले स्त्रियाना दुयम स्थान दिले गेली  शिक्षन, मालमत्ता आणी सार्वजनिक जीवनात सहबाग या बावतीत त्याना मर्यादा घालन्यात आल्या  पैरा आजचा कालात अनेक देशान मदे स्त्री पुरुष समानते साथी मोठी पावले उचलली जात आहेत  शिक्षन क्षेत्रात स्त्रीया पुढे येत आहेत नोकरीचा विविदक्षेत्रान मदे तैंचा सहबाग वाढ़त आहे आली राजकार्णात ही तैंची भुमिका महत्वाची थरत आहे  परंतु अजु नही अनेक ठिकानी समानते चा अभाव दिसुन येतो शिक्षन हे समानते चा दिशेने पहिले पावल आहे  मुल्गा आणी मुल्गी दोगानाई समान शिक्षनाचा संधी उपलब्द करुन दिल्या तरत खर्या अर्थाने समाच प्रगत होईल  शिक्षना मुले महिलाना स्वाव लंबनाची जानीव होते आणी स्वताचा निर्णयान मदे सहबाग गेन्याचा आत्मविश्वास येतो  नोकरीचा ठिकाणी स्त्रियाना समान वेतन, समान संधी आणी समान वागणुक मिलावी या साथी प्रयत्न केले जात आहेत  पण अने ठिकाणी महिलाना दुयम वागणुक दिली जाती त्याना बढती नेत्रुत्वाची संधी या मदे मागे ठेवले जाती  स्त्री सक्षमी करण मनजे महिलाना आर्थिक, सैक्षणिक आणी सामाजिक दुरुष्ट्या सक्षम करणे  समान तेचा विचार प्रत्यक्षात आणन्या साथी महिलाना संधी उपलब्ध करुंदिली पाईजी  स्त्रीयाना स्वावलंबी बनावने हे केवल त्यांचे हक्क नसून समाजाचा प्रगती साथी ही आवश्यक आहे  शिक्षण लाहान पणापासून मुला मुली ना समान तेचे शिक्षण दिले पाईजे  कुटुमबातिल योगदाना मधे कुटुमबात स्त्री आणि पूरुष दोगानाई समान वाग्णुक देने आवश्यक आहे  सामाजिक मानसिक ते मधे समाजातिल रुडी आणि परंपरा बदलन्या साथी सर्वानी पुढाकार घेतला पाईजी  राजकी यह सहबाग महिलाना राजकारनात समान प्रती निधीत्व देने आवश्यक आहे  अलीकडिल कालात समानते साथी अनेक सकारात्मक बदल जाले आहेत  महिलानी शिक्षन, खेल, उद्योजकता आणि राजकारनात आपले स्थान निर्मान केली आहे  परंतु अजु नहीं ग्रामेन भागात आणिकाई क्षेत्रान मदे समानतेचा बाबतीत मोठ्या सुधार्णा आवश्यक आहेत।  क्षेत्रान आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश्यक आवश</t>
+          <t>मराठी लघुलेखन शंभर शब्द प्रतिमिनिट पॅसेज ए रेडी स्टार्ट प्यारा स्त्री पुरुष समानता म्हणजे समाजात स्त्री आणि पुरुषांना समान हक्क संधी आणि सन्मान मिळणे या समानतेचा विचार शिक्षण नोकरी कौटुंबिक जबाबदाऱ्या राजकारण तसेच सामाजिक व सांस्कृतिक क्षेत्रांमध्ये होतो समानतेचे तत्त्व हे मानवतेच्या मुूलभूत तत्वांपैकी एक आहे प्राचीन काळात स्त्रियांना समाजात उच्च स्थान होते पण कालांतराने सामाजिक सांस्कृतिक आणि धार्मिक कारणांमुळे स्त्रियांना दुयम स्थान दिले गेले शिक्षण मालमत्ता आणि सार्वजनिक जीवनात सहभाग या बाबतीत त्यांना मर्यादा घालण्यात आल्या प्यारा आजच्या काळात अनेक देशांमध्ये स्त्री पुरुष समानतेसाठी मोठी पावले उचलली जात आहेत शिक्षण क्षेत्रात स्त्रिया पुढे येत आहेत नोकरीच्या विविध क्षेत्रांमध्ये त्यांचा सहभाग वाढत आहे आणि राजकारणातही त्यांची भूमिका महत्त्वाची ठरत आहे परंतु अजूनही अनेक ठिकाणी समानतेचा अभाव दिसून येतो शिक्षण हे समानतेच्या दिशेने पहिले पाऊल आहे मुलगा आणि मुलगी दोघांनाही समान शिक्षणाच्या संधी उपलब्ध करून दिल्या तरच खऱ्या अर्थाने समाज प्रगत होईल शिक्षणामुळे महिलांना स्वावलंबनाची जाणीव होते आणि स्वतःच्या निर्णयामध्ये सहभाग घेण्याचा आत्मविश्वास येतो नोकरीच्या ठिकाणी स्त्रियांना समान वेतन समान संधी आणि समान वागणूक मिळावी यासाठी प्रयत्न केले जात आहेत पण अनेक ठिकाणी महिलांना दयम वागणूक दिली जाते त्यांना बढती नेतृत्वाची संधी यामध्ये मागे ठेवले जाते स्त्री सक्षमीकरण म्हणजे महिलांना आर्थिक शैक्षणिक आणि सामाजिक दृष्ट्या सक्षम करणे समानतेचा विचार प्रत्यक्षात आणण्यासाठी महिलांना संधी उपलब्ध करून दिली पाहिजे स्त्रियाना स्वावलंबी बनवणे हे केवळ त्यांचे हक्क नसून समाजाच्या प्रगतीसाठी ह आवश्यक आहे शिक्षण लहानपणापासून मुला मुलींना समानतेचे शिक्षण दिले पाहिजे कुटुंबातील योगदानामध्ये कुटुंबात स्त्री आणि पुरुष दोघांनाही समान वागणूक देणे आवश्यक आहे सामाजिक मानसिकतेमध्ये समाजातील रूढी आणि परंपरा बदलण्यासाठी सर्वांनी पुढाकार घेतला पाहिजे राजकीय सहभाग महिलांना राजकारणात समान प्रतिनिधित्व देणे आवश्यक आहे अलीकडील काळात समानतेसाठी अनेक सकारात्मक बदल झाले आहेत महिलांनी शिक्षण खेळ उद्योजकता आणि राजकारणात आपले स्थान निर्माण केले आहे परंतु अजूनही ग्रामीण भागात आणि काही क्षेत्रांमध्ये समानतेच्या बाबतीत मोठ्या सुधारणा आवश्यक आहेत समानतेच्या मार्गावर अद्याप अनेक अडथळे आहेत जागतिक स्तरावरील वेतन विषमता अजूनही मोठी समस्या आहे गृहिणीना कुटुंबात योग्य मान्यता दिली जात नाही</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -3090,22 +3513,37 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>मराठी लगुलेखन, शंबर शब्द प्रती मिनिट, पैसेच, बी, रेडी, स्टार्ट, पैरा, जाडे ही प्रुथ्वीवरील परियावर्णाचा महत्वाचा घटक आहेत,  मानवाचे अस्तित्व, निसर्गाचा समतोल आणी परियावर्णाचा टिकाव धर्नेची क्षमता यामदे जाडांचे योगदान अमुल्य आहे, पन दुर्दैवाने मानवाने प्रगतीचा नावा खाली जंगल तोड आणी परियावर्णाचा रास केल्या मुले प्रुथ्  ती कालाची गरज बनली आहे, जाडे ही प्रुथ्वी वरिल परियावर्णाचा महत्वाचा घटक आहेत, ती फक्त ओक्सिजनचा पुरवठा करत नाहेत, तर जीवस रुष्टीचे संतूलन राखनयाचे काम करतात, जाडान मुले आपन शुद्ध हवा, अन्न आणी नि�  जाडान मुले परजन्यमान वाडते, आणी भूजल, पातली, टिकून, राहते, ती जमिनीचा पोत सुधारतात, आणी जैव विवीध तेला आश्रय देतात, अनेक प्राणी, पक्षी, आणी किटकान साथी जाडे ही निवासाची जागा असतात, जाडे वायु प्रदु  आर्थिक आणी सांस्कृतिक जीवनात ही जाडांचे महत्व खूप आहे, आउशदे, इमारती साथी लाखूड आणी विवीध वस्त्र निर्मिती साथी जाडे उपयुक्त ठारतात, धार्मिक विधिन मदे ही जाडाना महत्वाचे स्थान आहे, मात्र अलिकडचा कालात �  आर्णी य संतूलन बिघडत आहे, आनी हवामान बदलाचा धोका वाढत आहे, यावर उपाय मणून प्रत्यकाने जाडे लावुन ती जगवनेची जबाबदारी स्विकारली पाही जाडांचे महत्व आपल्या जिवनात अमुल्य आहे, त्या मुले आपन जाडे लावा  पुढे सरसावले पाही जे, आजचा आधुनेक युगात जाडांचे स्थान अधीक महत्वाचे आणी आवशक जाले आहे, प्रगती चा नावाखाली वाढते शहरी करण, आउद्योगी करण, आणी बे सुमार जंगल तोड या मुले जाडांची संख्या जापाट आने �  असुन, प्रुथ्वीवर जागतीक तापमान वाढ, परजन्यमान कमी होने, आणी जैव विवीध तेचा रास या सार्खी संकटे निर्मान जाली आहेत, पैरा जाडे निसर्गाचा समतोल राखन्याचे काम करतात, ती जमीनीचा पोत टिकवुन थेवतात, भूजल साठा  आणी वायू प्रदूशन कमी करतात, मात्र आज जाडान वरिल मानवाचा अव लंबित्व खूप जास्त असुन, तैंची तोड बे सुमार सुरू आहे, या परिस्तितीत जाडान चे संवर्धन करून संख्या वाडवने, ही कालाची गर जाहे, जाडे लावा जाडे जग</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन शंभर शब्द प्रतिमनिट पॅसेज बी रेडी स्टार्ट पॅरा झाडे ही पृथ्वीवरील पर्यावरणाचा महत्त्वाचा घटक आहेत मानवाचे अस्तित्व निसर्गाचा समतोल आणि पर्यावरणाचा टिकाव धरण्याची क्षमता यामध्ये झाडांचे योगदान अमूल्य आहे पण दुर्दैवाने मानवाने प्रगतीच्या नावाखाली जंगल तोड आणि पर्यावरणाचा रास केल्यामुळे पृथ्वीवरील सजीवसृष्टी धोक्यात आली आहे अशावेेळी झाडे लावा झाडे जगवा हा संदेश केवळ प्रचाराचा मुद्दा नसून ती काळाची गरज बनली आहे झाडे ही पृथ्वीवरील पर्यावरणाचा महत्वाचा घटक आहेत ती फक्त ऑक्सिजनचा पुरवठा करत नाही तर जीवसृष्टीचे संतुलन राखण्याचे काम करतात झाडांमुळे आपण शुद्ध हवा अन्न आणि निवासस्थान मिळवतो त्याशिवाय झाडे जमिनीचे धूप थांबवतात आणि जलचक्र संतुलित ठेवण्यास मदत करतात झाडांमुळे पर्जन्यमान वाढते आणि भूजल पातळी टिकून राहते ती जमिनीचा पोत सुधारतात आणि जैव विविधतेला आश्रय देतात अनेक प्राणी पक्षी आणि कीटकांसाठी झाडे ही निवासाची जागा असतात झाडे वायू प्रदूषण कमी करून पर्यावरण शुद्ध करतात पॅरा मानवाच्या आर्थिक आणि सांस्कृतिक जीवनातही झाडांचे महत्त्व खूप आहे औषधे इमारतीसाठी लाकूड आणि विविध वस्त्र निर्मितीसाठी झाडे उपयुक्त ठरतात धार्मिक विधीमध्येही झाडांना महत्वाचे स्थान आहे मात्र अलीकडच्या काळात झपाट्याने होत असलेल्या जंगल तोडीमुळे झाडांची संख्या कमी होत आहे यामुळे पर्यावरणीय संतुलन बिघडत आहे आणि हवामान बदलाचा धोका वाढत आहे यावर उपाय म्हणून प्रत्येकाने झाडे लावून ती जगवण्याची जबाबदारी स्वीकारली पाहिजे झाडांचे महत्व आपल्या जीवनात अमूल्य आहे त्यामुळे आपण झाडे लावा झाडे जगवा हा संदेश आचरणात आणून निसर्गाचे रक्षण करण्यासाठी पुढे सरसावले पाहिजे आजच्या आधुनिक युगात झाडांचे स्थान अधिक महत्वाचे आणि आवश्यक झाले आहे प्रगतीच्या नावाखाली वाढते शहरीकरण औद्योगकरण आणि बेसुमार जंगल तोड यामुळे झाडांची संख्या झपाट्याने घटत आहे याचा थेट परिणाम पर्यावरणावर होत असून पृथ्वीवर जागतिक तापमान वाढ पर्जन्यमान कमी होणे आणि जैव विविधतेचा राास यासारखी संकटे निर्माण झाली आहेत पॅरा झाडे निसर्गाचा समतोल राखण्याचे काम करतात ती जमिनीचा पोत टिकवून ठेवतात भूजल साठा वाढवतात आणि वायू प्रदूषण कमी करतात मात्र आज झाडांवरील मानवाचा अवलंबितव खूप जास्त असून त्यांची तोड बसमार सुरू आहे या परिस्थितीत झाडांचे संवर्धन करून संख्या वाढवणे ही काळाची गरज आहे झाडे लावा झाडे जगवा ही चळवळ प्रत्येकाने अंगीकारली पाहि</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U29" s="2" t="inlineStr">
-        <is>
-          <t>मराधी लगुलेखन, शम्भर शब्द प्रती मिनिट, ट्रायल पैसेच, रेडी, स्टांट, पैरा, आमचा राज्याचे अधिक्रूत धोरण समाजवादी आहे,  मनोन समाजवाद हा शब्द आमी हेत्तु पुरसर वापर्तो, परंतु समाजवादा बतल आमी बोलावयास लागले नंतर, काही मानसाना अगदी अउघल्ल्यास अरके वाटू लागले,  त्याना असे वाटू लागले की, हे लोग समाजवादा बतल बोलावयास लागले तर, आमचे सगले संपलेच, आमी मा काई बोलावयाचे,  परंतु मी त्याना सांगु इची तोकी, त्याचा समाजवाद बेगला आहे, आमी जो समाजवाद मानतो तो त्याचा समाजवादास सारखा नही,  ते मंतात त्यांचा समाजवात खास आही, त्यांचा समाजवात त्याना लखलाव हो.</t>
-        </is>
-      </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन शंभर शब्द प्रतिमनिट ट्रायल पॅसेज रेडी स्टार्ट प आमच्या राज्याचे अधिकृत धोरण समाजवादी आहे म्हणून समाजवाद हा शब्द आम्ही हेतूपरसर वापरतो परंतु समाजवादाबद्दल आम्ही बोलावयास लागल्यानंतर काही माणसांना अगदी अवघडल्यासारखे वाटू लागले त्यांना असे वाटू लागले की हे लोक समाजवादाबद्दल बोलावयास लागले तर आमचे सगळे संपलेच आम्ही मग काय बोलावायचे परंतु मीांूो की् ज त्यां सारख नाही ते म्हणतात त्यांचा स खास आहे त्यांचा सना लखलाभ हो</t>
+        </is>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3610,7 @@
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>मराठी लगुलेखन शंबर्शब्द प्रती मिनिट पैसेज ए रेडी स्टार्ट पैरा कोण त्याही देशाचा आर्थिक विकास हा त्या देशा तील नैसर्गेक साधने मनुष्य बल भांडवल वह संघटना काउशल्ड्य यान वर अवलंबुन अस्तु त्याच प्रमाणे  परिस्तितीचा घटकांचा सुधा महत्वाचा भाग अस्तु जेवा आपन भारताचा सामाजिक आर्थिक उनर अचने बदल बोलतो तेमा त्यांचा अर्थ आपल्याला काही विधायक स्वरुपाची उद्धिष्टे साध्य करावयाची आहेत असा अस्तु ते उद्धि�  सहभागाची जानेव निर्मान करने ही आहेत प्यारा सद्या भारताच असलेली तिवर स्वरुपाची बेकारी ही सर्वाना खूप अस्वस्त करनारी समस्या आहे देशात चार कोटी लोक बेकार आहेत असा अंदाज आहे  प्यारा लोकसंखे मदे जपाट्याने हो तसलेली वाड हे बेकारीचे महत्वाचे कारण आहे।  लगु वकुटिर उद्योगाला श्रम प्रधान उत्पादन पधती वर शासनाने भर दिलेला आहे।  अकिती अशिक्षित बेकारांची नोंद करन्यात आली। त्या पैकी किती बेकारांना काम देन्यात आले।  आज परियंत नोंदलेल्या पैकी किती बेकारांना अध्याप काम देने शिल्लक आहे।  या संबंधी माहिती तेनारी जी विवर्ण या विभागात प्राप्त जाली आहेत।  त्यांचे संकलन करून एक सविस्तर टिपणी या विभागात प्राप्त जाली आहेत।  त्यांचे संकलन करून एक सविस्तर टिपणी सोबत जोडली आहे।  आहे ती कुरुपया पहावी या टिपणी वरुन हे दिसुन यहिल की राज्यातिल सर्वप्रकारचा बेकारांचा संखेत प्रत्यक्षात वाड होत असुन सुशिक्षित बेकारांचा संखेत दर वर्षी होनारी वाड तर भयावह मनता यहिल आशा पातलीला यहुन पोचली �  न नोंदले गेलेले बेकार ही मुठा संखेने, असुन बेकारी निवालनेचा प्रिश्ण या राज्याने युद्ध पातली वर हाती घेनेची तातलीची गरच निर्मान झाली आहे, असे या विभागाला वाटते।  या राज्याने जा विवीध विकास योजना, तसेच रोजगार हमी योजना राज्यात हाती घेतलीआ आहेत, त्या मुळे मोठ्या प्रमानावर बेकाराना काम मिलनेची सोय जाली आहेत।</t>
+          <t>मराठी लघुलेखन शंभर शब्द प्रतिमिनिट पॅसेज ए रेडी स्टार्ट परा कोणत्याही देशाचा आर्थिक विकास हा त्या देशातील नैसर्गिक साधने मनुष्यबळ भांडवल व संघटना कौशल्य यांवर अवलंबून असतो त्याचप्रमाणे सामाजिक संस्था सांस्कृतिक दृष्टकोन यांसारख्या आर्थिक परिस्थितीच्या घटकांचा सुद्धा महत्वाचा भाग असतो जेव्हा आपण भारताच्या सामाजिक आर्थिक पुनररचनेबद्दल बोलतो तेव्हा त्यांचा अर्थ आपल्याला काही विधायक स्वरूपाची उद्दिष्टे साध्य करावयाची आहेत असा असतो ते उद्दिष्टे म्हणजे सर्वांना संधी प्राप्त करून देणे दुर्बळ घटकांमध्ये उद्योजकता वाढीला लावणे सहभागाची जाणीव निर्माण करणे ही आहेत परा सध्या भारतात असलेली तीव्र स्वरूपाची बेकारी ही सर्वांना खूप अस्वस्थ करणारी समस्या आहे देशात चार कोटी लोक बेकार आहेत असा अंदाज आहे परा लोकसंख्येमध्ये झपाट्याने होत असलेली वाढ हे बेकारचे महत्वाचे कारण आहे नियोजनात बेकारीच्या समस्येकडे पुरेसे लक्ष दिले जात आहे वास्तविक पहिल्या पंचवार्षिक योजनेच्या सुरवातीपासून बेकारीची समस्या सोडविण्याची गरज शासनाला भासली होती म्हणूनच जेथे शक्य आहे तेथे विशेषत लघु व कुटीर उद्योगाला श्रम प्रधान उपान पद्धतीवर शासनाने भर दिलेला आहे ग्रमीण बेकारीच्या क्षेत्रात आवर्षण प्रवण प्रदेश विकास योजना आहेत्याच्या विविध जिल्हा सेवा योजना कार्यालतर्फे गेल्या वर्षी त्यांच्या कार्यालयात किती सुशिक्षित व किती अशिक्षित बेची नोंद करण्यात आली त्यापैकी किती बेना काम देण्यात आले आजपर्यंत नोंदलेल्यापैकी किती बेना अदप काम देणे शिल्लक आहे या संबंधी माहिती देणारी जीणे या विभागात प्राप्त झाली आहेत त्यांचे संकलन करून एक सविस्तर टिपपणी या विभागात प्राप्त झाली आहेत त्यांचे संकलन करून एक सविस्तर टिपपणी सोबत जोडली आहे ती कृपया पाहावी या टिप्पणीवरून हे दिसून येईल कि राज्यातील सर्व प्रकारच्या बेकारांच्या संख्येत प्रत्यक्षात वाढ होत असून सुशिक्षित बेकारांच्या संख्येत दरवर्षी होणारी वाढ तर भयावह म्हणता येईल अशा पातळीला येऊन पोचली आहे या नोंदणीकृत बेकारांशिवाय न नोंदले गेलेले बेकारही मोठ्या संख्येने असून बेकारी निवारण्याचा प्रश्न या राज्याने युद्ध पातळीवर हाती घेण्याची तातडीची गरज निमाण झाली आहे असे या विभागाला वाटते या राज्याने ज्या विविध विकास योजना तसेच रोजगार हमी योजना राज्यात हाती घेतल्या आहेत त्यामुळे मोठ्या प्रमाणावर बेकारांना काम मिळण्याची सोय झाली आहे</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
@@ -3182,22 +3620,37 @@
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>मराठी लगुलेखन शंबर शब्द प्रती मिनिट, पैसेज बी, रेडी, स्टाट, पैरा, शेक्षणिक क्षेत्रा मदे काम करित असताना आपना समोर छोटी मोठी अनेका अवहने येवन उभी रातात,  कदी ती वर्गाचा, कदी शालेचा, तर कदी ती समाजाचा संदर्भात असतात, कदी ती अध्यापनाचा, तर कदी ती अध्ययनाचा संदर्भातील असतात, कदी ती व्यक्तिगत, तर कदी ती सामोहिक स्वरुपाची असतात,  कधी ती शालेय सोई बाबच्ची, तर कधी ती शैक्षणिक साहित्य साधना सम्मंदीची असतात, तर कधी ती व्यवहरा बाबच्ची असतात.  शिक्षकाना अशा आववानाना सामोरे जानेची नित्य तयारी धेवावी लागेल। त्या सठी एखादा दुसरा चोटा प्रकल्प हाती गेवुन, एखादी नवी पधती हातालून, एखादी नवी रीत शोधून काडून, एखादा मार्ग शोधून काडून आपणास का  आपनास आपलाही विकास करून घेता येईल आपल्या कार्याचा नवया दिशा धुन्डालता येतिल आपल्या आवडीचा एखादा छंद वाधीला लावने प्रसंगी लेखन करने मुलान सथी गानी गोष्टी लिहिने कथा कथन करने  रंजन मंडले चालविने शेक्षणीक पाहनी सर्खे उपक्रम हाती घेने इत्यादी प्रकार्चे नवे कार्यक्रम योजून आपनास आपल्या व्यावसाया मधे जीवन तपना आणता येईल  हे सारे आपनास स्वयाम प्रेरणे ने आणि स्वयाम प्रद्ने ने करावे लागेल पैरा विद्या पिठीय शिक्षणाचे हे जे विशेश अंग आहे त्याचा तुम्ही कालजी पुर्वक विचार करावा अशिमाजी तुम्हास विननती आहे  जा प्रदेशात व जाकालात आपन रहाता होत त्याचा संदरभात वस्तु स्थितीचा व घटनांचा अभ्यास करने हे तुम्हे आध्य कर्तव्य थरते  प्रतेक देशाला किम्बवना देशातील प्रतेक भागाला त्याचे असे काही विशिष्ट प्रश्ण व गरजा असतात  नव्या रक्ताचा तुम्हा तरुणानी या प्रश्णांचा सखोल अभ्यास करून ते सोडविन्याचा सातत त्याने प्रयतन केला पाईजे  वा अशा प्रकारे तुम्ही तुम्चा प्रदेशातील लोक कल्याणाचा कारियाचा एक अवी भाज्य व जिवन्त घटक असले पाहीजे  पुर्वीचा काली लोक विद्वान व व्यासंगी पुरुशान कडोन मार्ग दर्शनाची अपेक्षा करित असत  आज विद्या पिठातुन शिक्षण घेत लेल्या तरुण स्त्री पुरुशान कडोन अशा मार्ग दर्शनाची अपेक्षा आहे  प्यारा अर्थात न्यान दानाची पुर्वीची पद्धत व आजची पद्धत यात पुषकल फरक जालेले आहे  त्याच प्रमाणे सुख सम्रुद्धी चा कल्प नाही आज बदल लेल्या आहेत। थोड क्यात मनजे जीवनाकडे पाहन्याचा दुरुश्टिकोन पुर्वीच्षा आज आमुलागर बदलला आहे।  तथा पी अखील मनुष्य मात्राचे जास्ति जास्त कल्याण साधन्याचे मानवाचे अंतीम धेय हे बदल लेले नाही।  कर तτε हौतस्ति जास्ति जागर आमों अलागर साधनर आमुलागर िकल्श्टिकोन पुरुश्ट है का बदल लेख नात् »,</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन शंभर शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट प्यारा शैक्षणिक क्षेत्रामध्ये काम करीत असताना आपणा समोर छोटी मोठी अनेक आव्हाने येऊन उभी राहतात कधी ती वर्गाच्या कधी शाळेच्या तर कधी ती समाजाच्या संदर्भात असतात कधी ती अध्यापनाच्या तर कधी ती अध्ययनाच्या संदर्भातील असतात कधी ती व्यक्तिगत तर कधी ती सामूहिक स्वरूपाची असतात कधी ती शालेय सोयी बाबतची तर कधी ती शैक्षणिक साहित्य साधना संबंधीची असतात कधी ती व्यवसायासबंधीची असतात तर कधी ती व्यवहाराबाबतची असतात शिक्षकांना अशा आव्हानाना सामोरे जाण्याची नित्य तयारी ठेवावी लागेल त्यासाठी एखादा दुसरा छोटा प्रकल्प हाती घेऊन एखादी नवी पद्धती हाताळून एखादी नवी रीत शोधून काढून एखादा मार्ग शोधून काढून आपणास काम करावे लागेल नवे उपक्रम योजून आपणास आपलाही विकास करून घेता येईल आपल्या कार्याच्या नव्या दिशा धुंडाळता येतील आपल्या आवडीचा एखादा छंद वाढीला लावणे प्रसंगी लेखन करणे मुलांसाठी गाणी गोष्टी लिहिणे कथा कथन करणे रंजन मंडळे चालविणे शैक्षणिक पाहणी सारखे उपक्रम हाती घेणे इत्यादी प्रकारचे नवे कार्यक्रम योजून आपणास आपल्या व्यवसायामध्ये जिवंतपणा आणता येईल हे सारे आपणास स्वयं प्रेरणेने आणि स्वय प्रज्ञेने करावे लागेल प्यारा विद्यापीय शिक्षणाचे हे जे विशेष अंग आहे त्याचा तुम्ही काळजीपूर्वक विचार करावा अशी माझी तुम्हा विनंती आहे ज्या प्रदेशात व ज्या काळात आपण राहत आहोत त्याच्या संदर्भात वस्तुस्थितीचा व घटनाचा अभ्यास करणे हे तुमचे आद्य कर्तव्य ठरते प्रत्येक देशाला किबवना देशातील प्रत्येक भागाला त्याचे असे काही विशिष्ट प्रश्न व गरजा असतात नव्या रक्ताच्या तुम्हा तरुणानी या प्रश्नांचा सखोल अभ्यास करून ते सोडविण्याचा सातत्याने प्रयत्न केला पाहिजे व अशा प्रकारे तुम्ही तुमच्या प्रदेशातील लोक कल्याणाच्या कार्याचा एक अविभाज्य व जिवंत घटक असले पाहिजे पूर्वीच्या काळी लोक विद्वान व व्यासंगी पुरुषांकडून मार्गदर्शनाची अपेक्षा करीत असत आज विद्यापीठातून शिक्षण घेतलेल्या तरुण स्त्री पुरुषांकडून अशा मार्गदर्शनाची अपेक्षा आहे प्यारा अर्थात ज्ञानदानाची पूर्वीची पद्धत व आजची पद्धत यात पुष्कळ फरक झालेले आहे त्याचप्रमाणे सुख समृद्धीच्या कल्पनाही आज बदललेल्या आहेत थोडक्यात म्हणजे जीवनाकडे पाहण्याचा दृष्टकोन पूर्वीपेक्षा आज आमूलाग्र बदलला आहे तथापि अखिल मनुष्य मात्राचे जास्तीत जास्त कल्याण साधण्याचे मानवाचे अंतिम ध्येय हे बदललेले नाही</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U30" s="2" t="inlineStr">
-        <is>
-          <t>मराधी लगुलेखन, शम्भर शब्द प्रती मिनिट, ट्रायल पैसेच, रेडी, स्टांट, पैरा, आमचा राज्याचे अधिक्रूत धोरण समाजवादी आहे,  मनोन समाजवाद हा शब्द आमी हेत्तु पुरसर वापर्तो, परंतु समाजवादा बतल आमी बोलावयास लागले नंतर, काही मानसाना अगदी अउघल्ल्यास अरके वाटू लागले,  त्याना असे वाटू लागले की, हे लोग समाजवादा बतल बोलावयास लागले तर, आमचे सगले संपलेच, आमी मा काई बोलावयाचे,  परंतु मी त्याना सांगू इच्छितो की त्याचा समाजवाद बेगला आहे, आमचे समाजवाद बेगला आहे, आमी जो समाजवाद मानतो, तो त्यांचा समाजवादास सार्खा नही, ते मंतात त्यांचा समाजवाद खास आहे, त्यांचा समाजवाद त्याना लखला�</t>
-        </is>
-      </c>
       <c r="V30" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन शंभर शब्द प्रतिमनिट ट्रायल पॅसेज रेडी स्टार्ट प आमच्या राज्याचे अधिकृत धोरण समाजवादी आहे म्हणून समाजवाद हा शब्द आम्ही हेतूपरसर वापरतो परंतु समाजवादाबद्दल आम्ही बोलावयास लागल्यानंतर काही माणसांना अगदी अवघडल्यासारखे वाटू लागले त्यांना असे वाटू लागले की हे लोक समाजवादाबद्दल बोलावयास लागले तर आमचे सगळे संपलेच आम्ही मग काय बोलावायचे परंतु मीांूो की् ज त्यां सारख नाही ते म्हणतात त्यांचा स खास आहे त्यांचा सना लखलाभ हो</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3264,7 +3717,7 @@
       <c r="P31" s="2" t="n"/>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन 120 शब्द प्रती मिनिट, पैसेज ए, रेडी, स्टार्ट, प्रदूशन हे एक हलु हलु प्रभाव दाखवनारे वीश आहे, आनिते प्रत्येक दिशागणिक अपल्या जीवनाला नश्ट करित आहे, प्रदूशन नैसर्गीक वातावरनाला दूशित कर�  द्वनी प्रदूशन आनि जल प्रदूशन वायू प्रदूशन हे वाहनान मदून निगनारे इंदनाचे धूर अउद्ध्योगीक कार्खाने उबनारी धूर इत्याधी कारणान मोये होते, या दूशित वायूला श्वासाद्वारे आत घितल्याने रुदय संबंधी रो  अगन तसेच इतर समारंबातील आवाज इत्याधी अनेक कारणान मोये होते, अत्याधीक द्वनी प्रदूशना मोये बहिरेपना आनि काना संबंधी रोग वाडतात, जल प्रदूशन ही सुद्धा अतिशय मोठ्या प्रमानात निर्मान जालेली प्रदूशनाची समस्या �  पद्धतिने होत आहे, या प्रदूशनाचा समस्येला कमी करन्या साथी जास्तित जास्त जाडे लावायला हवी, वो लोकानना प्रदूशनाने होडार्या समस्यान विशयी जागृत करायला हवे, आजचे यूग हे, विद्न्यानाचे यूग आहे, जज़शे विद्न्या  आज प्रदुशन एक समस्या बनलेली आहे। परिच्छेद अपल्या धर्तिवर आज तीन तरह चे प्रदुशन आहे।  अपल्या नागरिकानना स्वच्छा पिन्याचे पाणी उपलब्ध करन्यास असमर्थ आहे। याचा परिणाम नागरिकानना अशुद्ध पाणी प्याईलेने अनेक रोग होतात आणी हे रोग आरोग्याला धोकादायक थरतात।  वायू प्रदुशनाचा सामना करत आहेत। विकसित जालेला शहरात अउध्योगी करनाचा दर हा खूप अधिक अस्तो। या मोले निशर्ग अपले संतुलन वाचवन्यात अयशस्वी होतो।  कार्खानेंचा दुराड्यातुन निगनारा अतिशय विशारी वायू वातावर्नातिल प्राण वायूचे प्रमाण कमी करतो आणी प्राण वायूचा अभाव जाल्याने स्वासान संबंधी रोग वाहला लागतात।  बर्याज्जा हे प्रदुशन अधिक जाल्याने रुदाई विकाराचा जटका सुद्धा येवू शक्तो। परिच्चेद द्वनी प्रदुशन हे सुद्धा वायू प्रदुशना एवडेच घातक आहे।  मोट मोठ्या महानगरात वहनांचे आवाज आणी कार्खान्यान मुए द्वनी प्रदुशन वाडते। बहिरे पणा मानसिक गोंधर आणी मानसिक असंतुलन हे द्वनी प्रदुशनाचे काही दुश्परिणाम आहे।  आज द्वनी प्रदुशन रोखन्या साथी कडक काईदे तयार करन्याची आवशकता आहे। मोठ्या आवाजात वाद्य वाजवी नावर बंदी आणायला हवी। मनुष्य निशर्गाला विशारी करीत आहे। मनुष्य स्वतहा वेईच सावत जाला नाही तर त्याला या</t>
+          <t>मराठी लघुलेखन एकशे वीस शब्द प्रतिमिनिट पॅसेज ए रेडी स्टार्ट प्रदूषण हे एक हळूहळू प्रभाव दाखवणारे विष आहे आणि ते प्रत्येक दिवसागणिक आपल्या जीवनाला नष्ट करीत आहे प्रदूषण नैसर्गिक वातावरणाला दूषित करून पर्यावरणात असथिरता निर्माण करते प्रदूषणाला मुख्यतः तीन भागात विभाजित केले आहे वायू प्र्रदूषण ध्वनी प्रदूषण आणि जलप्रदूषण वायू प्रदूषण हे वाहनांमधून निघणारे इंधनाचे धूर औद्योगिक कारखाने उडणारी धूळ इत्यादी कारणांमुळे होते या दूषित वायूला श्वासाद्वारे आत घेतल्याने हृदय संबंधी रोग निर्माण होतात निसर्गाला हानी पोहोचवणारे दुसरे प्रदूषण ध्वनी प्रदूषण आहे हे प्रदूषण वाहनांचे हॉर्न औद्योगिक कारखान्यातील मशीनचे आवाज लग्न तसेच इतर समारंभातील आवाज इत्यादी अनेक कारणांमुळे होते अत्याधिक ध्वनी प्रदूषणामुळे बहिरेपणा आणि कानासबंधी रोग वाढतात जल प्र्रदूषण ही सुद्धा अतिशय मोठ्या प्रमाणात निर्माण झालेली प्रदूषणाची समस्या आहे नदी व तलावात कारखान्यातून निघणारे टाकाऊ पदार्थ व प्लास्टिक कचरा टाकल्याने जल प्र्रदूषण होते आज प्रदूषण हे अनेक पद्धतीने होत आहे या प्रदूषणाच्या समस्येला कमी करण्यासाठी जास्तीत जास्त झाडे लावायला हवीत व लोकांना प्रदूषणाने होणाऱ्या समस्यांविषयी जागृत करायला हवे आजचे युग हे विज्ञानाचे युग आहे जस जसे विज्ञान आणि तंत्रज्ञान प्रगत होत आहे तस तसे त्याचे दुष्परिणाम देख वाढत आहेत प्रदूषण हा अशाच तंत्रज्ञानाचा एक दुष्पिणाम आहे आज प्रदूषण एक समस्या बनलेली आहे परिच्छेद आपल्या धर्तीवर आज तीन तऱहेचे प्रदूषण आहे जलप्रदूषण वायू प्रदूषण आणि ध्वनी प्रदूषण विकसनशील देश जसे भारत श्रीलंका पाकिस्तान आणि अन्य अनेक देश प्रदूषणाच्या समस्येला सामोरे जात आहेत नैसर्गिक स्रोतांचा योग्य वापर न करणे आणि अधिक तंत्रज्ञान माहीत नसलेले हे देश आपल्या नागरिकांना स्वच्छ पिण्याचे पाणी उपलब्ध करण्यास असमर्थ आहेत याचा परिणाम नागरिकांना अशुद्ध पाणी प्यायल्याने अनेक रोग होतात आणि हे रोग आरोग्याला धोकादायक ठरतात म्हणून अशुद्ध पाणी हा प्राणघातक शत्रू आहे आज मोठमठे शहर वाढते मोटरसायकल चारचाकी वाहने आणि इतर मोटर वाहनांमुळे वायू प्रदूषणाचा सामना करत आहेत विकसित झालेल्या शहरात औद्योगकरणाचा दर हा खूप अधिक असतो यामुळे निसर्ग आपले संतुलन वाचवण्यात अयशस्वी होतो कारखान्यांच्या धुराड्यातून निघणारा अतिशय विषारी वायू वातावरणातील प्राणवायूचे प्रमाण कमी करतो आणि प्राणवायूचा अभाव झाल्याने श्वासांसबंधी रोग व्हायला लागतात बऱ्याचदा हे प्रदूषण अधिक झाल्याने हृदय विकाराचा झटका सुद्धा येऊ शकतो परिच्छेद ध्वनी प्रदूषण हे सुद्धा वायू प्रदूषणा एवढेच घातक आहे मोठमठ्या महानगरात वाहनांचे आवाज आणि कारखान्यांमुळे ध्वनी प्रदूषण वाढते बहिरेपणा मानसिक गोंधळ आणि मानसिक असंतुलन हे ध्वनी प्रदूषणाचे काही दुष्पिणाम आहेत आज ध्वनी प्रदूषण रोखण्यासाठी कडक कायदे तयार करण्याची आवश्यकता आहे मोठ्या आवाजात वाद्य वाजविण्यावर बंदी आणायला हवी मनुष्य निसर्गाला विषारी करीत आहे मनुष्य स्वतः वेळीच सावध झाला नाही तर त्याला या प्रदूषणामुळे होणाऱ्या धोक्यापासून कोणीच वाचवू शकणार नाही</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
@@ -3274,22 +3727,37 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगू लेखन 120 शब्द प्रती मिनिट, पैसेज बी, रेडी, स्टार्ट  प्रदूशन कोंत्याही प्रकारचे असो, ते मनुष्य जीवना साथी दोकादायकतर आहेच, पन या सोबत वनस्पती आणी प्राणयान नाही ते घातक आहे  प्रदूशन मानव जाती साथी एक समस्या आहे, जो परियंत आपन विद्न्यान आणी तंत्रद्न्यानाने होनार्या या दुष्परिणामानना कमी करन्या साथी उपाय सोधून गेत नाही, तो परियंत मानवी जीवन दोक्यात आहे  शासनाने याची दखल ग्याईला हवी आणी परिया वरणाला वाचावन्या साथी उरुक्ष लागवड जल शुद्धी करन ग्यास्वर चालनार्या चुली इत्यादी उपक्रम राबवाईला हवेत  आपल्याला प्रदुशनाशी लड़ा देऊन, त्याला कोंत्याही किम्ती वर संपवायचे आहे  आज प्रुत्वी वर वाढ़त असलेल्या समस्यान मद्धे प्रदुशन ही सर्वात मोठी समस्या आहे  प्रदुशनाशा अर्थ होतो नैसर्गीक संतुलनात दोसनिर्मान होने  स्वासोच्छवसाथी सुध्ध हवा न मिणे, प्याईला स्वच्छ पाणी न मिणे, स्वच्छ अन्न न मिणे  आनि श्यान्त वातावरन उपलब्ध न होने  प्रदुशन मानवजाती साथी किती हानी कारक आहे, हे सर्वान्नास्ट माहीत जाले आहे, परंतु हे ध्न्यान फक्त कुस्तका परियंत सीमीत आहे, वास्तविक जीवनात मनुष्य अपली प्रगती आणी सुखह सुविधा मध्ये वृद्धी करनी चाथी दिवसेंदिवास  तर त्याला प्रदुशन मटले जाते।  चोविस्टास चालनारे कारखाने गाड्या मोटारी इत्यादी मदून निगनारा काला धूर वायू प्रदुशन वाढवनाचे कारिय करतों।  परिच्छेद जल प्रदुशना अनंतर सर्वात मोठी प्रदुशन समस्या मंजे ध्वनी प्रदुशन होय।  द्वनी प्रदुशन कारखाने गाड्या मोटारी लाउड स्पीकर इत्यादी चा आवाजा मुले वाढ़त आहे।  द्वनी प्रदुशना मुले बहिरेपना सर्ख्या समस्या वाढ़त आहेत।  सतत मुठ्या प्रमानात करकश आवाज ऐकल्याने मानसिक तनाव वाडतो मनुन ध्वनी प्रदुशन कमी करन्या साथी कारखाने वन आगरिकाननी उच्च दर्जाची यंत्रे वाप्रायला हवी।  वायू, जल, वध्वनी प्रदूशन कमी करने साथी अनेक प्रकारचे उपाय केले जाओ शक्तात।  जासित जास्त हिर्वल निर्मान करायला हवी।  रस्त्याचा दोनी बाजुन्ना अधिक-अधिक जाडे लावायला हवी।  जाडे लावा, जाडे जगवा, हाँ संदेश प्रशारीक करायला हवा।  कार्खानेनना मनुष्य वस्ति पाशून दूर ठेवायला हवे।  खाजगी वाहनाचा वापर कमी प्रमानात करायला हवा।  इत्यादी उपाय जर आपनकेलेत तर प्रदुशन सार्ख्या समस्यला दूर करन्या साथी खूप मदत होईल।  प्रदुशन हे हलु-हलु परिणाम करनारे एक विश आहे।  ते हवा, पाणी, वधुएईचा माध्यमाने फक्त मनुष्यस नवेतर जीव, जन्तू, पशू, पक्षी, जाडे, जुडूपे या वनस्पतिनना देखील नश्ट करते।  वार्त्या प्रदुशनामुले देशाचे खूप मोठे नुक्सान होते।  जाडे जेवा, जाडे नुक्सान होते।</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन एकशे वीस शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट प्रदूषण कोणत्याही प्रकारचे असो ते मनुष्य जीवनासाठी धोकादायक तर आहेच पण यासोबत वनस्पती आणि प्राण्यांनाही ते घातक आहे प्रदूषण मानव जातीसाठी एक समस्या आहे जोपर्यंत आपण विज्ञान आणि तंत्रज्ञानाने होणाऱ्या या दुषपिणामांना कमी करण्यासाठी उपाय शोधून घेत नाही तोपर्यंत मानवी जीवन धोक्यात आहे शासनाने याची दखल घ्यायला हवी आणि पर्यावरणाला वाचवण्यासाठी वृक्ष लागवड जलशुद्धीकरण गॅसवर चालणाऱ्या चुली इत्यादी उपक्रम राबवायला हवेत आपल्याला प्रदूषणाशी लढा देऊन त्याला कोणत्याही किमतीवर संपवायचे आहे आज पृथ्वीवर वाढत असलेल्या समस्यांमध्ये प्रदूषण ही सर्वात मोठी समस्या आहे प्रदूषणाचा अर्थ होतो नैसर्गिक संतुलनात दोष निर्माण होणे श्वासोच्छवासाठी शुद्ध हवा न मिळणे प्यायला स्वच्छ पाणी न मिळणे स्वच्छ अन्न न मिळणे आणि शांत वातावरण उपलब्ध न होणे प्रदूषण मानव जातीसाठी किती हानकारारक आहे हे सर्वांनाच माहीित झाले आहे परंतु हे ज्ञान फक्त पुस्तकापर्यंत सीमित आहे वास्तविक जीवनात मनुष्य आपली प्रगती आणि सुख सुुविधामध्ये वृद्धी करण्यासाठी दिवसेंदिवस प्रदूषण करीत आहे पृथ्वी पाणी हवा ध्वनी इत्यादीमध्ये आढळणारे तत्व जर असंतुलित असतील तर त्याला प्रदूषण म्हटले जाते मनुष्याद्वारे निर्माण झालेला कचरा व टाकाऊ पदार्थ जे निसर्गात फेकले जातात त्या पदना प्रदूषक म्हटले जाते प्रदूषण अनेक प्रकारचे असते प्रदूषणाचे काही प्रमुख प्रकार पुढील प्रमाणे आहेत जल प्र्रदूषण वायू प्रदूषण आणि ध्वनी प्रदूषण भारतातील मोठमठ्या महानगरांमध्ये वायू प्रदूषण मोठ्या प्रमाण पसरत आहे चोवीस तास चालणारे कारखाने गाड्या मोटारी इतदी मधून निघणारा काळाधूर वायू प्रदूषण वाढवण्याचे कार्य करतो दिल्ली मुंबई यासारख्या मोठ्या शहरांमध्ये श्वास घेणे सुद्धा कठीण आहे मोठ्या प्रमाणात वायू प्रदूषण वाढल्याने श्वासासबंधी विकार जडतात वायू प्रदूषण रोखण्यासाठी अधिकाधिक झाडे लावायला हवी गाड्या मोटारीचा कमीत कमी वापर करायला हवा परिच्छेद जल प्र्रदूषणानंतर सर्वात मोठी प्रदूषण समस्या म्हणजे ध्वनी प्रदूषण होय ध्वनी प्रदूषण कारखाने गाड्या मोटारी लाऊड स्पीकर इत्यादीच्या आवाजामुळे वाढत आहे ध्वनी प्रदूषणामुळे बहिरेपणासारख्या समस्या वाढत आहेत सतत मोठ्या प्रमाणात कर्कश आवाज ऐकल्याने मानसिक तणाव वाढतो म्हणून ध्वनी प्रदूषण कमी करण्यासाठी कारखाने व नागरिकांनी उच्च दर्जाची यंत्रे वापरायला हवी वायू जल व ध्वनी प्रदूषण कमी करण्यासाठी अनेक प्रकारचे उपाय केले जाऊ शकतात जास्तीत जास्त हिरवळ निर्माण करायला हवी रस्त्याच्या दोन्ही बाजूंना अधिकाधिक झाडे लावायला हवीत झाडे लावा झाडे जगवा हा संदेश प्रसारित करायला हवा कारखान्यांना मनुष्य वस्तीपासून दूर ठेवायला हवे खजगी वाहनाचा वापर कमी प्रमाणात करायला हवा इत्यादी उपाय जर आपण केलेत तर प्रदूषण सारख्या समस्येला दूर करण्यासाठी खूप मदत होईल प्रदूषण हे हळूहळू परिणाम करणारे एक विष आहे ते हवा पाणी व धुळीच्या माध्यमाने फक्त मनुष्यच नव्हे तर जीव जंतू पशु पक्षी झाडे झुडूपे या वनस्पतींना देखील नष्ट करते वाढत्या प्रदूषणामुळे देशाचे खूप मोठे नुकसान होते</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U31" s="2" t="inlineStr">
-        <is>
-          <t>मराथी लगुलेखन 120 सब्द प्रती मिनिट ट्रायल पैसेज रेडी स्टार्ट  उत्पादकाननी जीवन आणी आरोग्याला अपायकारक किव्वा माल मत्तेला दोका निर्मान करनार्या वस्तुंचे उत्पादन वविपणन करू नए  आरोग्याला अपायकारक असे रंग किव्वा स्वाद यंचा वापर करू नए  खेलनी, कपडे, गर्गूती उपकरने वापरनास सुरक्षित आहे हे पाहनाची जबाबदारी काईदयाने विक्रेत्यावर टाकली आहे  वस्तुंची गुणवत्ता, प्रमान, शमता, किम्मद उत्पादनाची तारीक वस्तु उत्पादना साथी वापरलेले घटक इत्यादी महिती आनी अनुचित प्रक्षे पासून वा जाहराती पासून सौरक्षन मिलविनाचा प्रत्यक ग्राहकाला हक्क आहे  या मुए वस्तु विकध्यापूर्वी ग्राहकानना संपूर्ण महिती चा विचार करून वस्तु विकध्यावी किवा नाही याचा विचार करता यहीन</t>
-        </is>
-      </c>
       <c r="V31" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन एकशे वीस शब्द प्रतिमिनिट ट्रायल पॅसेज रेडी स्टार्ट उत्पादकांनी जीवन आणि आरोग्याला अपायकारक किंवा मालमत्तेला धोका निर्माण करणाऱ्या वस्तूचे उत्पादन व विपणन करू नये आरोग्याला अपायकारक असे रंग किंवा स्वाद यांचा वापर करू नये खेळणी कपडे घरगुती उपकरणे वापरण्यास सुरक्षित आहेत हे पाहण्याची जबाबदारी कायद्याने विक्रेत्यावर टाकली आहे वस्तूंची गुणवत्ता प्रमाण क्षमता किंमत उत्पादनाची तारीख वस्तू उत्पादनासाठी वापरलेले घटक माहिती आणि अनु प्रक्षेराती संक्षण्या प्र्येक हक्क आहे यामुळे वस्तू विकत घेण्यापूर्वी ग्राहकांना संपूर्ण माहितीचा विचार करून वस्तू विकत घ्यावी किंवा नाही याचा विचार करता येईल</t>
+        </is>
+      </c>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3824,7 @@
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन, 120 शब्द प्रती मिनेट, पैसेज एड, रेडी, स्टार्ट  अध्यक्षा महराज, आज अपल्या राज्या मद्धे, ग्रामीन विभागात पिन्याचा पान्याची समस्या अत्यंत उग्रस्वरूप धारण करू लगली आहे  या कडे मला शासनाचे लक्ष वेधावयाचे आहे, पाउसाल्याचे चार महिने सोडले तर, वर्षातून सहा महिने ग्रामीन विभागाती लोकानना पिन्याचा पान्याची टंचाई सहन करावी लागते  सरकारने पिन्याचा पान्याची टंचाई दूर करन्या साथी मोठ्या प्रमाणावर योजना हाती गितल्या आहे याची मला जानेव आहे  अध्यापही हा प्रश्ण सुटलेला नाही किववा त्याची गंभीरता कमी जालेली नाही  हेही मला येथे नमूद करने अवश्यक वटते  पानी ही मानसाची मुलभूत गरज आहे आनी पानी नसले की त्याचे सारे व्यवहार थंडावतात  त्याचे दैनन्दिन जीवन विश्कलित होते  महराष्ट्रातील बहुताउंस ग्रामिन भाग हा टंचाई ग्रस्त अस्तो  आनी ही टंचाई केवल अन्न धन्याची नस्ते तर पिन्याचा पान्याची अस्ते  टंचाई ग्रस्त भागात पिनयाचा पाणयाचा प्रश्ण सोडविने ही अत्यावश्चक गोष्ट होउन बसली आहे  शासना तरफे टंचाईचा कालात टैंकरचा मदतीने ग्रामिन भागातील लोकानना पाणी पुरविले जाते  किववा बैल गाड्यांची ही मदत गेतली जाते परंतु हा वर वरचा उपाय जाला त्या भागातील पाणयाची टंचाई कायमची दूर करावयाची असेल तर त्या करिता व्यापक प्रमानावर योजना हाती गेने अवश्यक आहे  अशा तंचाई ग्रस्त भागात नविन कूप नलीका विहरी खोदने जुन्या विहरी अधिक खोल करने किववा नव्या विहरी बांधने अशा उपाय योजना शासना तरफे हाती गेतल्या जात आहेत  परिछेद सामुदाईक विहरी ही बांधल्या जात आहेत परंतु त्यांची डाग डुजी वेलेवर करने अवश्यक अस्ते ग्राम पंचायती कडे हे काम सोपविन्यात आले अशुन त्या साथी त्यान्ना मदत ही केली जात आहे  राज्यात टंचाय ग्रस्त भागात आता परियंत अशा अनेक नलीका विहरी खोद्न्यात आले अशुन जुन्या विहरी खोल करन्यात आले आहेत अवश्यक तेथे नव्या विहरी बांधन्यात आले आहेत परंतु मला नमूत करने अवश्यक वाटते की  जा नवीन विहिरी बांदले जातात त्या विहिरीनना पुरेशे पाणी लागले आहे, किववा नाही याची खात्री संबंधित ग्राम सैवकान तरफे करून भेतली जाने अवश्यक आहे, अन्य था दुसर्या वर्षी त्या विहिरी आठतात आणी त्या गावाचा पिन्य  चा कडून गेतली जावी आणी त्या थिकानी नवीन विहिरी गेतली जावी अशी सूचना मला या निमित्ताने करावयाची आहे, असे केल्यास आज अ यशस्वी जालेला विहिरीनची संख्या आणी परिणाम तहा वाया गेलेला शासनाचा पैशांची रक्कम जी सार्ख  अवश्यक तो निधी उपलब्ध करून देन्या साथी शासन तयार आहे याचा मला मुद्दाम उल्लेख करावयाचा आहे  पाजर तलावा मुले आसपास चा भागातील वीरिंचा पान्याची पातली वाडन्यास मदत होते  या उपाय योजना पान्याची तंचाई दूर करन्या साथी केल्या जातात</t>
+          <t>मराठी लघुलेखन एकशे वीस शब्द प्रति मिनिट पॅसेज हे रेडी स्टार्ट अध्यक्ष महाराज आज आपल्या राज्यामध्ये ग्रामीण विभागात पिण्याच्या पाण्याची समस्या अत्यंत उग्र स्वरूप धारण करू लागली आहे याकडे मला शासनाचे लक्ष वेधावयाचे आहे पावसाळ्याचे चार महिने सोडले तर वर्षातून सहा महिने ग्रामीण विभागातील लोकांना पिण्याच्या पाण्याची टंचाई सहन करावी लागते सरकारने पिण्याच्या पाण्याची टंचाई दूर करण्यासाठी मोठ्या प्रमाणावर योजना हाती घेतल्या आहेत याची मला जाणीव आहे अद्यापही हा प्रश्न सुटलेला नाही किंवा त्याची गंभीरता कमी झालेली नाही हेही मला येथे नमूद करणे आवश्यक वाटते पाणी ही माणसाची मूलभूत गरज आहे आणि पाणी नसले की त्याचे सारे व्यवहार थंडावतात त्याचे दैनंदिन जीवन विस्कळीत होते महाराष्ट्रातील बहुतांश ग्रामीण भाग हा टंचाईग्रस्त असतो आणि ही टंचाई केवळ अन्नधान्याची नसते तर पिण्याच्या पाण्याची असते टंचाईग्रस्त भागात पिण्याच्या पाण्याचा प्रश्न सोडविणे ही अत्यावश्यक गोष्ट होऊन बसली आहे शासनातर्फे टंचाईच्या काळात टँकरच्या मदतीने ग्रामीण भागातील लोकांना पाणी पुरविले जाते किंवा बैलगाड्यांचीही मदत घेतली जाते परंतु हा वरवररचा उपाय झाला त्या भागातील पाण्याची टंचाई कायची दूर करावयाची असेल तर त्याकरिता व्यापक प्रमाणावर योजना हाती घेणे आवश्यक आहे अश टंचाईग्रस्त भागात नवीन कूपनलिका विहिरी खोदणे जुन्या विहिरी अधिक खोल करणे किंवा नव्या विहिरी बांधणे अशा उपाय योजना शासनातर्फे हाती घेतल्या जात आहेत परच्छद सामुदायिक विहिरी ह बांधल्या जात आहेत परंतु त्यांची डागडुजी वेळेवर करणे आवश्यक असते ग्रामपंचायतीकडे हे काम सोपविण्यात आले असून त्यासाठी त्यांना मदतही केली जात आहे्यात टंचाईग्रस्त भागात आतापर्यंत अशा अनेक नलिका विहिरी खोण्यात आल्या असून जुन्या विहिरी खोल करण्यात आल्या आहेत आवश्यक तेथे नव्या विहिरी बांधण्यात आल्या आहेत परंतु मला नमूद करणे आवश्यक वाटते की ज्या नवीन विहिरी बांधल्या जातात त्या विहिरींना पुरेसे पाणी लागले आहे किंवा नाही याची खात्री संबंधित ग्रामसेवकांतर्फे करून घेतली जाणे आवश्यक आहे अन्यथा दुसऱ्या वर्षी त्या विहिरी आटतात आणि त्या गावाच्या पिच्या पाण्याचा प्रश्न कायमच राहतो म्हणून जमिनीत कोठे पाणी लागण्याचा संभव आहे याची माहिती प्रथम संबंधित विभागाच्या कडून घेतली जावी आणि त्याच ठिकाणी नवीन विहिरी घेतली जावी अशी सूचना मला या निमित्ताने करावयाची आहे असे केल्यास आज अयशस्वी झालेल्या विहिरींची संख्या आणि परिणामत वाया गेलेल्या शासनाच्या पैशांची रक्कम जी सारखी वाढत आहे ती वाढणार नाही हे सारे काम युद्ध पातळीवर हाती घेतले जाणे आवश्यक आहे त्याकरिता आवश्यक तो निधी उपलब्ध करून देण्यासाठी शासन तयार आहे याचा मला मुद्दाम उल्लेख करावयाचा आहे पाझर तलावामुळे आसपासच्या भागातील विहिरींच्या पाण्याची पातळी वाढण्यास मदत होते या उपाय योजना पाण्याची टंचाई दूर करण्यासाठी केल्या जातात</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr">
@@ -3366,22 +3834,37 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>मराथी लगुलेखन, 120 शब्द प्रति मिनिट, पैसेज बी, रेडी, स्टार्ट  वुरुक्ष हे मानवा साथी अत्यंत उपयुक्त असु नहीं, मानवाने अनेक वर्षा पासुन, वुरुक्षांची अपरिमीत तोड केली, या मुले निसर्गाचे संतुलन बिघडले  परजन्य मानावर परिणाम जाला, प्रदुशन वाडी मुले मानवाचा अस्टित्वास धोका जाला, अशा संकटानना मानवाने अपल्या अविचाराने दारात आनुन सोडले आहे  या संकटाची तीवरता कमी भावी या साथी महराष्ट्र शासनाने महावरुक्ष लागवडीचा महत्वा कांक्षी कार्यक्रम जुलै मद्दे राबवला आहे  हा केवल शासनाचा कार्यक्रम न रहता याद सर्व थरातील नागरिक उच्छाहाने सामील जाले ही अतिशे आनंदाची बाब ठरली  आता सर्वांची जबाबदारी वाडली असुन लावलेला व्रुक्षांचे संगोपन आनी सववर्धन करने ही आवशक आहे  लावलेला प्रत्यक व्रुक्ष जगला पाहीजे याचा संकल्प आपन करने अत्यंत गर्जेचे थरते  आपन सर्वांची व्रुक्ष संगोपनाचा केलेला संकल्प महाराष्ट्राला हरित आनी सम्रुद्ध करने साथी उत्तुंग अशी जेब ठरू शक्तो  गेल्या काही दिवसान पासुन महाराष्ट्राचा विविध भागात चांगला पाउस पड़त आहे या मुले चैतन्यदाई वातावरण निर्मान जाले आहे  सामान्य शेतकर्यांचा चेहर्यावर हसु परत आले आहे  मुख्य मंत्राणनी जलयुक्त शिवाराचा कामानवर प्राधान्याने लक्ष दिले आहे असे दिसुन येते  उपलब्ध माहितीनुसार विविध जलयुक्त प्रकलपान मद्धे चांगला जलसाठा चाला आहे  संग लोकसेवा आयोगा मार्फत गेनात आलेल्या नागरी सेवा परिक्ष द उत्तिर्ण जलेल्या आणि नाशिक येथील पोलीस उपनिरिक्षक प्रशिक्षनात विशेश पुरसकाराने सन्मानित जलेल्याची मुलाखत  लोक राज्येचा तरुन वाचकानना निश्चीतस मोठे यश मिलवना साथी प्रेरणा देईल याची खातरी वाटते परिछेद जाडे लावनेची जगवनेची आस्था प्रतेक सर्वसामान्यांचा मनात आहे  त्या अस्थेला खतपानी घालन्याची जबाबदारी शासनाने उचल्ली आहे शासन सरावर महा व्रुक्ष लागवड अभी आनाला आकार देत अस्थाना चर्वांचा सहभाग हवा आहे  जाडे लावनारे आनी ते जगवनारे हात हवे आहे द वनमंत्री यांचा दूरदर्शी विचारधारे तुन कोट्या वधी व्रुक्षा रोपनाचा अतिशे महत्वा कांक्षी अगला वेगला आनी नाविन्य पूर्ण उपक्रम या वर्षाचा काला वधी मध्धे हाती �  सर्व घटकांचा मोठा पाठिमभा आनी समर्थन मियाले आहे व्रुक्षा रोपनाचा कार्यक्रम जन चलवली तुन सातत्य पुर्वक पुढे सुरूर आहील अशी अपेक्षा आहे प्रथम तप्यात दोन कोटी व्रुक्ष लागवडीचे उद्दिष्ट थरवले अस्त  जनतेचा प्रचंड उत्साहा मुले आम्मी जास्त जाडे लावू शकलो या उपक्रमाची नोंद जागतिक विश्व विक्रमात दुसर्यांदा घेतली आनी राज्य शासनास प्रमान पत्र दिले राज्याचे व्रुक्ष व वन अच्छादन वाडवनाचे दुष्टीने  व्रुक्ष लागवडी चा उद्दिष्टा पेक्षा अधिक व्रुक्ष लावनाचा विक्रम राज्याने केला आहे।</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
+          <t>मराठी लघुलेखन एकशे वीस शब्द प्रतिमिनिट पॅसेज बी रेडी स्टार्ट वृक्ष हे मानवासाठी अत्यंत उपयुक्त असूनही मानवाने अनेक वर्षापासून वृक्षांची अपरिमित तोड केली यामुळे निसर्गाचे संतुलन बिघडले पर्जन्यमानावर परिणाम झाला प्रदूषण वाढीमुळे मानवाच्या अस्तित्वास धोका झाला अशा संकटांना मानवाने आपल्या अविचाराने दारात आणून सोडले आहे या संकटाची तीव्रता कमी व्हावी यासाठी महाराष्ट्र शासनाने महावृक्ष लागवडीचा महत्त्वाकांक्षी कार्यक्रम जुलैमध्ये राबवला आहे हा केवळ शासनाचा कार्यक्रम न राहता यात सर्व थरातील नागरिक उत्साहाने सामील झाले ही अतिशय आनंदाची बाब ठरली आता सर्वांची जबाबदारी वाढली असून लावलेल्या वृक्षांचे संगोपन आणि संवर्धन करणेही आवश्यक आहे लावलेला प्रत्येक वृक्ष जगला पाहिजे याचा संकल्प आपण करणे अत्यंत गरजेचे ठरते आपण सर्वांनी वृक्ष संगोपनाचा केलेला संकल्प महाराष्ट्राला हरित आणि समृद्ध करण्यासाठी उत्तुंग अशी झेप ठरू शकतो गेल्या काही दिवसांपासून महाराष्ट्राच्या विविध भागात चांगला पाऊस पडत आहे यामुळे चैतन्यदायी वातावरण निर्माण झाले आहे सामान्य शेतकऱ्यांच्या चेहऱ्यावर हसू परत आले आहे मुख्यमंत्र्यांनी जलयुक्त शिवारच्या कामांवर प्राधान्याने लक्ष दिले आहे असे दिसून येते उपलब्ध माहितीनुसार विविध जलयुक्त प्रकल्पांमध्ये चांगला जलसाठा झाला आहे संघ लोकसेवा आयोगामार्फत घेण्यात आलेल्या नागरी सेवा परीक्षेत उत्तीर् झालेल्या आणि नाशिक येथील पोलीस उपनिरीक्षक प्रशिक्षण विशेष पुरस्काराने सन्मानित झालेल्याची मुलाखत लोकरा्याच्या तरुण वाचकांना निश्चितच मोठे यश मिळवण्यासाठी प्रेरणा देईल याची खात्री वाटते पररीछेत झाडे लावण्याची जगवण्याची आस्था प्रत्येक सर्व सामानच्या मनात आहे त्या आस्थेला खतपाणी घालण्याची जबाबदारी शासनाने उचलली आहे शासन स्तरावर महावृक्ष लागवड अभियानाला आकार देत असताना सर्वांचा सहभाग हवा आहे झाडे लावणारे आणि ते जगवणारे हात हवे आहेत वनमंत्री यांच्या दूरदर्शी विचारधारेतून कोट्यावधी वृक्षारोपणाचा अतिशय महत्वाकांक्षी आगळा वेगळा आणि नाविन्यपूर्ण उपक्रम या वर्षाच्या कालावधीमध्ये हाती घेण्यात आला आहे त्यास प्रधानमंत्री राज्यपाल मुख्यमंत्री महाराष्ट्राचे केंद्रातील मंत्री आणि समाजातील सर्व घटकांचा मोठा पाठिंबा आणि समर्थन मिळाले आहे वृक्षारोपणाचा कार्यक्रम जन चळवळीतून सातत्यपूर्वक पुढे सुरू राहील अशी अपेक्षा आहे प्रथम टप्प्यात दोन कोटी वृक्ष लागवडीचे उद्दिष्ट ठरवले असताना प्रत्यक्षात जास्त वृक्ष लावले गेले या उपक्रमाची नोंद जागतिक विश्वविक्रमात घेतली वृक्ष लागवडीचे उद्दिष्ट असताना जनतेच्या प्रचंड उत्साहामुळे आम्ही जास्त झाडे लावू शकलो या उपक्रमाची नोंद जागतिक विश्वविक्रमात दुसऱ्यांदा घेतली आणि राज्य शासनास प्रमाणपत्र दिले राज्याचे वृक्ष व वनच्छादन वाढवण्याच्या दृष्टीने पुढील तीन वर्षांमध्ये राज्य शासनामार्फत लोकसहभागातून पन्नास कोटी झाडे लावली जाणार आहेत यापूर्वी अनेक वृक्ष लागवडीच्या उद्दिष्टापेक्षा अधिक वृक्ष लावण्याचा विक्रम राज्याने केला आहे</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
         </is>
       </c>
-      <c r="U32" s="2" t="inlineStr">
-        <is>
-          <t>मराथी लगुलेखन 120 सब्द प्रती मिनिट ट्रायल पैसेज रेडी स्टार्ट  उत्पादकाननी जीवन आणी आरोग्याला अपायकारक किव्वा माल मत्तेला दोका निर्मान करनार्या वस्तुंचे उत्पादन वविपणन करू नए  आरोग्याला अपायकारक असे रंग किव्वा स्वाद यंचा वापर करू नए  खेलनी, कपडे, गर्गूती उपकरने वापरनास सुरक्षित आहे हे पाहनाची जबाबदारी काईदयाने विक्रेत्यावर टाकली आहे  वस्तुंची गुणवत्ता, प्रमान, शमता, किम्मद उत्पादनाची तारीक वस्तु उत्पादना साथी वापरलेले घटक इत्यादी महिती आनी अनुचित प्रक्षे पासून वा जाहराती पासून सौरक्षन मिलविनाचा प्रत्यक ग्राहकाला हक्क आहे  या मुए वस्तु विकध्यापूर्वी ग्राहकानना संपूर्ण महिती चा विचार करून वस्तु विकध्यावी किवा नाही याचा विचार करता यहीन</t>
-        </is>
-      </c>
       <c r="V32" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>मराठी लघुलेखन एकशे वीस शब्द प्रतिमिनिट ट्रायल पॅसेज रेडी स्टार्ट उत्पादकांनी जीवन आणि आरोग्याला अपायकारक किंवा मालमत्तेला धोका निर्माण करणाऱ्या वस्तूचे उत्पादन व विपणन करू नये आरोग्याला अपायकारक असे रंग किंवा स्वाद यांचा वापर करू नये खेळणी कपडे घरगुती उपकरणे वापरण्यास सुरक्षित आहेत हे पाहण्याची जबाबदारी कायद्याने विक्रेत्यावर टाकली आहे वस्तूंची गुणवत्ता प्रमाण क्षमता किंमत उत्पादनाची तारीख वस्तू उत्पादनासाठी वापरलेले घटक माहिती आणि अनु प्रक्षेराती संक्षण्या प्र्येक हक्क आहे यामुळे वस्तू विकत घेण्यापूर्वी ग्राहकांना संपूर्ण माहितीचा विचार करून वस्तू विकत घ्यावी किंवा नाही याचा विचार करता येईल</t>
+        </is>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
           <t>mr</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3931,7 @@
       <c r="P33" s="2" t="n"/>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन साथ शब्द प्रतिमिनेट पैसेज ए रड़ी स्टार्ड उपाध्यक्षम होदय परिच्छे वित्त मंत्री को देश की आर्थिक स्थिती और निर्धन्ता के संबंध में  जितनी जानकारी प्राप्त होती है उतनी किसी अन्यमंत्री को संभव नहीं होती  बजट बनाते समय वैसे तो बजट में आय व्यय का ब्यवरा होता ही है  लेकिन मूल रूप में देश की आर्थिक नीतियों में किस प्रकार का परिवर्तन हो तथा किस मार्ग पर वह देश को चलाना चाहते हैं  सरकार का लक्ष क्या है इन सब नीतियों का बजट में विवरन होता है  हमारे विट्ट मंत्रे चाहे जिस पद पर भी रहे हो चाहे वे मुख्य मंत्री रहे हो या केंद्रीय सरकार में रहे हो  उन्होंने शांदार काम किया जिस समय उन्होंने बजट प्रस्तूत किया उस समय देश को और विशेश रूप से गरिबों को उनसे बहुत सी आशाएं थी  देश में लगभख छे लाख गाओं है उनमें जो बेरोजगारी है गरिबी है उसके संबंध में देश की जनता को  उनसे बड़ी आशाएं थी और जनता देखना चाहती थी कि इस अवसर पर सरकारी नीतियों के द्वारा  देश को वे क्या मार्गदर्शन देना चाहते हैं परिचित इस द्रिष्टी से तीन महत्वपूर्ण बाते इस समय देश के सामने थी  देश का आर्थी क्विकास टेजी से हो अधिक लोगों को काम मिल सके और मुल्यों में स्थिरता आए  जहां तक इन तीन उद्देशों का संबंध है हमने देखा कि गरिबी हटाओ के संबंध में विशेश रूप से प्रयत्न किये है  झाल</t>
+          <t>हिंदी लघु लेखन साठ शब्द प्रतिमिनिट पैसेज ए रडी स्टार्ट उपाध्यक्ष महोदय परिचय वित्त मंत्री को देश की आर्थिक स्थिति और निर्धनता के संबंध में जितनी जानकारी प्राप्त होती है उतनी किसी अन्य मंत्री को संभव नहीं होती बजट बनाते समय वैसे तो बजट में आय व्यय का ब्यौरा होता ही है लेकिन मूल रूप में देश की आर्थिक नीतियों में किस प्रकार का परिवर्तन हो तथा किस मार्ग पर वह देश को चलाना चाहते हैं सरकार का लक्ष्य क्या है इन सब नीतियों का बजट में विवरण होता है हमारे वित्तमंत्री चाहे जिस पद पर भी रहे हो चाहे वे मुख्यमंत्री रहे हो या केंद्रीय सरकार में रहे हो उन्होंने शानदार काम किया जिस समय उन्होंने बजट प्रस्तुत किया उस समय देश को और विशेष रूप से गरीबों को उनसे बहुत सी आशाएं थी देश में लगभग छह लाख गांव है उनमें जो बेरोजगारी है गरीबी है उसके संबंध में देश की जनता को उनसे बड़ी आशाए थी और जनता देखना चाहती थी कि इस अवसर पर सरकारी नीतियों के द्वारा देश को वे क्या मार्गदर्शन देना चाहते हैं परिित इस दृष्टि से तीन महत्वपूर्ण बातें इस समय देश के सामने थी देश का आर्थिक विकास तेजी से हो अधिक लोगों को काम मिल सके और मूल्यों में स्थिरता आए जहां तक इन तीन उद्देशों का संबंध है हमने देखा कि गरीबी हटाव के संबंध में विशेष रूप से प्रयत्न किए है</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
@@ -3458,22 +3941,37 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन साथ शब्द प्रतिमिनेट  पैसेज ए रेडी स्टार्ट  उपाध्यक्षम हो दै परिछेद  तब उन लोगों को कुछ आशा हुई कि  हम लोग भी उसी तरह चल सकते है  जिस तरह से पहले चल रहे थे  लेकिन अभी हाल में जो चुनाव हुआ  उससे देश के धनिकों के मन में  बड़ा संदेह पैदा हुआ कि इस चुनाव के बाद  उनकी स्थिती वैसी नहीं रहेगी  जो अब तक चली आती रही है गरीबों और अमीरों के बीच में  अब तक जो बहुत बड़ा अंतर चला आ रहा था  उसको अब तेजी से दूर करने का प्रयत्न किया जाएगा  श्रीमान मैं आपका बहुत आभारी हूँ जो आपने सदन में  चालू वर्ष के बजट पर अपने विचार प्रकट करने का अवसर दिया है  मैं इस बजट का समर्थन करना चाहता हूँ परिछिद  श्रीमान मैं सबसे पहले अपने दल के नेता  प्रधानमंत्री को इस बात के लिए बधाई देना चाहता हूँ  कि उनके नेतृत्व में देश में कॉंग्रेस दल को सपष्ट बहुमत मिला  और इसके फलस्वरूप यहां पर केंद्र में  एक ऐसी सरकार का गठन हुआ जो की देश में वास्तों में समाजवाद लाना चाहती हैं  मैं वित्तमंत्री जी को इस बात के लिए बधाई देना चाहता हूँ  कि लोकसभा के मध्यवदी चुनाओं में जनताद्वारा विपक्ष दल को जो आदेश दिया गया था  उन्हें समरण है और वह तन मन धन से उस आदेश का पालन करना चाहते हैं  और जरूर उसका पालन करेंगे  गालन करेंगे</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
+          <t>हिदी लघुलेखन साठ शब्द प्रतिमिनट पैसेज ए रेडी स्टार्ट उपाध्यक्ष महोदय परि्द तब उन लोगों को कुछ आशा हुई कि हम लोग भी उसी तरह चल सकते हैं जिस तरह से पहले चल रहे थे लेकिन अभी हाल में जो चुनाव हुआ उससे देश के धनिकों के मन में बड़ा संदेह पैदा हुआ कि इस चुनाव के बाद उनकी स्थिति वैसी नहीं रहेगी जो अब तक चली आती रही है गरीबों और अमीरों के बीच में अब तक जो बहुत बड़ा अंतर चला आ रहा था उसको अब तेजी से दूर करने का प्रयत्न किया जाएगा श्रीमान मैं आपका बहुत आभारी हू जो आपने सदन में चालू वर्ष के बजट पर अपने विचार प्रकट करने का अवसर दिया है मैं इस बजट का समर्थन करना चाहता हूं परिचछद श्रीमान मैं सबसे पहले अपने दल के नेता प्रधानमंत्री को इस बात के लिए बधाई देना चाहता हूं कि उनके नेतृत्व में देश में कांग्रेस दल को स्पष्ट बहुमत मिला और इसके फलस्वरूप यहां पर केंद्र में एक ऐसी सरकार का गठन हुआ जो कि देश में वास्तव में समाजवाद लाना चाहती हैं मैं वित्तमंत्री जी को इस बात के लिए बधाई देना चाहता हूं कि लोकसभा के मध्यवधि चुनाव में जनता द्वारा विपक्ष दल को जो आदेश दिया गया था उन्हें स्मरण है और वह तन मन धन से उस आदेश का पालन करना चाहते हैं और जरूर उसका पालन करेंगे</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="U33" s="2" t="inlineStr">
-        <is>
-          <t>हिंदी लगुलेखन, साथ शब्द प्रतिमिनेट, ट्राइल पैसेज, रेडी स्टार्ड, उपाध्यक्ष महोदै, मैं इस बिल का स्वागत करता हूँ,  मुझे दुख है कि कई माननिय सदस्यों ने, जिनोंने पता नहीं किस कारण से कहा, तो यह कि वे इस बिल का स्वागत करते हैं,  लेकिन वास्तव में इसका विरोध करने का उन्होंने प्रयत्न किया है, हम सब इस प्रयत्न का दिल से स्वागत करते हैं,</t>
-        </is>
-      </c>
       <c r="V33" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>हिंदी लघुलेखन साठ शब्द प्रतिमिनिट ट्रायल पैसेज रेडी स्टार्ट उपाध्यक्ष महोदय मै इस बिल का स्वागत करता हूँ मुझे दुख है कि कई माननीय सदस्यों ने जिन्होंने पता नहीं किस कारण से कहा तो यह कि वे इस बिल का स्वागत करते हैं लेकिन वास्तव में इसका विरोध करने का उन्होंने प्रयत्न किया है हम सब इस प्रयत्न का दिल से स्वागत करते हैं</t>
+        </is>
+      </c>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3540,7 +4038,7 @@
       <c r="P34" s="2" t="n"/>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन ताठ शब्द प्रती मिनेट पैसेज ए रेडी साठ अध्यक्षजी कारा किसी भी देश की विदेश नीती अपने में कोई स्वतंत्र नीती नहीं होती है  वरन वह किसी देश की आंतरिक नीती को स्पष्ट करती है उदाहरन के लिए हम अमरिका को ले सकते है  उसने अपने यहा अधिक अन्न पैदा किया और जब उसके पास अनाज फाल्तु बच गया  तब वह अपने बकाया अनाज की बिक्री के लिए ऐसे देशों की तलाश करने लगा  जो उधार पर माल ले सकते हो किन्तु हमारी आंतरिक नीती ने यहा तै किया की  कि खर्चीले ढंग से सरकार चलाएंगे और स्वदेशी मुद्रा की कोई राशी हमारे पास नहीं बचेंगी  हमने कर भी लगा दिये और मुद्रा प्रसार भी कर दिया कुछ संकट पढ़ने के बाद  इस बात की अवशकता को नहीं समझा की उस पैसे का कही अन्यत्र उपयोग कर सके  पैरा श्रीमन मुझे माननिय प्रधानमंत्री जी के इस कथन पर दुख होता है की  दुनिया के अमीर और गरीब देशों का अंतर लगातार बढ़ता जा रहा है  मैं उनसे यह पूछना चाहती हूँ की  भारत की विदेश नीती ने उस अंतर को घटाने की क्या कोशिश की है  क्या भारत सरकार ने कभी दुनिया की पंचायत में यह कहने की हिम्मत की है  की बालिग मताधिकार के आधार पर यू एन ओ का चुनाव होकर एक संसद बनाई जाए  और क्या आप में यह देखने की हिम्मत है की फौज को कर लगा कर एक विकास का खाता खोल दिया जाए</t>
+          <t>हिंदी लघुलेखन साठ शब्द प्रति मिनट पैसेज ए रेडी स्टार्ट अध्यक्ष जी तारा किसी भी देश की विदेश नीति अपने में कोई स्वतंत्र नीति नहीं होती है वरन वह किसी देश की आंतरिक नीति को स्पष्ट करती है उदाहरण के लिए हम अमरीका को ले सकते है उसने अपने यहा अधिक अन्न पैदा किया और जब उसके पास अनाज फालतू बच गया तब वह अपने बकाया अनाज की बिक्री के लिए ऐसे देशों की तलाश करने लगा जो उधार पर माल ले सकते हो किंतु हमारी आंतरिक नीति ने यह तय किया कि खर्चीले ढंग से सरकार चलाएेंगे और स्वदेशी मुद्रा की कोई राशि हमारे पास नहीं बचेंगी हमने कर भी लगा दिए और मुद्रा प्रसार भी कर दिया कुछ संकट पड़ने के बाद इस बात की आवश्यकता को नहीं समझा कि उस पैसे का कहीं अन्यत्र उपयोग कर सके प्यारा श्रीमन मुझे माननीय प्रधानमंत्री जी के इस कथन पर दुख होता है कि दुनिया के अमीर और गरीब देशों का अंतर लगातार बढ़ता जा रहा है मैं उनसे यह पूछना चाहती हू कि भारत की विदेश नीति ने उस अंतर को घटाने की क्या कोशिश की है क्या भारत सरकार ने कभी दुनिया की पंचायत में यह कहने की हिम्मत की है कि बालिग मताधिकार के आधार पर यूएन ओ का चुनाव होकर एक संसद बनाई जाए और क्या आप में यह देखने की हिम्मत है कि फौज को कर लगाकर एक विकास का खाता खोल दिया जाए</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr">
@@ -3550,22 +4048,37 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन 60 शब्द प्रती मिनिट, पैसेज बी, रेडी, साथ.  अध्यक्षजी पैरा जिस समय पाकिस्तान ने भारत पर हमला किया था, उस समय उन्होंने देश की रक्षा के लिए महत्वपूर्ण कारिय किया था.  इसके साथ ही मैं मंत्री महोदय को यह भी स्मरण दिलाना चाहता हूँ की,  शायद उन्होंने इस पर ध्यान नहीं दिया की,  इस बार जो राश्ट्रिय पुरसकार मिले है, उन्में रेल्वे प्रशासन को केवल दो ही प्राप्त हुए है.  जब की मैं ऐसा मानता हूँ की, हमारी सेना के बाद,  अगर किसी ने युद्ध काल में सराहनिय कारिय किया है तो,  वह रेल्वे प्रशासन अत्वा, रेल्वे कर्मचारी और अधिकारी है,  इसलिए उनके मनोबल को बनाए रखने के लिए, और उनको प्रोच्छाहित करने के लिए,  रेल मंत्री को इस बात पर भी ध्यान रखना चाहिए, और इसका प्रयास करना चाहिए की,  जो भी इस तरह के प्रोच्छाहन मिले, उनमें रेल्वे का विशेश ध्यान रखा जाए,  तरह रेल मंत्री महोदय ने अपने वक्तव्य में भी रेल्वे कर्मचारियों की प्रशंसा की है,  या उनको प्रोच्छाहन दिलाया है, लेकिन यह प्रोच्छाहन शांती काल में भी बना रहना चाहिए,  रेल्वे ने युद्ध काल में जो काम किया, वह तो देश की रक्षा का महान उद्देश था,  लेकिन उसके बाद देश के निर्मान में या गरीबी मिटाने के लिए जो युद्ध होता है,  उसमें भी प्रत्यक रेल्वे कर्मचारी का मनोबल उसी तरीके से बना रहे,  इसके लिए भी रेल मंत्री महोदय को कुछ कदम उठाने की अवशकता है,</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
+          <t>हिंदी लघुलेखन साठ शब्द प्रति मिनट पैसेज भी रेडी स्ार्ट अध्यक्ष जी तारा जिस समय पाकिस्तान ने भारत पर हमला किया था उस समय उन्होंने देश की रक्षा के लिए महत्वपूर्ण कार्य किया था इसके साथ ही मैं मंत्री महोदय को यह भी स्मरण दिलाना चाहता हू कि शायद उन्होंने इस पर ध्यान नहीं दिया कि इस बार जो राष्ट्रीय पुरस्कार मिले है उनमें रेलवे प्रशासन को केवल दो ही प्राप्त हुए है जब कि मैं ऐसा मानता हू कि हमारी सेना के बाद अगर किसी ने युद्ध काल में सराहनीय कार्य किया है तो वह रेलवे प्रशासन अथवा रेलवे कर्मचारी और अधिकारी है इसलिए उनके मनोबल को बनाए रखने के लिए और उनको प्रोत्साहित करने के लिए रेल मंत्री को इस बात पर भी ध्यान रखना चाहिए और इसका प्रयास करना चाहिए कि जो भी इस तरह के प्रोत्साहन मिले उनमें रेलवे का विशेष ध्यान रखा जाए तारा रेल मंत्री महोदय ने अपने वक्तव्य में भी रेलवे कर्मचारियों की प्रशंसा की है या उनको प्रोत्साहन दिलाया है लेकिन यह प्रोत्साहन शांत काल में भी बना रहना चाहिए रेलवे ने युद्ध काल में जो काम किया वह तो देश की रक्षा का महान उद्देश्य था लेकिन उसके बाद देश के निर्माण में या गरीबी मिटाने के लिए जो युद्ध होता है उसमें भी प्रत्येक रेलवे कर्मचारी का मनोबल उसी तरीके से बना रहे इसके लिए भी रेल मंत्री महोदय को कुछ कदम उठाने की आवश्यकता है</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="U34" s="2" t="inlineStr">
-        <is>
-          <t>इन्दी लगुलेखन साठ शब्द प्रती मिनेट ट्रायल पैसेज रेडी साठ उपाध्यक्ष महोदय मैं इस बिल का स्वागत करता हूँ  मुझे दुख है की कई माननी या सदस्यों ने जिनोंने पता नहीं किस कारण से कहा तो यह की वे इस बिल का स्वागत करते है  लेकिन वास्तव में इसका विरोध करने का उन्होंने प्रयत्न किया है  हम सब इस प्रयत्न का दिल से स्वागत करते है</t>
-        </is>
-      </c>
       <c r="V34" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>हिंदी लघुलेखन साठ शब्द प्रति मिनट ट्रायल पैसेज रेडी स्टार्ट उपाध्यक्ष महोदय मैं इस बिल का स्वागत करता हूँ मुझे दुख है कि कई माननीय सदस्यों ने जिन्होंने पता नहीं किस कारण से कहा तो यह कि वे इस बिल का स्वागत करते हैं लेकिन वास्तव में इसका विरोध करने का उन्होंने प्रयत्न किया है हम सब इस प्रयत्न का दिल से स्वागत करते हैं</t>
+        </is>
+      </c>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3632,7 +4145,7 @@
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगूलेखन 100 शब्द प्रती मिनेट, पैसेज ए, रेडी, स्टार्ट  महोगय, बच्चे किसी भी देश के भविश्य होते है  यह यथार्थ सत्य है और सदीयों से इस और विशेश ध्यान देने की आवशकता पर बल दिया गया है  जन्म से लेकर बच्चों के स्वास्थ्य रहन सहन और उनकी शिक्षा को लेकर उनके माता पिता का चिंतित होना स्वाभवित है  लेकिन तेजी से अपनी जड़े जमा रहे भवतिक वादने हर छोटे बड़े समाज के सामने  ऐसे कई सवाल खड़े कर दिये है की बच्चों को किस तरह उनका हक दिलाया जाए  जिससे वे आगे चलकर मजबुती और आत्मविश्वास के साथ समाज के सजग प्रहरी बन सके  पिछले कुछ दशकों से बच्चों के भविश्य को लेकर उपजी चिन्ताओंने वैद्न्यानिकों और मनों वैद्न्यानिकों को  शोध और अनुसंधान के लिए बाध्य किया है  नित नई नई समस्याओंने माता पिता को दुविधा में डाल दिया है  एक और जहां जीवन यापन के लिए महिलाए भी पुरुशों की तरह कमर कसकर घर की चार दिवारों से बाहर निकल रही है  वही इसके कारण सदियों से चली आ रही सामाजिक संरचना गड़ बड़ाने लगी है  आ जीवी का कमाने और अत्यधिक सुखवैभव की चाहत ने हर दमपत्ती को जीवन शैली बदलने पर मजबूर कर दिया है  समाज में हो रहे इस बदलाव के कारण बच्चे सबसे ज़्यादा उपेक्षित होने लगे है  अब तक की तमाम रिपोर्टों के मुताबिक यह स्पश्ट है कि अगर बच्चों के प्रती माता पीता की उदासीनता इसी प्रकार बढ़ती रही  तो आने वाला वक्त तमाम परेशानियों के कारण जटिलता भरा हो जाएगा  बच्चों के सरवांगिन विकास के लिए जो सबसे पहली समस्या सामने आती है वह है उनका स्वास्थ्य  परिछेद माता पिता अपने बच्चों के स्वास्थ्य को लेकर चिंतित रहते है अपने सामर्थ्य के अनुसार वह कम से कम बच्चों के खाने पीने में कोई कोर कसर बाकी नहीं रहने देना चाहते  इस प्रयास में अकसर यही देखा गया है कि माता पिता खाने पीने के मामले में बच्चों पर मनोवईद्यानिक दबाव रखने में लगे रहते है  उनकी कोशिश यही रहती है कि उनका बच्चा हमेशा खाता पीता रहे और फिर यह होता है कि बच्चे के खाने पीने का कोई समय निर्धारित नहीं हो पाता  और समय खाने पीने के कारण कई प्रकार की समस्याए पैदा होती है बच्चों में मुटापा होना प्रमुख बाब है</t>
+          <t>हिंदी लघु लेखन सौ शब्द प्रति मिनट पैसेज ए रेडी स्टार्ट महोदय बच्चे किसी भी देश के भविष्य होते है यह यथार्थ सत्य है और सदियों से इस और विशेष ध्यान देने की आवश्यकता पर बल दिया गया है जन्म से लेकर बच्चों के स्वास्थ्य रहन सहन और उनकी शिक्षा को लेकर उनके माता पिता का चिंतित होना स्वाभाविक है लेकिन तेजी से अपनी जड़े जमा रहे भौतिकवाद ने हर छोटे बड़े समाज के सामने ऐसे कई सवाल खड़े कर दिए है कि बच्चों को किस तरह उनका हक दिलाया जाए जिससे वे आगे चलकर मजबूती और आत्मविश्वास के साथ समाज के सजग प्रहरी बन सके पिछले कुछ दशकों से बच्चों के भविष्य को लेकर उपजी चिंताओ ने वैज्ञानिकों और मनोवैज्ञानिकों को शोध और अनुसंधान के लिए बाध्य किया है नित नई नई समस्याओ ने माता पिता को दुविधा में डाल दिया है एक और जहाँ जीवन यापन के लिए महिलाए भी पुरुषों की तरह कमर कस कर घर की चार दीवारों से बाहर निकल रही है वही इसके कारण सदियों से चली आ रही सामाजिक संरचना गड़बड़ाने लगी है आजीविका कमाने और अत्यधिक सुख वैभव की चाहत ने हर दंपति को जीवन शैली बदलने पर मजबूर कर दिया है समाज में हो रहे इस बदलाव के कारण बच्चे सबसे ज्यादा उपेक्षित होने लगे है अब तक की तमाम रिपोर्टो के मुताबिक यह स्पष्ट है की अगर बच्चों के प्रति माता पिता की उदासीनता इसी प्रकार बढ़ती रही तो आने वाला वक्त तमाम परेशानियों के कारण जटिलता भरा हो जाएगा बच्चों के सर्वांगीण विकास के लिए जो सबसे पहली समस्या सामने आती है वह है उनका स्वास्थ्य परि्छेद माता पिता अपने बच्चों के स्वास्थ्य को लेकर चिंतित रहते है अपने सामर्थ्य के अनुसार वह कम से कम बच्चों के खाने पीने में कोई कोर कसर बाकी नहीं रहने देना चाहते इस प्रयास में अक्सर यही देखा गया है की माता पिता खाने पीने के मामले में बच्चों पर मनोवैज्ञानिक दबाव रखने में लगे रहते है उनकी कोशिश यही रहती है की उनका बच्चा हमेशा खाता पीता रहे और फिर यह होता है की बच्चे के खाने पीने का कोई समय निर्धारित नहीं हो पाता असमय खाने पीने के कारण कई प्रकार की समस्याए पैदा होती है बच्चों में मोटापा होना प्रमुख बाब है</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr">
@@ -3642,22 +4155,37 @@
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन चाव शब्द रती मिनेट, पैसेज बी, रेडी, स्टार्ट  महोदय, विकसित देशों के भाती, विकास शिल देशों में फिलहाल यह समस्या नहीं है  लेकिन बदली हुई परिस्थितियों में विशेशकर सम्भांत परिवारों और समस्या नहीं है  बच्चों के बीच मोटापे की समस्या तेजी से बढ़ रही है  वैसे तो बच्चों के मोटे होने के लिए कई परिस्थितिया जिम्मेदार होती है  जैसे उनके पैत्रुक गुण, भूख, उसका स्वभाव और दुखी होना  किनी विशेश प्रकर्णों में हार्मोन संचय में गड़बडी होना मोटापे का कारण बन जाता है  यदि बच्चे के माता-पिता मोटे है तो बच्चे की भी मोटे होने की संभावना बढ़ जाती है  पैत्रुक कारणों के अलावा बच्चे का स्वभाव भी उसके मोटापे के लिए जिम्मेदार साबित होता है  जो बच्चे ज्यादा नाखुश रहते है वे प्रक्ट्यक्ष रूप से ज्यादा खाने की आदी हो जाते है  ऐसे बच्चों में और समय खाने की आदते ज्यादा होती है  जब कभी उनका मन नहीं लगता वे कुछ खा पी कर अपना मन बहलाने की कोशिश करते है  और धीरे धीरे यह आदत बढ़ती जाती है जो उनके मोटापे का कारण बन जाती है  इसके अलावा जो बच्चे खेल कूद में दिल्चस्पी नहीं रखते उनके भी मोटा होने की संभावना होती है  व्यायाम की कमी से शरीर की उर्जा चर्बी में परिनत होने लगती है  इन सब परिस्षितियों में मोटापे के आसार बढ़ने लगते है  अधिक भूख लगना और अधिक भोजन खाना मोटापे का सबसे बड़ा कारण होता है  नवजात शिशू ही क्यों न हो उसे आवशकता के अधिक दूद पिलाना अवांचनिय है  दूद के स्थान पर थोस आहार देना अधिक स्रेयसकर होता है  जैसे जैसे बच्चा बड़ा होता है उसके खाने पीने में  खासकर इस बात का ध्यान रखा जाना चाहिए कि उसमें चर्चा बढ़ाने का कारण बनने वाले खाद्य पदार्थ  खासकर घी मखन आदी का इस्तेमाल अनुपात से ज्यादा न होने पाए  परिछेद करीब 6-7 वर्ष से लेकर 14-15 वर्ष तक की उम्रके बच्चों का शारिरीक विकास अत्याधिक टेज हो जाता है  इस उम्रके दवरान विभिन्न शारिरीक एवं हार्मोन परिवर्तनों के कारण बच्चों में मोटापा बढ़ने का खत्रा रहता है  मोटापा बच्चों के लिए तई बार एक अभिशाप बन जाता है  अन्य बच्चे उसे मोटा कहकर चिढाते है तथा उसके साथ खेलना पसंद नहीं करते  इस प्रकार बच्चे दुखी होते है और स्वयम को अकेले पन महसूस करते है</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
+          <t>हिंदी लघु लेखन स शब्द प्रति मिनट पैसेज भी रेडी स्टार्ट महोदय विकसित देशों के भांति विकासशील देशो में फिलहाल यह समस्या नहीं है लेकिन बदली हुई परिस्थितियों में विशेषकर संभ्रांत परिवारों और समस्या नहीं है बच्चों के बीच मोटापे की समस्या तेजी से बढ़ रही है वैसे तो बच्चों के मोटे होने के लिए कई परिस्थितिया जिम्मेदार होती है जैसे उनके पैतृक गुण भूख उसका स्वभाव और दुखी होना किन्हीं विशेष प्रकरणों में हारमोन संचय में गड़बड़ी होना मोटापे का कारण बन जाता है यदि बच्चे के माता पिता मोटे है तो बच्चे की भी मोटे होने की संभावना बढ़ जाती है पैतृक कारणों के अलावा बच्चे का स्वभाव भी उसके मोटापे के लिए जिम्मेदार साबित होता है जो बच्चे ज्यादा ना खुश रहते है वे प्रत्यक्ष रूप से ज्यादा खाने की आदि हो जाते है ऐसे बच्चों में असमय खाने की आदत ज्यादा होती है जब कभी उनका मन नहीं लगता वे कुछ खा पी कर अपना मन बहलाने की कोशिश करते है और धीरे धीरे यह आदत बढ़ती जाती है जो उनके मोटापे का कारण बन जाती है इसके अलावा जो बच्चे खेल कूद में दिलचस्पी नहीं रखते उनके भी मोटा होने की संभावना होती है व्यायाम की कमी से शरीर की ऊर्जा चरबी में परिणत होने लगती है इन सब परिस्थितियों में मोटापे के आसार बढ़ने लगते है अधिक भूख लगना और अधिक भोजन खाना मोटापे का सबसे बड़ा कारण होता है नवजात शिशु ही क्यों न हो उसे आवश्यकता के अधिक दूध पिलाना अवाछनीय है दूध के स्थान पर ठोस आहार देना अधिक श्रेयस्कर होता है जैसे जैसे बच्चा बड़ा होता है उसके खाने पीने में खास कर इस बात का ध्यान रखा जाना चाहिए की उसमें चर्चा बढ़ाने का कारण बनने वाले खाद्य पदार्थ खासकर घी मक्खन आदि का इस्तेमाल अनुपात से ज्यादा न होने पाए परि्छेद करीब छह से सात वर्ष से लेकर चौदह से पंद्रह वर्ष तक की उम्र के बच्चों का शारीरिक विकास अत्यधिक तेज हो जाता है इस उम्र के दौरान विभिन्न शारीरिक एवं हारमोन परिवर्तनों के कारण बच्चों में मोटापा बढ़ने का खतरा रहता है मोटापा बच्चों के लिए कई बार एक अभिशाप बन जाता है अन्य बच्चे उसे मोटा कहकर चिढ़ाते है तथा उसके साथ खेलना पसंद नहीं करते इस प्रकार बच्चे दुखी होते है और स्वयं को अकेलेपन महसूस करते है</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="U35" s="2" t="inlineStr">
-        <is>
-          <t>हिंदी लगुलेखन सव शब्द प्रति मिनेट ट्रायल पैसेज रेडी स्टार्ट  सभापती जी शिक्षा का दूसरा प्रयोजन यह है कि वह प्रत्तिक मानव को अपनी करमेंद्रियों का ऐसा प्रयोग सिखाए  जो उसे अपनी शारिरिक और अन्य प्रकार की आवशकताओं की पूर्ति करने के योग्य बना सके  इन करमेंद्रियों के उचित प्रयोग के लिए तो ग्यान की आवशकता होती है  कितना ही सबल व्यक्ति क्यों न हो कितना ही हूर्ति में कोई क्यों न हो  वह तब तक कुछ अधिक फलमें कारिय नहीं कर सकता जब तक की उस कारिय के संपादन के लिए उसकी आवशकता पड़ती है  क्या अवशकता जब तक की आवशकता है</t>
-        </is>
-      </c>
       <c r="V35" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="inlineStr">
+        <is>
+          <t>हिंदी लघु लेखन सौ शब्द प्रति मिनट ट्रायल पैसेज रेडी स्टार्ट सभापति जी शिक्षा का दूसरा प्रयोजन यह है की वह प्रत्येक मानव को अपनी कर्मेंद्रियों का ऐसा प्रयोग सिखाए जो उसे अपनी शारीरिक और अन्य प्रकार की आवश्यकताओं की पूर्ति करने के योग्य बना सके इन कर्मेंद्रियों के उचित प्रयोग के लिए तो ज्ञान की आवश्यकता होती है कितना ही सबल व्यक्ति क्यों न हो कितना ही स्फूर्तिमय कोई क्यों न हो वह तब तक कुछ अधिक फलमय कार्य नहीं कर सकता जब तक की उस कार्य के संपादन के लिए उसकी आवश्यकता पड़ती है</t>
+        </is>
+      </c>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
+        </is>
+      </c>
+      <c r="Y35" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -3724,7 +4252,7 @@
       <c r="P36" s="2" t="n"/>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन सव शब्द प्रतिमिनेट, पैसेज ए, रेडी, स्टार्ड, सज्जनों और दीवियों, परिछेत विगत दो दशकों से मेरा संपर्क जहा तक कार्यालाईन कारभार का प्रश्ण है, देश के विबिन्न भागों में कार्यरत स्वैचीक हिंदी संस्तावों  और उनके इर्दगिर्द की बातों पर अपने विचार केंद्रीत करूंगा, जहां हिंदी शिक्षन एवं परिक्षा संचलन हिंदी प्रचार प्रसार के सरवाधिक रचनात्मक कार्यक्रम है, वहीं हिंदी तर क्षेत्र में हिंदी के लिए अनुकूल वातावरन निर्मान �  आज इन कार्यक्रमों के संचालन सहज सुगम नहीं रहे गए, बलकि चुनवती पुर्ण हो गए है, विद्यार्थियों की योग्यता बढ़ाने के लिए शिक्षा एवं परिक्षा के अतिरिक्त हिंदी वक्तव्य निबंद वाद विवाद के साथ साथ नाटक एकां की प्र  पुरस्कार योजना जाई से कार्यक्रम आयोजीत किये चाते है, अनुकूल वातावरन निर्मान के लिए जहा इन कार्यक्रमों को अधिक प्रभावी बनाने की अवशक्ता है, वही अन्य प्रभावी कार्यक्रमों की परिकलपना करनी होगी  हिंदी शिक्षन परिक्षा संचलन और वातावरन निर्मान इन तिनों के सफल आयोजन पर विद्यार्थियों का हिंदी ग्यान अर्थात हिंदी बोलने पढ़ने एवं लिखने की दक्षता का पुरा दारोंदार टिका रहता है  आज जबकी अधिक विद्यार्थी शिक्षक बनने की राहमें प्रशिक्षन प्राप्त कर रहे है तो हिंदी शिक्षक की योग्यता एवं दक्षता ऐसे ध्यान देने का विशय है  जो राज्य के इतने सारे हिंदी शिखने वाले विद्यार्थियों के स्तर के लिए निरनायक पहलू है।  यह नकरा नहीं जा सकता की। किसी भी संस्ता के लिए उनके प्रचारक ही अधारबूत होते है।  प्रचारकों के सत्प्रयास एवं सुकार्य से संस्ता की जड़े मजबूत होती है।  विद्यार्थी और अंत में किन्तू कदापी कम नहीं, सरकारी व्यवस्तता के तालमेल पर इन सबके कारियों के उचीत समनवय का प्रयत्न स्वस्थ दुरुष्टी से निरंतर जारी रहना चाहिए, और यह भी ध्यान रहे की जाने अंजाने दामन में दाग न लग जाए,  परिछेत भारत ग्रामों का देश है और अधिकाउंश भारतिय जनता ग्रामों में बस्ती है, नगरों और शहरों के नागरिकों को शिक्षा की कई सुविदाय प्राप्त है, यह उने हिंदी पढ़ने के उचीत अउसर उपलब्द हो जाते है, अधिक अउसर प्रदान किये �</t>
+          <t>हिंदी लघुलेखन सौ शब्द प्रतिमिनट पैसेज ए रेडी स्टार सज्जनों और दवियों परि्ेद विगत दो दशकों से मेरा संपर्क जहा तक कार्यालयन कारभार का प्रश्न है देश के विभिन्न भागों में कार्यरत स्वैच्छिक हिंदी संस्थाओं से रहा है आज इस मंच से संस्थाओं और उनके इर्द गिर्द की बातों पर अपने विचार केंद्रित करूंगा जहाँ हिंदी शिक्षण एवं परीक्षा संचालन हिंदी प्रचार प्रसार के सर्वाधिक रचनात्मक कार्यक्रम है वही हिंदीतर क्षेत्र में हिंदी के लिए अनुकूल वातावरण निर्माण भी एक महत्वपूर्ण पहलू है आज इन कार्यक्रमों के संचालन सहज सुगम नहीं रह गए बल्कि चुनौती पूूर्ण हो गए है विद्यार्थियों की योग्यता बढ़ाने के लिए शिक्षा एवं परीक्षा के अतिरिक्त हिंदी वक्तव्य निबंध वाद विवाद के साथ साथ नाटक एकांकी प्रतियोगिताए आयोजित की जाती है हिंदी शिक्षकों प्रचारकों के लिए शिविर पुनश्चर्या कार्य शिविर पुरस्कार योजना जैसे कार्यक्रम आयोजित किए जाते हैं अनुकूल वातावरण निर्माण के लिए जहाँ इन कार्यक्रमों को अधिक प्रभावी बनाने की आवश्यकता है वही अन्य प्रभावी कार्यक्रमों की परिकल्पना करनी होगी हिंदी शिक्षण परीक्षा संचालन और वातावरण निर्माण इन तीनों के सफल आयोजन पर विद्यार्थियों का हिंदी ज्ञान अर्थात हिंदी बोलने पढ़ने एवं लिखने की दक्षता का पूरा दारमदार टिका रहता है आज जबकि अधिक विद्यार्थी शिक्षक बनने की राह में प्रशिक्षण प्राप्त कर रहे है तो हिंदी शिक्षक की योग्यता एवं दक्षता ऐसे ध्यान देने का विषय है जो राज्य के इतने सारे हिंदी सीखने वाले विद्यार्थियों के स्तर के लिए निर्णायक पहलू है यह नकारा नहीं जा सकता की किसी भी संस्था के लिए उनके प्रचारक ही आधारभूत होते है प्रचारकों के स प्रयास एवं सुकार्य से संस्था की जड़े मजबूत होती है वास्तव में हिंदी की प्रचार योजनाओं का सफल कार्यान्वयन सभी संबंधित पक्षों के प्रयास के समन्वय से ही संभव है संस्था के पदाधिकारी कार्यकर्ता प्रचारक गण विद्यार्थी और अंत में किंतु कदापि कम नहीं सरकारी व्यवस्थता के तालमेल पर इन सबके कार्यों के उचित समन्वय का प्रयत्न स्वस्थ दृष्टि से निरंतर जारी रहना चाहिए और यह भी ध्यान रहे कि जाने अन जााने दामन में दाग न लग जाए पर्ेद भारत ग्रामों का देश है और अधिकांश भारतीय जनता ग्रामों में बसती है नगरों और शहरों के नागरिकों को शिक्षा की कई सुविधाए प्राप्त है यो उन्हें हिंदी पढ़ने के उचित अवसर उपलब्ध हो जाते है अधिक अवसर प्रदान किए जाए</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr">
@@ -3734,22 +4262,37 @@
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>हिंदी लगुलेखन सव शब्द प्रतिमिनेट पैसेज बी रेडी स्टार्ट महोदय परिछेत कुछ लोग आज यह कहते देखे गए है की राष्ट्रिय एकता अंग्रेजी की माध्यम से हो सकती है  कई लोगों की धारना है की अंग्रेजी निकाल दी जाये तो राष्ट्र टुकडे टुकडे हो जायेगा वैज्यानीक प्रगती रूक जायेगी आदी इससे बढ़कर ब्रहमक विचार और कुछ भी नहीं हो सकता  मैं अंग्रेजी की उपादेता को नकार नहीं रहा किन्तु हर जगह उसका वर्चस्व हो यह स्विकार्य नहीं हो सकता  किसी देश की भाषा के साथ उस देश की संस्कृती विचारधारा और मान्यताये जुडी रहती है और उने प्रकट करने के लिए उस देश की भाषा ही सर्वसक्षम होती है  स्वतंत्रता के पुर्व राष्ट्रिय गवरव आम जन्ता को दुरुष्टी में रखकर किया जाता था  राष्ट्रिय एकता का अर्थ है करोडो भार्तियों की एकता और यह एकता हिंदे से ही लाई जा सकती है  अंग्रेजी से नहीं अंग्रेजी को बनाए रखने की नीती मानसिक दासता की ज्योतक है  यदि हिंदी और भारतिय भाषाओं के विरुद्ध अंग्रेजी शर्यंत्र को विफल नहीं किया गया  तो जनतंत्र एक मखोल बनकर रह जाएगा हिंदी और भारतिय भाषाओं तो सहो दराए है  उनमें आपसी कोई विरुद नहीं उनका विरुद और संगर्षतों अंग्रेजी के साथ है  जिस दिन क्षेत्रिय भाषाए अपने क्षेत्र के प्रशासन, न्याय, शिक्षा आदी में स्तापीत हो जाएंगी  उसी दिन राश्ट्रिय स्तर पर राश्ट्र भाषा, राज भाषा और संपर्क भाषा के रूप में हिंदी के स्तापीत हो जाने का मार्ग प्रशस्त हो जाएगा  स्वैचिक हिंदी संस्ताए अपने इस मूल उद्देश्य को कभी भी धुमिल नहीं खोने देंगे क्योंकि हिंदी के प्रचार प्रसार के खेत्र में वे सरवाधिक महत्वपुर्ण इकाईया है  इस द्रुष्टी से महिसूर हिंदी प्रचार प्रिशत का यह कार्यक्रम उलेखनिय है की वह हिंदी के साथ कंणड एतर जिग्या सों के लिए कंणड की कारंभिक और उच्चक अक्षाये एवं परिक्षाये चला रही है  अपनी दैनन्दिने में भी हिंदी के साथ साथ कंणड में दीन और तिथिया दी है  इस तरह के छोटे किन्तु दीन दीन के विवहार में राष्ट्र भाषा और ख्षेत्रिय भाषा साथ साथ मील जूल कर चले  इससे बढ़कर सुखद स्थिती और क्या हो सकती है परिछेत और प्रियस नातको आज का दीन आपका है और कल का दीन भी आपका ही होगा  विगत वर्षों में आपने कठीन परिश्रम कर हिंदी रत्न अत्वा हिंदी प्रशुक्षन की परिक्षाय दी है उत्तिर्न हुए है आपकी दिक्षा पुरी हो चुकी है</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="T36" s="2" t="inlineStr">
         <is>
+          <t>हिंदी लघुलेखन सौ शब्द प्रतिमिनट पैसेज बी रेडी स्टार महोदय परि्ेद कुछ लोग आज यह कहते देखे गए है कि राष्ट्रीय एकता अंग्रेजी के माध्यम से हो सकती है कई लोगों की धारणा है कि अंग्रेजी निकाल दी जाए तो राष्ट्र टुकड़े टुकड़े हो जाएगा वैज्ञानिक प्रगति रुक जाएगी आदि इससे बढ़कर भ्रामक विचार और कुछ भी नहीं हो सकता मै अंग्रेजी की उपादेयता को नकार नहीं रहा किंतु हर जगह उसका वर्चस्व हो यह स्वीकार्य नहीं हो सकता किसी देश की भाषा के साथ उस देश की संस्कृति विचारधारा और मान्यताए जुड़ी रहती है और उन्हें प्रकट करने के लिए उस देश की भाषा ही सर्व सक्षम होती है स्वतंत्रता के पूर्व राष्ट्रीय गौरव आम जनता को दृष्टि में रखकर किया जाता था राष्ट्रीय एकता का अर्थ है करोड़ों भारतीयों की एकता और यह एकता हिंदी से ही लाई जा सकती है अंग्रेजी से नहीं अंग्रेजी को बनाए रखने की नीति मानसिक दासता की द्योतक है यदि हिंदी और भारतीय भाषाओं के विरुद्ध अंग्रेजी षडयंत्र को विफल नहीं किया गया तो जनतंत्र एक मखौल बनकर रह जाएगा हिंदी और भारतीय भाषाए तो सहोदराय है उनमें आपसी कोई विरोध नहीं उनका विरोध और संघर्ष तो अंग्रेजी के साथ है जिस दिन क्षेत्रीय भाषाए अपने क्षेत्र के प्रशासन न्याय शिक्षा आदि में स्थापित हो जाएंग उसी दिन राष्ट्रीय स्तर पर राष्ट्रभााषा राजभाषा और संपर्क भाषा के रूप में हिंदी के स्थापित हो जाने का मार्ग प्रशस्त हो जाएगा स्वैच्छिक हिंदी संस्थाएं अपने इस मूल उद्देश्य को कभी भी धूमिल नहीं होने देंगे क्योंकि हिंदी के प्रचार प्रसार के क्षेत्र में वे सर्वाधिक महत्वपूर्ण इकाइया है इस दृष्टि से मैसूर हिंदी प्रचार परिषद का यह कार्यक्रम उल्लेखनीय है कि वह हिंदी के साथ कन्नड़ेतर जिज्ञासओ के लिए कन्नड़ की प्रारंभिक और उच्च कक्षाए एवं परीक्षाए चला रही है अपनी दैनदिनी में भी हिंदी के साथ साथ कन्नड़ में दीन और तिथिया दी है इस तरह के छोटे किंतु दीन दिन के व्यवहार में राष्ट्रभााषा और क्षेत्रीय भाषा साथ साथ मिलजुल कर चले इससे बढ़कर सुखद स्थिति और क्या हो सकती है परिछेद और प्रिय स्नातकों आज का दिन आपका है और कल का दिन भी आपका ही होगा विगत वर्षों में आपने कठिन परिश्रम कर हिंदी रत्न अथवा हिंदी प्रशिक्षण की परीक्षाएं दी है उत्तीर्ण हुए है आपकी दीक्षा पूरी हो चुकी है</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
         </is>
       </c>
-      <c r="U36" s="2" t="inlineStr">
-        <is>
-          <t>हिंदी अशुलेखन, सव शब्द प्रतिमिनिट, ट्रायल पैसेज, रेडी? स्टार्ड, सभा पतीजी, शिक्षा का दुसरा प्रयोजन, यह है कि वह प्रत्यक मानव को अपनी कर्मेंद्रियों का ऐसा प्रयोग सिखाएं,  जो उसे अपनी शारिरीक और अन्य प्रकार की अवशक्ताओं की पुर्ती करने के योग्य बना सके, इन कर्मेंद्रियों के उचेत प्रयोग के लिये, तो ज्यान की अवशक्ता हुती है,  कितना ही सबल व्यक्ती क्यों न हो, कितना ही स्फूर्ती में क्यों न हो, वह तब तक कुछ अधिक फलमें कारिय नहीं कर सकता,  जब तक की उस कारिय के संपादन के लिये उसकी अवशक्ता पड़ती है,</t>
-        </is>
-      </c>
       <c r="V36" s="2" t="inlineStr">
         <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="inlineStr">
+        <is>
+          <t>हिंदी अशलेखन सौ शब्द प्रतिमिनट ट्रायल पैसेज रेडी स्टार सभापति जी शिक्षा का दूसरा प्रयोजन यह है कि वह प्रत्येक मानव को अपनी कर्मेंद्रियों का ऐसा प्रयोग सिखाए जो उसे अपनी शारीरिक और अन्य प्रकार की आवश्यकताओं की पूर्ति करने के योग्य बना सके इन कर्मेंद्रियों के उचित प्रयोग के लिए तो ज्ञान की आवश्यकता होती है कितना ही सबल व्यक्ति कों न होतना ही स्फूर्ति्य न हो व तब तक कुछ अधिक फलमय कार्य नहीं कर सकता जब तक कि उस कार्य के संपादन के लिए उसकी आवश्यकता पड़ती है</t>
+        </is>
+      </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
           <t>hi</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>

</xml_diff>